<commit_message>
chore(data): batch update intraday dim_rca - 08:01:04
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2427"/>
+  <dimension ref="A1:D2429"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21640,7 +21640,7 @@
     <row r="1179">
       <c r="A1179" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B1179" t="n">
@@ -43025,37 +43025,37 @@
     <row r="2367">
       <c r="A2367" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2814</v>
+        <v>2833</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>ADEILZA PINTO DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>39</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2368">
       <c r="A2368" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2646</v>
+        <v>2814</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2368" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2369">
@@ -43065,11 +43065,11 @@
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2650</v>
+        <v>2646</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2369" t="n">
@@ -43083,15 +43083,15 @@
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2652</v>
+        <v>2650</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2371">
@@ -43101,15 +43101,15 @@
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2372">
@@ -43119,15 +43119,15 @@
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2654</v>
+        <v>2653</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2372" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2373">
@@ -43137,51 +43137,51 @@
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2655</v>
+        <v>2654</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2374">
       <c r="A2374" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2821</v>
+        <v>2655</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>69</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2375">
       <c r="A2375" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2683</v>
+        <v>2821</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2375" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2376">
@@ -43191,33 +43191,33 @@
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2376" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2749</v>
+        <v>2684</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2377" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2378">
@@ -43227,195 +43227,195 @@
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2812</v>
+        <v>2749</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>145</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2379">
       <c r="A2379" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2715</v>
+        <v>2812</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2379" t="n">
-        <v>90</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2380">
       <c r="A2380" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2651</v>
+        <v>2715</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2380" t="n">
-        <v>145</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2381">
       <c r="A2381" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2819</v>
+        <v>2834</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2382">
       <c r="A2382" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2699</v>
+        <v>2651</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2383">
       <c r="A2383" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2706</v>
+        <v>2819</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS BARREIRINHAS</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2707</v>
+        <v>2699</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>EVANESSA DA SILVA E SILVA</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2385">
       <c r="A2385" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2693</v>
+        <v>2706</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>SETOR VAGO PLUS BARREIRINHAS</t>
         </is>
       </c>
       <c r="D2385" t="n">
-        <v>80</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2386">
       <c r="A2386" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2705</v>
+        <v>2707</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>EVANESSA DA SILVA E SILVA</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>146</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2387">
       <c r="A2387" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2664</v>
+        <v>2693</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2670</v>
+        <v>2705</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>69</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2389">
@@ -43425,141 +43425,141 @@
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2730</v>
+        <v>2664</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2671</v>
+        <v>2670</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2691</v>
+        <v>2730</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2692</v>
+        <v>2671</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2724</v>
+        <v>2691</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2394">
       <c r="A2394" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2773</v>
+        <v>2692</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>VIVIANE LEAL DA SILVA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2825</v>
+        <v>2724</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2396">
       <c r="A2396" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2787</v>
+        <v>2773</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>VIVIANE LEAL DA SILVA</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2397">
@@ -43569,51 +43569,51 @@
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2648</v>
+        <v>2825</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2666</v>
+        <v>2787</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>63</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2779</v>
+        <v>2648</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>105</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2400">
@@ -43623,15 +43623,15 @@
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2780</v>
+        <v>2666</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2401">
@@ -43641,51 +43641,51 @@
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2786</v>
+        <v>2779</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2402">
       <c r="A2402" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2660</v>
+        <v>2780</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>38</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2403">
       <c r="A2403" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2716</v>
+        <v>2786</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2404">
@@ -43695,51 +43695,51 @@
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2734</v>
+        <v>2660</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2405">
       <c r="A2405" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2742</v>
+        <v>2716</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2794</v>
+        <v>2734</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2407">
@@ -43749,11 +43749,11 @@
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2795</v>
+        <v>2742</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2407" t="n">
@@ -43767,15 +43767,15 @@
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2796</v>
+        <v>2794</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2409">
@@ -43785,11 +43785,11 @@
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2797</v>
+        <v>2795</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
         </is>
       </c>
       <c r="D2409" t="n">
@@ -43803,11 +43803,11 @@
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2798</v>
+        <v>2796</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2410" t="n">
@@ -43817,73 +43817,73 @@
     <row r="2411">
       <c r="A2411" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2668</v>
+        <v>2797</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2412">
       <c r="A2412" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2690</v>
+        <v>2798</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2413">
       <c r="A2413" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2696</v>
+        <v>2668</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>69</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2414">
       <c r="A2414" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2697</v>
+        <v>2690</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2415">
@@ -43893,11 +43893,11 @@
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2698</v>
+        <v>2696</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2415" t="n">
@@ -43907,37 +43907,37 @@
     <row r="2416">
       <c r="A2416" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2775</v>
+        <v>2697</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2416" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2417">
       <c r="A2417" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2776</v>
+        <v>2698</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2418">
@@ -43947,11 +43947,11 @@
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2777</v>
+        <v>2775</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2418" t="n">
@@ -43965,11 +43965,11 @@
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2778</v>
+        <v>2776</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2419" t="n">
@@ -43983,15 +43983,15 @@
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2781</v>
+        <v>2777</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2421">
@@ -44001,11 +44001,11 @@
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2822</v>
+        <v>2778</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2421" t="n">
@@ -44019,87 +44019,87 @@
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2740</v>
+        <v>2781</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2423">
       <c r="A2423" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2710</v>
+        <v>2822</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2424">
       <c r="A2424" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2711</v>
+        <v>2740</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2424" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2425">
       <c r="A2425" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2712</v>
+        <v>2710</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2425" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2426">
       <c r="A2426" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2717</v>
+        <v>2711</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D2426" t="n">
-        <v>69</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2427">
@@ -44109,14 +44109,50 @@
         </is>
       </c>
       <c r="B2427" t="n">
+        <v>2712</v>
+      </c>
+      <c r="C2427" t="inlineStr">
+        <is>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
+        </is>
+      </c>
+      <c r="D2427" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2428">
+      <c r="A2428" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2428" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2428" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2428" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2429">
+      <c r="A2429" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2429" t="n">
         <v>2801</v>
       </c>
-      <c r="C2427" t="inlineStr">
+      <c r="C2429" t="inlineStr">
         <is>
           <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
-      <c r="D2427" t="n">
+      <c r="D2429" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:01:16
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -25168,7 +25168,7 @@
     <row r="1375">
       <c r="A1375" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B1375" t="n">
@@ -34096,7 +34096,7 @@
     <row r="1871">
       <c r="A1871" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B1871" t="n">

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:01:01
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2429"/>
+  <dimension ref="A1:D2430"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43331,37 +43331,37 @@
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2699</v>
+        <v>2835</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>ROGÉRIO LIRA DA GAMA</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>95</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2385">
       <c r="A2385" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2706</v>
+        <v>2699</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS BARREIRINHAS</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2385" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2386">
@@ -43371,11 +43371,11 @@
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2707</v>
+        <v>2706</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>EVANESSA DA SILVA E SILVA</t>
+          <t>SETOR VAGO PLUS BARREIRINHAS</t>
         </is>
       </c>
       <c r="D2386" t="n">
@@ -43385,127 +43385,127 @@
     <row r="2387">
       <c r="A2387" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2693</v>
+        <v>2707</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>EVANESSA DA SILVA E SILVA</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>80</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2705</v>
+        <v>2693</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>146</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2389">
       <c r="A2389" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2664</v>
+        <v>2705</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>90</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2670</v>
+        <v>2664</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2730</v>
+        <v>2670</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2671</v>
+        <v>2730</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2691</v>
+        <v>2671</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2394">
@@ -43515,11 +43515,11 @@
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2394" t="n">
@@ -43529,55 +43529,55 @@
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2724</v>
+        <v>2692</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2396">
       <c r="A2396" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2773</v>
+        <v>2724</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>VIVIANE LEAL DA SILVA</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2397">
       <c r="A2397" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2825</v>
+        <v>2773</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>VIVIANE LEAL DA SILVA</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2398">
@@ -43587,15 +43587,15 @@
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2787</v>
+        <v>2825</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2399">
@@ -43605,33 +43605,33 @@
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2648</v>
+        <v>2787</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2400">
       <c r="A2400" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2666</v>
+        <v>2648</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2401">
@@ -43641,15 +43641,15 @@
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2779</v>
+        <v>2666</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2402">
@@ -43659,11 +43659,11 @@
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2780</v>
+        <v>2779</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2402" t="n">
@@ -43677,33 +43677,33 @@
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2786</v>
+        <v>2780</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2404">
       <c r="A2404" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2660</v>
+        <v>2786</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2405">
@@ -43713,15 +43713,15 @@
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2716</v>
+        <v>2660</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2406">
@@ -43731,11 +43731,11 @@
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2734</v>
+        <v>2716</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2406" t="n">
@@ -43745,19 +43745,19 @@
     <row r="2407">
       <c r="A2407" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2742</v>
+        <v>2734</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2408">
@@ -43767,15 +43767,15 @@
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2794</v>
+        <v>2742</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2409">
@@ -43785,15 +43785,15 @@
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2795</v>
+        <v>2794</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2410">
@@ -43803,11 +43803,11 @@
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2796</v>
+        <v>2795</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
         </is>
       </c>
       <c r="D2410" t="n">
@@ -43821,11 +43821,11 @@
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2797</v>
+        <v>2796</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2411" t="n">
@@ -43839,11 +43839,11 @@
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2798</v>
+        <v>2797</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2412" t="n">
@@ -43853,55 +43853,55 @@
     <row r="2413">
       <c r="A2413" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2668</v>
+        <v>2798</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2414">
       <c r="A2414" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2690</v>
+        <v>2668</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>38</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2415">
       <c r="A2415" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2696</v>
+        <v>2690</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2415" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2416">
@@ -43911,11 +43911,11 @@
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2416" t="n">
@@ -43929,11 +43929,11 @@
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2417" t="n">
@@ -43943,19 +43943,19 @@
     <row r="2418">
       <c r="A2418" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2775</v>
+        <v>2698</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2418" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2419">
@@ -43965,11 +43965,11 @@
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2776</v>
+        <v>2775</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2419" t="n">
@@ -43983,11 +43983,11 @@
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2777</v>
+        <v>2776</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2420" t="n">
@@ -44001,11 +44001,11 @@
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2778</v>
+        <v>2777</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2421" t="n">
@@ -44019,15 +44019,15 @@
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2781</v>
+        <v>2778</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2423">
@@ -44037,15 +44037,15 @@
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2822</v>
+        <v>2781</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2424">
@@ -44055,11 +44055,11 @@
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2740</v>
+        <v>2822</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2424" t="n">
@@ -44069,90 +44069,108 @@
     <row r="2425">
       <c r="A2425" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2710</v>
+        <v>2740</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2425" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2426">
       <c r="A2426" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2711</v>
+        <v>2710</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2426" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2427">
       <c r="A2427" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2712</v>
+        <v>2711</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D2427" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2428">
       <c r="A2428" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2717</v>
+        <v>2712</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
         </is>
       </c>
       <c r="D2428" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2429">
       <c r="A2429" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2429" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2429" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2429" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2430">
+      <c r="A2430" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2430" t="n">
         <v>2801</v>
       </c>
-      <c r="C2429" t="inlineStr">
+      <c r="C2430" t="inlineStr">
         <is>
           <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
-      <c r="D2429" t="n">
+      <c r="D2430" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:03:00
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2430"/>
+  <dimension ref="A1:D2432"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41279,73 +41279,73 @@
     <row r="2270">
       <c r="A2270" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2270" t="n">
-        <v>2799</v>
+        <v>2836</v>
       </c>
       <c r="C2270" t="inlineStr">
         <is>
-          <t>VOLFRAMIO DALFREDO ALMEIDA</t>
+          <t>MARIA EDUARDA SILVA SANTOS</t>
         </is>
       </c>
       <c r="D2270" t="n">
-        <v>69</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2271">
       <c r="A2271" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2271" t="n">
-        <v>2719</v>
+        <v>2837</v>
       </c>
       <c r="C2271" t="inlineStr">
         <is>
-          <t>SETOR SÃO RDO NONATO VAGO  (DEDICADA)</t>
+          <t>MERCYA BERCE NASCIMENTO DE MESQUITA</t>
         </is>
       </c>
       <c r="D2271" t="n">
-        <v>39</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2272">
       <c r="A2272" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2272" t="n">
-        <v>2731</v>
+        <v>2799</v>
       </c>
       <c r="C2272" t="inlineStr">
         <is>
-          <t>VAGO ANDERSON A. S. - FARMA (CAMAÇARI)</t>
+          <t>VOLFRAMIO DALFREDO ALMEIDA</t>
         </is>
       </c>
       <c r="D2272" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2273">
       <c r="A2273" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2273" t="n">
-        <v>2732</v>
+        <v>2719</v>
       </c>
       <c r="C2273" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN DE JESUS - HB</t>
+          <t>SETOR SÃO RDO NONATO VAGO  (DEDICADA)</t>
         </is>
       </c>
       <c r="D2273" t="n">
-        <v>98</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2274">
@@ -41355,11 +41355,11 @@
         </is>
       </c>
       <c r="B2274" t="n">
-        <v>2733</v>
+        <v>2731</v>
       </c>
       <c r="C2274" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAGO CENTRO CAROLINE LEMOS - FARMA </t>
+          <t>VAGO ANDERSON A. S. - FARMA (CAMAÇARI)</t>
         </is>
       </c>
       <c r="D2274" t="n">
@@ -41369,19 +41369,19 @@
     <row r="2275">
       <c r="A2275" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2275" t="n">
-        <v>2752</v>
+        <v>2732</v>
       </c>
       <c r="C2275" t="inlineStr">
         <is>
-          <t>SETOR BAIXADA PLUS (ELILTON ROMEU)</t>
+          <t>VAGO BRENO ALLAN DE JESUS - HB</t>
         </is>
       </c>
       <c r="D2275" t="n">
-        <v>114</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2276">
@@ -41391,33 +41391,33 @@
         </is>
       </c>
       <c r="B2276" t="n">
-        <v>2662</v>
+        <v>2733</v>
       </c>
       <c r="C2276" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
+          <t xml:space="preserve">VAGO CENTRO CAROLINE LEMOS - FARMA </t>
         </is>
       </c>
       <c r="D2276" t="n">
-        <v>50</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2277">
       <c r="A2277" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2277" t="n">
-        <v>2663</v>
+        <v>2752</v>
       </c>
       <c r="C2277" t="inlineStr">
         <is>
-          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
+          <t>SETOR BAIXADA PLUS (ELILTON ROMEU)</t>
         </is>
       </c>
       <c r="D2277" t="n">
-        <v>100</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2278">
@@ -41427,15 +41427,15 @@
         </is>
       </c>
       <c r="B2278" t="n">
-        <v>2685</v>
+        <v>2662</v>
       </c>
       <c r="C2278" t="inlineStr">
         <is>
-          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
         </is>
       </c>
       <c r="D2278" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2279">
@@ -41445,15 +41445,15 @@
         </is>
       </c>
       <c r="B2279" t="n">
-        <v>2718</v>
+        <v>2663</v>
       </c>
       <c r="C2279" t="inlineStr">
         <is>
-          <t>KALILLA FERREIRA COSTA - FARMA</t>
+          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
         </is>
       </c>
       <c r="D2279" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2280">
@@ -41463,11 +41463,11 @@
         </is>
       </c>
       <c r="B2280" t="n">
-        <v>2674</v>
+        <v>2685</v>
       </c>
       <c r="C2280" t="inlineStr">
         <is>
-          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
+          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2280" t="n">
@@ -41481,15 +41481,15 @@
         </is>
       </c>
       <c r="B2281" t="n">
-        <v>2753</v>
+        <v>2718</v>
       </c>
       <c r="C2281" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA - HB</t>
+          <t>KALILLA FERREIRA COSTA - FARMA</t>
         </is>
       </c>
       <c r="D2281" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2282">
@@ -41499,15 +41499,15 @@
         </is>
       </c>
       <c r="B2282" t="n">
-        <v>2772</v>
+        <v>2674</v>
       </c>
       <c r="C2282" t="inlineStr">
         <is>
-          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
+          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
         </is>
       </c>
       <c r="D2282" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2283">
@@ -41517,69 +41517,69 @@
         </is>
       </c>
       <c r="B2283" t="n">
-        <v>2827</v>
+        <v>2753</v>
       </c>
       <c r="C2283" t="inlineStr">
         <is>
-          <t>JOELTON MUNIZ DE SOUZA - HB</t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA - HB</t>
         </is>
       </c>
       <c r="D2283" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2284">
       <c r="A2284" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2284" t="n">
-        <v>2756</v>
+        <v>2772</v>
       </c>
       <c r="C2284" t="inlineStr">
         <is>
-          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
+          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2284" t="n">
-        <v>39</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2285">
       <c r="A2285" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2285" t="n">
-        <v>2813</v>
+        <v>2827</v>
       </c>
       <c r="C2285" t="inlineStr">
         <is>
-          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
+          <t>JOELTON MUNIZ DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2285" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2286">
       <c r="A2286" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2286" t="n">
-        <v>2738</v>
+        <v>2756</v>
       </c>
       <c r="C2286" t="inlineStr">
         <is>
-          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
+          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
         </is>
       </c>
       <c r="D2286" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2287">
@@ -41589,15 +41589,15 @@
         </is>
       </c>
       <c r="B2287" t="n">
-        <v>2739</v>
+        <v>2813</v>
       </c>
       <c r="C2287" t="inlineStr">
         <is>
-          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
+          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
         </is>
       </c>
       <c r="D2287" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2288">
@@ -41607,87 +41607,87 @@
         </is>
       </c>
       <c r="B2288" t="n">
-        <v>2824</v>
+        <v>2738</v>
       </c>
       <c r="C2288" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2288" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2289">
       <c r="A2289" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2289" t="n">
-        <v>2747</v>
+        <v>2739</v>
       </c>
       <c r="C2289" t="inlineStr">
         <is>
-          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
+          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2289" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2290">
       <c r="A2290" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2290" t="n">
-        <v>2748</v>
+        <v>2824</v>
       </c>
       <c r="C2290" t="inlineStr">
         <is>
-          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D2290" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2291">
       <c r="A2291" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2291" t="n">
-        <v>2766</v>
+        <v>2747</v>
       </c>
       <c r="C2291" t="inlineStr">
         <is>
-          <t>SETOR VAGO PEDREIRAS</t>
+          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
         </is>
       </c>
       <c r="D2291" t="n">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2292">
       <c r="A2292" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2292" t="n">
-        <v>2767</v>
+        <v>2748</v>
       </c>
       <c r="C2292" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
         </is>
       </c>
       <c r="D2292" t="n">
-        <v>39</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2293">
@@ -41697,51 +41697,51 @@
         </is>
       </c>
       <c r="B2293" t="n">
-        <v>2688</v>
+        <v>2766</v>
       </c>
       <c r="C2293" t="inlineStr">
         <is>
-          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
+          <t>SETOR VAGO PEDREIRAS</t>
         </is>
       </c>
       <c r="D2293" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2294">
       <c r="A2294" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2294" t="n">
-        <v>2694</v>
+        <v>2767</v>
       </c>
       <c r="C2294" t="inlineStr">
         <is>
-          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D2294" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2295">
       <c r="A2295" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2295" t="n">
-        <v>2714</v>
+        <v>2688</v>
       </c>
       <c r="C2295" t="inlineStr">
         <is>
-          <t>PRISCILA DOS SANTOS LOPES - HB</t>
+          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2295" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2296">
@@ -41751,15 +41751,15 @@
         </is>
       </c>
       <c r="B2296" t="n">
-        <v>2722</v>
+        <v>2694</v>
       </c>
       <c r="C2296" t="inlineStr">
         <is>
-          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
+          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2296" t="n">
-        <v>50</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2297">
@@ -41769,15 +41769,15 @@
         </is>
       </c>
       <c r="B2297" t="n">
-        <v>2723</v>
+        <v>2714</v>
       </c>
       <c r="C2297" t="inlineStr">
         <is>
-          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
+          <t>PRISCILA DOS SANTOS LOPES - HB</t>
         </is>
       </c>
       <c r="D2297" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2298">
@@ -41787,15 +41787,15 @@
         </is>
       </c>
       <c r="B2298" t="n">
-        <v>2803</v>
+        <v>2722</v>
       </c>
       <c r="C2298" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
+          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
         </is>
       </c>
       <c r="D2298" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2299">
@@ -41805,249 +41805,249 @@
         </is>
       </c>
       <c r="B2299" t="n">
-        <v>2804</v>
+        <v>2723</v>
       </c>
       <c r="C2299" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA - HB</t>
+          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2299" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2300">
       <c r="A2300" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2300" t="n">
-        <v>2830</v>
+        <v>2803</v>
       </c>
       <c r="C2300" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 1</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
         </is>
       </c>
       <c r="D2300" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2301">
       <c r="A2301" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2301" t="n">
-        <v>2831</v>
+        <v>2804</v>
       </c>
       <c r="C2301" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 2</t>
+          <t>PAULA CARLA CALDAS MOTA - HB</t>
         </is>
       </c>
       <c r="D2301" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2302">
       <c r="A2302" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2302" t="n">
-        <v>2647</v>
+        <v>2830</v>
       </c>
       <c r="C2302" t="inlineStr">
         <is>
-          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
+          <t>SETOR VAGO BALSAS 1</t>
         </is>
       </c>
       <c r="D2302" t="n">
-        <v>147</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2303">
       <c r="A2303" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2303" t="n">
-        <v>2661</v>
+        <v>2831</v>
       </c>
       <c r="C2303" t="inlineStr">
         <is>
-          <t>MARIA ISADORA DOS REIS REGO</t>
+          <t>SETOR VAGO BALSAS 2</t>
         </is>
       </c>
       <c r="D2303" t="n">
-        <v>76</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2304">
       <c r="A2304" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2304" t="n">
-        <v>2686</v>
+        <v>2647</v>
       </c>
       <c r="C2304" t="inlineStr">
         <is>
-          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
+          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
         </is>
       </c>
       <c r="D2304" t="n">
-        <v>120</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2305">
       <c r="A2305" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2305" t="n">
-        <v>2687</v>
+        <v>2661</v>
       </c>
       <c r="C2305" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
+          <t>MARIA ISADORA DOS REIS REGO</t>
         </is>
       </c>
       <c r="D2305" t="n">
-        <v>120</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2306">
       <c r="A2306" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2306" t="n">
-        <v>2681</v>
+        <v>2686</v>
       </c>
       <c r="C2306" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL PI</t>
+          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2306" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2307">
       <c r="A2307" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2307" t="n">
-        <v>2682</v>
+        <v>2687</v>
       </c>
       <c r="C2307" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL MA</t>
+          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
         </is>
       </c>
       <c r="D2307" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2308">
       <c r="A2308" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2308" t="n">
-        <v>2826</v>
+        <v>2681</v>
       </c>
       <c r="C2308" t="inlineStr">
         <is>
-          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
+          <t>RCA PRINCIPIA OL PI</t>
         </is>
       </c>
       <c r="D2308" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2309">
       <c r="A2309" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2309" t="n">
-        <v>2677</v>
+        <v>2682</v>
       </c>
       <c r="C2309" t="inlineStr">
         <is>
-          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
+          <t>RCA PRINCIPIA OL MA</t>
         </is>
       </c>
       <c r="D2309" t="n">
-        <v>72</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2310">
       <c r="A2310" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2310" t="n">
-        <v>2678</v>
+        <v>2826</v>
       </c>
       <c r="C2310" t="inlineStr">
         <is>
-          <t>ADRIEL XERXES BARROS MARTINS</t>
+          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
         </is>
       </c>
       <c r="D2310" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2311" t="n">
-        <v>2735</v>
+        <v>2677</v>
       </c>
       <c r="C2311" t="inlineStr">
         <is>
-          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
+          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
         </is>
       </c>
       <c r="D2311" t="n">
-        <v>100</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2312">
       <c r="A2312" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2312" t="n">
-        <v>2736</v>
+        <v>2678</v>
       </c>
       <c r="C2312" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
+          <t>ADRIEL XERXES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D2312" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2313">
@@ -42057,11 +42057,11 @@
         </is>
       </c>
       <c r="B2313" t="n">
-        <v>2737</v>
+        <v>2735</v>
       </c>
       <c r="C2313" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
+          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2313" t="n">
@@ -42075,11 +42075,11 @@
         </is>
       </c>
       <c r="B2314" t="n">
-        <v>2743</v>
+        <v>2736</v>
       </c>
       <c r="C2314" t="inlineStr">
         <is>
-          <t>VAGO SEABRA - FARMA</t>
+          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2314" t="n">
@@ -42093,15 +42093,15 @@
         </is>
       </c>
       <c r="B2315" t="n">
-        <v>2744</v>
+        <v>2737</v>
       </c>
       <c r="C2315" t="inlineStr">
         <is>
-          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
         </is>
       </c>
       <c r="D2315" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2316">
@@ -42111,15 +42111,15 @@
         </is>
       </c>
       <c r="B2316" t="n">
-        <v>2745</v>
+        <v>2743</v>
       </c>
       <c r="C2316" t="inlineStr">
         <is>
-          <t>CIRLANE ARAUJO SOUZA - HB</t>
+          <t>VAGO SEABRA - FARMA</t>
         </is>
       </c>
       <c r="D2316" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2317">
@@ -42129,11 +42129,11 @@
         </is>
       </c>
       <c r="B2317" t="n">
-        <v>2783</v>
+        <v>2744</v>
       </c>
       <c r="C2317" t="inlineStr">
         <is>
-          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
+          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
         </is>
       </c>
       <c r="D2317" t="n">
@@ -42143,19 +42143,19 @@
     <row r="2318">
       <c r="A2318" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2318" t="n">
-        <v>2768</v>
+        <v>2745</v>
       </c>
       <c r="C2318" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>CIRLANE ARAUJO SOUZA - HB</t>
         </is>
       </c>
       <c r="D2318" t="n">
-        <v>69</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2319">
@@ -42165,15 +42165,15 @@
         </is>
       </c>
       <c r="B2319" t="n">
-        <v>2703</v>
+        <v>2783</v>
       </c>
       <c r="C2319" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2319" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2320">
@@ -42183,15 +42183,15 @@
         </is>
       </c>
       <c r="B2320" t="n">
-        <v>2828</v>
+        <v>2768</v>
       </c>
       <c r="C2320" t="inlineStr">
         <is>
-          <t>LYERKA MARDANIA RODRIGUES MELO</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2320" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2321">
@@ -42201,69 +42201,69 @@
         </is>
       </c>
       <c r="B2321" t="n">
-        <v>2750</v>
+        <v>2703</v>
       </c>
       <c r="C2321" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2321" t="n">
-        <v>50</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2322">
       <c r="A2322" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2322" t="n">
-        <v>2689</v>
+        <v>2828</v>
       </c>
       <c r="C2322" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>LYERKA MARDANIA RODRIGUES MELO</t>
         </is>
       </c>
       <c r="D2322" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2323">
       <c r="A2323" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2708</v>
+        <v>2750</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2323" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2324">
       <c r="A2324" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2709</v>
+        <v>2689</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2324" t="n">
-        <v>39</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2325">
@@ -42273,11 +42273,11 @@
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2789</v>
+        <v>2708</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2325" t="n">
@@ -42287,73 +42287,73 @@
     <row r="2326">
       <c r="A2326" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2790</v>
+        <v>2709</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
+          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
         </is>
       </c>
       <c r="D2326" t="n">
-        <v>114</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2327">
       <c r="A2327" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2791</v>
+        <v>2789</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>DANIELY PEREIRA PINHEIRO</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2327" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2328">
       <c r="A2328" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2805</v>
+        <v>2790</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
         </is>
       </c>
       <c r="D2328" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2806</v>
+        <v>2791</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>DANIELY PEREIRA PINHEIRO</t>
         </is>
       </c>
       <c r="D2329" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2330">
@@ -42363,11 +42363,11 @@
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2807</v>
+        <v>2805</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2330" t="n">
@@ -42381,11 +42381,11 @@
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2808</v>
+        <v>2806</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2331" t="n">
@@ -42395,37 +42395,37 @@
     <row r="2332">
       <c r="A2332" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2820</v>
+        <v>2807</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2332" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2333">
       <c r="A2333" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2765</v>
+        <v>2808</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2333" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2334">
@@ -42435,15 +42435,15 @@
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2741</v>
+        <v>2820</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2334" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2335">
@@ -42453,51 +42453,51 @@
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2758</v>
+        <v>2765</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2335" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2336">
       <c r="A2336" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2659</v>
+        <v>2741</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2336" t="n">
-        <v>100</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2337">
       <c r="A2337" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2669</v>
+        <v>2758</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2337" t="n">
-        <v>135</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2338">
@@ -42507,141 +42507,141 @@
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2672</v>
+        <v>2659</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2338" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2339">
       <c r="A2339" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2673</v>
+        <v>2669</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2339" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2676</v>
+        <v>2672</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2341">
       <c r="A2341" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2760</v>
+        <v>2673</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2341" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2342">
       <c r="A2342" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2823</v>
+        <v>2676</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2343">
       <c r="A2343" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2792</v>
+        <v>2760</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2343" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2344">
       <c r="A2344" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2344" t="n">
-        <v>2793</v>
+        <v>2823</v>
       </c>
       <c r="C2344" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2344" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2345">
       <c r="A2345" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2345" t="n">
-        <v>2802</v>
+        <v>2792</v>
       </c>
       <c r="C2345" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2345" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2346">
@@ -42651,11 +42651,11 @@
         </is>
       </c>
       <c r="B2346" t="n">
-        <v>2656</v>
+        <v>2793</v>
       </c>
       <c r="C2346" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2346" t="n">
@@ -42665,19 +42665,19 @@
     <row r="2347">
       <c r="A2347" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2347" t="n">
-        <v>2657</v>
+        <v>2802</v>
       </c>
       <c r="C2347" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2347" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2348">
@@ -42687,33 +42687,33 @@
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2658</v>
+        <v>2656</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2348" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2349">
       <c r="A2349" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2729</v>
+        <v>2657</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D2349" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2350">
@@ -42723,33 +42723,33 @@
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2759</v>
+        <v>2658</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2350" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2351">
       <c r="A2351" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2832</v>
+        <v>2729</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2351" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2352">
@@ -42759,11 +42759,11 @@
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2769</v>
+        <v>2759</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2352" t="n">
@@ -42773,73 +42773,73 @@
     <row r="2353">
       <c r="A2353" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2679</v>
+        <v>2832</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
         </is>
       </c>
       <c r="D2353" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2354">
       <c r="A2354" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2680</v>
+        <v>2769</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2354" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2355">
       <c r="A2355" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2815</v>
+        <v>2679</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2355" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2356">
       <c r="A2356" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2816</v>
+        <v>2680</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2356" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2357">
@@ -42849,87 +42849,87 @@
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2817</v>
+        <v>2815</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2357" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2358">
       <c r="A2358" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2701</v>
+        <v>2816</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2358" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2359">
       <c r="A2359" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2644</v>
+        <v>2817</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2359" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2360">
       <c r="A2360" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2645</v>
+        <v>2701</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2361">
       <c r="A2361" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2754</v>
+        <v>2644</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2361" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2362">
@@ -42939,51 +42939,51 @@
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2755</v>
+        <v>2645</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2362" t="n">
-        <v>80</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2363">
       <c r="A2363" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2665</v>
+        <v>2754</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2363" t="n">
-        <v>141</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2364">
       <c r="A2364" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2667</v>
+        <v>2755</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2364" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2365">
@@ -42993,15 +42993,15 @@
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2727</v>
+        <v>2665</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2365" t="n">
-        <v>120</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2366">
@@ -43011,51 +43011,51 @@
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2728</v>
+        <v>2667</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
         </is>
       </c>
       <c r="D2366" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2367">
       <c r="A2367" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2833</v>
+        <v>2727</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>ADEILZA PINTO DA SILVA - FARMA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2368">
       <c r="A2368" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2814</v>
+        <v>2728</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2368" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2369">
@@ -43065,11 +43065,11 @@
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2646</v>
+        <v>2833</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>ADEILZA PINTO DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2369" t="n">
@@ -43079,19 +43079,19 @@
     <row r="2370">
       <c r="A2370" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2650</v>
+        <v>2814</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2371">
@@ -43101,15 +43101,15 @@
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2652</v>
+        <v>2646</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2372">
@@ -43119,11 +43119,11 @@
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2653</v>
+        <v>2650</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2372" t="n">
@@ -43137,15 +43137,15 @@
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2654</v>
+        <v>2652</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2374">
@@ -43155,33 +43155,33 @@
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2655</v>
+        <v>2653</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2375">
       <c r="A2375" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2821</v>
+        <v>2654</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2375" t="n">
-        <v>69</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2376">
@@ -43191,159 +43191,159 @@
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2683</v>
+        <v>2655</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2376" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2684</v>
+        <v>2821</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2377" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2378">
       <c r="A2378" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2749</v>
+        <v>2683</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>111</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2379">
       <c r="A2379" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2812</v>
+        <v>2684</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2379" t="n">
-        <v>145</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2380">
       <c r="A2380" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2715</v>
+        <v>2749</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2380" t="n">
-        <v>90</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2381">
       <c r="A2381" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2834</v>
+        <v>2812</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>GILVANA DA SILVA MONTELES</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>114</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2382">
       <c r="A2382" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2651</v>
+        <v>2715</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>145</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2383">
       <c r="A2383" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2819</v>
+        <v>2834</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2835</v>
+        <v>2651</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>ROGÉRIO LIRA DA GAMA</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>116</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2385">
@@ -43353,11 +43353,11 @@
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2699</v>
+        <v>2819</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2385" t="n">
@@ -43367,109 +43367,109 @@
     <row r="2386">
       <c r="A2386" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2706</v>
+        <v>2835</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS BARREIRINHAS</t>
+          <t>ROGÉRIO LIRA DA GAMA</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2387">
       <c r="A2387" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2707</v>
+        <v>2699</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>EVANESSA DA SILVA E SILVA</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2693</v>
+        <v>2706</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>SETOR VAGO PLUS BARREIRINHAS</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>80</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2389">
       <c r="A2389" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2705</v>
+        <v>2707</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>EVANESSA DA SILVA E SILVA</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>146</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2664</v>
+        <v>2693</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2670</v>
+        <v>2705</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>69</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2392">
@@ -43479,141 +43479,141 @@
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2730</v>
+        <v>2664</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2671</v>
+        <v>2670</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2394">
       <c r="A2394" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2691</v>
+        <v>2730</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2692</v>
+        <v>2671</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2396">
       <c r="A2396" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2724</v>
+        <v>2691</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2397">
       <c r="A2397" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2773</v>
+        <v>2692</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>VIVIANE LEAL DA SILVA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2825</v>
+        <v>2724</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2787</v>
+        <v>2773</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>VIVIANE LEAL DA SILVA</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2400">
@@ -43623,51 +43623,51 @@
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2648</v>
+        <v>2825</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2401">
       <c r="A2401" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2666</v>
+        <v>2787</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>63</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2402">
       <c r="A2402" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2779</v>
+        <v>2648</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>105</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2403">
@@ -43677,15 +43677,15 @@
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2780</v>
+        <v>2666</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2404">
@@ -43695,51 +43695,51 @@
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2786</v>
+        <v>2779</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2405">
       <c r="A2405" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2660</v>
+        <v>2780</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>38</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2716</v>
+        <v>2786</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2407">
@@ -43749,51 +43749,51 @@
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2734</v>
+        <v>2660</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2742</v>
+        <v>2716</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2794</v>
+        <v>2734</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2410">
@@ -43803,11 +43803,11 @@
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2795</v>
+        <v>2742</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2410" t="n">
@@ -43821,15 +43821,15 @@
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2796</v>
+        <v>2794</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2412">
@@ -43839,11 +43839,11 @@
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2797</v>
+        <v>2795</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
         </is>
       </c>
       <c r="D2412" t="n">
@@ -43857,11 +43857,11 @@
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2798</v>
+        <v>2796</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2413" t="n">
@@ -43871,73 +43871,73 @@
     <row r="2414">
       <c r="A2414" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2668</v>
+        <v>2797</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2415">
       <c r="A2415" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2690</v>
+        <v>2798</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2415" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2416">
       <c r="A2416" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2696</v>
+        <v>2668</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2416" t="n">
-        <v>69</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2417">
       <c r="A2417" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2697</v>
+        <v>2690</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2418">
@@ -43947,11 +43947,11 @@
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2698</v>
+        <v>2696</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2418" t="n">
@@ -43961,37 +43961,37 @@
     <row r="2419">
       <c r="A2419" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2775</v>
+        <v>2697</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2419" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2420">
       <c r="A2420" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2776</v>
+        <v>2698</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2421">
@@ -44001,11 +44001,11 @@
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2777</v>
+        <v>2775</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2421" t="n">
@@ -44019,11 +44019,11 @@
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2778</v>
+        <v>2776</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2422" t="n">
@@ -44037,15 +44037,15 @@
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2781</v>
+        <v>2777</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2424">
@@ -44055,11 +44055,11 @@
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2822</v>
+        <v>2778</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2424" t="n">
@@ -44073,87 +44073,87 @@
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2740</v>
+        <v>2781</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2425" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2426">
       <c r="A2426" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2710</v>
+        <v>2822</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2426" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2427">
       <c r="A2427" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2711</v>
+        <v>2740</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2427" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2428">
       <c r="A2428" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2712</v>
+        <v>2710</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2428" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2429">
       <c r="A2429" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2717</v>
+        <v>2711</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D2429" t="n">
-        <v>69</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2430">
@@ -44163,14 +44163,50 @@
         </is>
       </c>
       <c r="B2430" t="n">
+        <v>2712</v>
+      </c>
+      <c r="C2430" t="inlineStr">
+        <is>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
+        </is>
+      </c>
+      <c r="D2430" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2431">
+      <c r="A2431" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2431" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2431" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2431" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2432">
+      <c r="A2432" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2432" t="n">
         <v>2801</v>
       </c>
-      <c r="C2430" t="inlineStr">
+      <c r="C2432" t="inlineStr">
         <is>
           <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
-      <c r="D2430" t="n">
+      <c r="D2432" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:03:01
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2432"/>
+  <dimension ref="A1:D2433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41319,15 +41319,15 @@
         </is>
       </c>
       <c r="B2272" t="n">
-        <v>2799</v>
+        <v>2838</v>
       </c>
       <c r="C2272" t="inlineStr">
         <is>
-          <t>VOLFRAMIO DALFREDO ALMEIDA</t>
+          <t>CAIO LUA MENDES DE ARAUJO</t>
         </is>
       </c>
       <c r="D2272" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2273">
@@ -41337,33 +41337,33 @@
         </is>
       </c>
       <c r="B2273" t="n">
-        <v>2719</v>
+        <v>2799</v>
       </c>
       <c r="C2273" t="inlineStr">
         <is>
-          <t>SETOR SÃO RDO NONATO VAGO  (DEDICADA)</t>
+          <t>VOLFRAMIO DALFREDO ALMEIDA</t>
         </is>
       </c>
       <c r="D2273" t="n">
-        <v>39</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2274">
       <c r="A2274" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2274" t="n">
-        <v>2731</v>
+        <v>2719</v>
       </c>
       <c r="C2274" t="inlineStr">
         <is>
-          <t>VAGO ANDERSON A. S. - FARMA (CAMAÇARI)</t>
+          <t>SETOR SÃO RDO NONATO VAGO  (DEDICADA)</t>
         </is>
       </c>
       <c r="D2274" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2275">
@@ -41373,15 +41373,15 @@
         </is>
       </c>
       <c r="B2275" t="n">
-        <v>2732</v>
+        <v>2731</v>
       </c>
       <c r="C2275" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN DE JESUS - HB</t>
+          <t>VAGO ANDERSON A. S. - FARMA (CAMAÇARI)</t>
         </is>
       </c>
       <c r="D2275" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2276">
@@ -41391,51 +41391,51 @@
         </is>
       </c>
       <c r="B2276" t="n">
-        <v>2733</v>
+        <v>2732</v>
       </c>
       <c r="C2276" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAGO CENTRO CAROLINE LEMOS - FARMA </t>
+          <t>VAGO BRENO ALLAN DE JESUS - HB</t>
         </is>
       </c>
       <c r="D2276" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2277">
       <c r="A2277" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2277" t="n">
-        <v>2752</v>
+        <v>2733</v>
       </c>
       <c r="C2277" t="inlineStr">
         <is>
-          <t>SETOR BAIXADA PLUS (ELILTON ROMEU)</t>
+          <t xml:space="preserve">VAGO CENTRO CAROLINE LEMOS - FARMA </t>
         </is>
       </c>
       <c r="D2277" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2278">
       <c r="A2278" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2278" t="n">
-        <v>2662</v>
+        <v>2752</v>
       </c>
       <c r="C2278" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
+          <t>SETOR BAIXADA PLUS (ELILTON ROMEU)</t>
         </is>
       </c>
       <c r="D2278" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2279">
@@ -41445,15 +41445,15 @@
         </is>
       </c>
       <c r="B2279" t="n">
-        <v>2663</v>
+        <v>2662</v>
       </c>
       <c r="C2279" t="inlineStr">
         <is>
-          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
         </is>
       </c>
       <c r="D2279" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2280">
@@ -41463,15 +41463,15 @@
         </is>
       </c>
       <c r="B2280" t="n">
-        <v>2685</v>
+        <v>2663</v>
       </c>
       <c r="C2280" t="inlineStr">
         <is>
-          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
+          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
         </is>
       </c>
       <c r="D2280" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2281">
@@ -41481,15 +41481,15 @@
         </is>
       </c>
       <c r="B2281" t="n">
-        <v>2718</v>
+        <v>2685</v>
       </c>
       <c r="C2281" t="inlineStr">
         <is>
-          <t>KALILLA FERREIRA COSTA - FARMA</t>
+          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2281" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2282">
@@ -41499,15 +41499,15 @@
         </is>
       </c>
       <c r="B2282" t="n">
-        <v>2674</v>
+        <v>2718</v>
       </c>
       <c r="C2282" t="inlineStr">
         <is>
-          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
+          <t>KALILLA FERREIRA COSTA - FARMA</t>
         </is>
       </c>
       <c r="D2282" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2283">
@@ -41517,15 +41517,15 @@
         </is>
       </c>
       <c r="B2283" t="n">
-        <v>2753</v>
+        <v>2674</v>
       </c>
       <c r="C2283" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA - HB</t>
+          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
         </is>
       </c>
       <c r="D2283" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2284">
@@ -41535,15 +41535,15 @@
         </is>
       </c>
       <c r="B2284" t="n">
-        <v>2772</v>
+        <v>2753</v>
       </c>
       <c r="C2284" t="inlineStr">
         <is>
-          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA - HB</t>
         </is>
       </c>
       <c r="D2284" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2285">
@@ -41553,51 +41553,51 @@
         </is>
       </c>
       <c r="B2285" t="n">
-        <v>2827</v>
+        <v>2772</v>
       </c>
       <c r="C2285" t="inlineStr">
         <is>
-          <t>JOELTON MUNIZ DE SOUZA - HB</t>
+          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2285" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2286">
       <c r="A2286" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2286" t="n">
-        <v>2756</v>
+        <v>2827</v>
       </c>
       <c r="C2286" t="inlineStr">
         <is>
-          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
+          <t>JOELTON MUNIZ DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2286" t="n">
-        <v>39</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2287">
       <c r="A2287" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2287" t="n">
-        <v>2813</v>
+        <v>2756</v>
       </c>
       <c r="C2287" t="inlineStr">
         <is>
-          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
+          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
         </is>
       </c>
       <c r="D2287" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2288">
@@ -41607,15 +41607,15 @@
         </is>
       </c>
       <c r="B2288" t="n">
-        <v>2738</v>
+        <v>2813</v>
       </c>
       <c r="C2288" t="inlineStr">
         <is>
-          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
+          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
         </is>
       </c>
       <c r="D2288" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2289">
@@ -41625,11 +41625,11 @@
         </is>
       </c>
       <c r="B2289" t="n">
-        <v>2739</v>
+        <v>2738</v>
       </c>
       <c r="C2289" t="inlineStr">
         <is>
-          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
+          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2289" t="n">
@@ -41643,33 +41643,33 @@
         </is>
       </c>
       <c r="B2290" t="n">
-        <v>2824</v>
+        <v>2739</v>
       </c>
       <c r="C2290" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2290" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2291">
       <c r="A2291" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2291" t="n">
-        <v>2747</v>
+        <v>2824</v>
       </c>
       <c r="C2291" t="inlineStr">
         <is>
-          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D2291" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2292">
@@ -41679,11 +41679,11 @@
         </is>
       </c>
       <c r="B2292" t="n">
-        <v>2748</v>
+        <v>2747</v>
       </c>
       <c r="C2292" t="inlineStr">
         <is>
-          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
+          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
         </is>
       </c>
       <c r="D2292" t="n">
@@ -41693,73 +41693,73 @@
     <row r="2293">
       <c r="A2293" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2293" t="n">
-        <v>2766</v>
+        <v>2748</v>
       </c>
       <c r="C2293" t="inlineStr">
         <is>
-          <t>SETOR VAGO PEDREIRAS</t>
+          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
         </is>
       </c>
       <c r="D2293" t="n">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2294">
       <c r="A2294" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2294" t="n">
-        <v>2767</v>
+        <v>2766</v>
       </c>
       <c r="C2294" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>SETOR VAGO PEDREIRAS</t>
         </is>
       </c>
       <c r="D2294" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2295">
       <c r="A2295" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2295" t="n">
-        <v>2688</v>
+        <v>2767</v>
       </c>
       <c r="C2295" t="inlineStr">
         <is>
-          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D2295" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2296">
       <c r="A2296" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2296" t="n">
-        <v>2694</v>
+        <v>2688</v>
       </c>
       <c r="C2296" t="inlineStr">
         <is>
-          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
+          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2296" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2297">
@@ -41769,15 +41769,15 @@
         </is>
       </c>
       <c r="B2297" t="n">
-        <v>2714</v>
+        <v>2694</v>
       </c>
       <c r="C2297" t="inlineStr">
         <is>
-          <t>PRISCILA DOS SANTOS LOPES - HB</t>
+          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2297" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2298">
@@ -41787,15 +41787,15 @@
         </is>
       </c>
       <c r="B2298" t="n">
-        <v>2722</v>
+        <v>2714</v>
       </c>
       <c r="C2298" t="inlineStr">
         <is>
-          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
+          <t>PRISCILA DOS SANTOS LOPES - HB</t>
         </is>
       </c>
       <c r="D2298" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2299">
@@ -41805,15 +41805,15 @@
         </is>
       </c>
       <c r="B2299" t="n">
-        <v>2723</v>
+        <v>2722</v>
       </c>
       <c r="C2299" t="inlineStr">
         <is>
-          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
+          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
         </is>
       </c>
       <c r="D2299" t="n">
-        <v>95</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2300">
@@ -41823,15 +41823,15 @@
         </is>
       </c>
       <c r="B2300" t="n">
-        <v>2803</v>
+        <v>2723</v>
       </c>
       <c r="C2300" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
+          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2300" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2301">
@@ -41841,11 +41841,11 @@
         </is>
       </c>
       <c r="B2301" t="n">
-        <v>2804</v>
+        <v>2803</v>
       </c>
       <c r="C2301" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA - HB</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
         </is>
       </c>
       <c r="D2301" t="n">
@@ -41855,19 +41855,19 @@
     <row r="2302">
       <c r="A2302" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2302" t="n">
-        <v>2830</v>
+        <v>2804</v>
       </c>
       <c r="C2302" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 1</t>
+          <t>PAULA CARLA CALDAS MOTA - HB</t>
         </is>
       </c>
       <c r="D2302" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2303">
@@ -41877,11 +41877,11 @@
         </is>
       </c>
       <c r="B2303" t="n">
-        <v>2831</v>
+        <v>2830</v>
       </c>
       <c r="C2303" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 2</t>
+          <t>SETOR VAGO BALSAS 1</t>
         </is>
       </c>
       <c r="D2303" t="n">
@@ -41891,55 +41891,55 @@
     <row r="2304">
       <c r="A2304" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2304" t="n">
-        <v>2647</v>
+        <v>2831</v>
       </c>
       <c r="C2304" t="inlineStr">
         <is>
-          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
+          <t>SETOR VAGO BALSAS 2</t>
         </is>
       </c>
       <c r="D2304" t="n">
-        <v>147</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2305">
       <c r="A2305" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2305" t="n">
-        <v>2661</v>
+        <v>2647</v>
       </c>
       <c r="C2305" t="inlineStr">
         <is>
-          <t>MARIA ISADORA DOS REIS REGO</t>
+          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
         </is>
       </c>
       <c r="D2305" t="n">
-        <v>76</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2306">
       <c r="A2306" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2306" t="n">
-        <v>2686</v>
+        <v>2661</v>
       </c>
       <c r="C2306" t="inlineStr">
         <is>
-          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
+          <t>MARIA ISADORA DOS REIS REGO</t>
         </is>
       </c>
       <c r="D2306" t="n">
-        <v>120</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2307">
@@ -41949,11 +41949,11 @@
         </is>
       </c>
       <c r="B2307" t="n">
-        <v>2687</v>
+        <v>2686</v>
       </c>
       <c r="C2307" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
+          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2307" t="n">
@@ -41963,109 +41963,109 @@
     <row r="2308">
       <c r="A2308" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2308" t="n">
-        <v>2681</v>
+        <v>2687</v>
       </c>
       <c r="C2308" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL PI</t>
+          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
         </is>
       </c>
       <c r="D2308" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2309">
       <c r="A2309" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2309" t="n">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="C2309" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL MA</t>
+          <t>RCA PRINCIPIA OL PI</t>
         </is>
       </c>
       <c r="D2309" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2310">
       <c r="A2310" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2310" t="n">
-        <v>2826</v>
+        <v>2682</v>
       </c>
       <c r="C2310" t="inlineStr">
         <is>
-          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
+          <t>RCA PRINCIPIA OL MA</t>
         </is>
       </c>
       <c r="D2310" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2311" t="n">
-        <v>2677</v>
+        <v>2826</v>
       </c>
       <c r="C2311" t="inlineStr">
         <is>
-          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
+          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
         </is>
       </c>
       <c r="D2311" t="n">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2312">
       <c r="A2312" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2312" t="n">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="C2312" t="inlineStr">
         <is>
-          <t>ADRIEL XERXES BARROS MARTINS</t>
+          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
         </is>
       </c>
       <c r="D2312" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2313">
       <c r="A2313" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2313" t="n">
-        <v>2735</v>
+        <v>2678</v>
       </c>
       <c r="C2313" t="inlineStr">
         <is>
-          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
+          <t>ADRIEL XERXES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D2313" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2314">
@@ -42075,15 +42075,15 @@
         </is>
       </c>
       <c r="B2314" t="n">
-        <v>2736</v>
+        <v>2735</v>
       </c>
       <c r="C2314" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
+          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2314" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2315">
@@ -42093,15 +42093,15 @@
         </is>
       </c>
       <c r="B2315" t="n">
-        <v>2737</v>
+        <v>2736</v>
       </c>
       <c r="C2315" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
+          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2315" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2316">
@@ -42111,15 +42111,15 @@
         </is>
       </c>
       <c r="B2316" t="n">
-        <v>2743</v>
+        <v>2737</v>
       </c>
       <c r="C2316" t="inlineStr">
         <is>
-          <t>VAGO SEABRA - FARMA</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
         </is>
       </c>
       <c r="D2316" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2317">
@@ -42129,11 +42129,11 @@
         </is>
       </c>
       <c r="B2317" t="n">
-        <v>2744</v>
+        <v>2743</v>
       </c>
       <c r="C2317" t="inlineStr">
         <is>
-          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
+          <t>VAGO SEABRA - FARMA</t>
         </is>
       </c>
       <c r="D2317" t="n">
@@ -42147,15 +42147,15 @@
         </is>
       </c>
       <c r="B2318" t="n">
-        <v>2745</v>
+        <v>2744</v>
       </c>
       <c r="C2318" t="inlineStr">
         <is>
-          <t>CIRLANE ARAUJO SOUZA - HB</t>
+          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
         </is>
       </c>
       <c r="D2318" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2319">
@@ -42165,105 +42165,105 @@
         </is>
       </c>
       <c r="B2319" t="n">
-        <v>2783</v>
+        <v>2745</v>
       </c>
       <c r="C2319" t="inlineStr">
         <is>
-          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
+          <t>CIRLANE ARAUJO SOUZA - HB</t>
         </is>
       </c>
       <c r="D2319" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2320">
       <c r="A2320" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2320" t="n">
-        <v>2768</v>
+        <v>2783</v>
       </c>
       <c r="C2320" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2320" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2321">
       <c r="A2321" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2321" t="n">
-        <v>2703</v>
+        <v>2768</v>
       </c>
       <c r="C2321" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2321" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2322">
       <c r="A2322" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2322" t="n">
-        <v>2828</v>
+        <v>2703</v>
       </c>
       <c r="C2322" t="inlineStr">
         <is>
-          <t>LYERKA MARDANIA RODRIGUES MELO</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2322" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2323">
       <c r="A2323" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2750</v>
+        <v>2828</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>LYERKA MARDANIA RODRIGUES MELO</t>
         </is>
       </c>
       <c r="D2323" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2324">
       <c r="A2324" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2689</v>
+        <v>2750</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2324" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2325">
@@ -42273,69 +42273,69 @@
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2708</v>
+        <v>2689</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2325" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2326">
       <c r="A2326" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2709</v>
+        <v>2708</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2326" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2327">
       <c r="A2327" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2789</v>
+        <v>2709</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
         </is>
       </c>
       <c r="D2327" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2328">
       <c r="A2328" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2790</v>
+        <v>2789</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2328" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2329">
@@ -42345,11 +42345,11 @@
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2791</v>
+        <v>2790</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>DANIELY PEREIRA PINHEIRO</t>
+          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
         </is>
       </c>
       <c r="D2329" t="n">
@@ -42359,19 +42359,19 @@
     <row r="2330">
       <c r="A2330" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2805</v>
+        <v>2791</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>DANIELY PEREIRA PINHEIRO</t>
         </is>
       </c>
       <c r="D2330" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2331">
@@ -42381,11 +42381,11 @@
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2806</v>
+        <v>2805</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2331" t="n">
@@ -42399,11 +42399,11 @@
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2807</v>
+        <v>2806</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2332" t="n">
@@ -42417,11 +42417,11 @@
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2808</v>
+        <v>2807</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2333" t="n">
@@ -42431,73 +42431,73 @@
     <row r="2334">
       <c r="A2334" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2820</v>
+        <v>2808</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2334" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2765</v>
+        <v>2820</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2335" t="n">
-        <v>98</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2336">
       <c r="A2336" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2741</v>
+        <v>2765</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2336" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2337">
       <c r="A2337" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2758</v>
+        <v>2741</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2337" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2338">
@@ -42507,51 +42507,51 @@
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2659</v>
+        <v>2758</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2338" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2339">
       <c r="A2339" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2669</v>
+        <v>2659</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2339" t="n">
-        <v>135</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2672</v>
+        <v>2669</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2341">
@@ -42561,11 +42561,11 @@
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2341" t="n">
@@ -42575,19 +42575,19 @@
     <row r="2342">
       <c r="A2342" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2676</v>
+        <v>2673</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2343">
@@ -42597,69 +42597,69 @@
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2760</v>
+        <v>2676</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2343" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2344">
       <c r="A2344" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2344" t="n">
-        <v>2823</v>
+        <v>2760</v>
       </c>
       <c r="C2344" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2344" t="n">
-        <v>80</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2345">
       <c r="A2345" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2345" t="n">
-        <v>2792</v>
+        <v>2823</v>
       </c>
       <c r="C2345" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2345" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2346">
       <c r="A2346" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2346" t="n">
-        <v>2793</v>
+        <v>2792</v>
       </c>
       <c r="C2346" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2346" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2347">
@@ -42669,15 +42669,15 @@
         </is>
       </c>
       <c r="B2347" t="n">
-        <v>2802</v>
+        <v>2793</v>
       </c>
       <c r="C2347" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2347" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2348">
@@ -42687,47 +42687,47 @@
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2656</v>
+        <v>2802</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2348" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2349">
       <c r="A2349" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2657</v>
+        <v>2656</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2349" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2350">
       <c r="A2350" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D2350" t="n">
@@ -42737,37 +42737,37 @@
     <row r="2351">
       <c r="A2351" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2729</v>
+        <v>2658</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2351" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2352">
       <c r="A2352" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2759</v>
+        <v>2729</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2352" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2353">
@@ -42777,15 +42777,15 @@
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2832</v>
+        <v>2759</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2353" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2354">
@@ -42795,33 +42795,33 @@
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2769</v>
+        <v>2832</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
         </is>
       </c>
       <c r="D2354" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2355">
       <c r="A2355" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2679</v>
+        <v>2769</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2355" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2356">
@@ -42831,11 +42831,11 @@
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2356" t="n">
@@ -42845,19 +42845,19 @@
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2815</v>
+        <v>2680</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2357" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2358">
@@ -42867,15 +42867,15 @@
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2816</v>
+        <v>2815</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2358" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2359">
@@ -42885,11 +42885,11 @@
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2817</v>
+        <v>2816</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2359" t="n">
@@ -42899,19 +42899,19 @@
     <row r="2360">
       <c r="A2360" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2701</v>
+        <v>2817</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2361">
@@ -42921,29 +42921,29 @@
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2644</v>
+        <v>2701</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2361" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2362">
       <c r="A2362" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2645</v>
+        <v>2644</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2362" t="n">
@@ -42957,15 +42957,15 @@
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2754</v>
+        <v>2645</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2363" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2364">
@@ -42975,33 +42975,33 @@
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2755</v>
+        <v>2754</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2364" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2365">
       <c r="A2365" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2665</v>
+        <v>2755</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2365" t="n">
-        <v>141</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2366">
@@ -43011,15 +43011,15 @@
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2667</v>
+        <v>2665</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2366" t="n">
-        <v>114</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2367">
@@ -43029,15 +43029,15 @@
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2727</v>
+        <v>2667</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2368">
@@ -43047,11 +43047,11 @@
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2728</v>
+        <v>2727</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2368" t="n">
@@ -43061,55 +43061,55 @@
     <row r="2369">
       <c r="A2369" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2833</v>
+        <v>2728</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>ADEILZA PINTO DA SILVA - FARMA</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2369" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2370">
       <c r="A2370" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2814</v>
+        <v>2833</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>ADEILZA PINTO DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>39</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2646</v>
+        <v>2814</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2372">
@@ -43119,11 +43119,11 @@
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2650</v>
+        <v>2646</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2372" t="n">
@@ -43137,15 +43137,15 @@
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2652</v>
+        <v>2650</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2374">
@@ -43155,15 +43155,15 @@
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2375">
@@ -43173,15 +43173,15 @@
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2654</v>
+        <v>2653</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2375" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2376">
@@ -43191,51 +43191,51 @@
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2655</v>
+        <v>2654</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2376" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2821</v>
+        <v>2655</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2377" t="n">
-        <v>69</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2378">
       <c r="A2378" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2683</v>
+        <v>2821</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2379">
@@ -43245,33 +43245,33 @@
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2379" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2380">
       <c r="A2380" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2749</v>
+        <v>2684</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2380" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2381">
@@ -43281,33 +43281,33 @@
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2812</v>
+        <v>2749</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>145</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2382">
       <c r="A2382" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2715</v>
+        <v>2812</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>90</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2383">
@@ -43317,105 +43317,105 @@
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2834</v>
+        <v>2715</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>GILVANA DA SILVA MONTELES</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2651</v>
+        <v>2834</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>145</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2385">
       <c r="A2385" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2819</v>
+        <v>2651</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2385" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2386">
       <c r="A2386" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2835</v>
+        <v>2819</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>ROGÉRIO LIRA DA GAMA</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>116</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2387">
       <c r="A2387" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2699</v>
+        <v>2835</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>ROGÉRIO LIRA DA GAMA</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>95</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2706</v>
+        <v>2699</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS BARREIRINHAS</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2389">
@@ -43425,11 +43425,11 @@
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2707</v>
+        <v>2706</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>EVANESSA DA SILVA E SILVA</t>
+          <t>SETOR VAGO PLUS BARREIRINHAS</t>
         </is>
       </c>
       <c r="D2389" t="n">
@@ -43439,127 +43439,127 @@
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2693</v>
+        <v>2707</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>EVANESSA DA SILVA E SILVA</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>80</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2705</v>
+        <v>2693</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>146</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2664</v>
+        <v>2705</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>90</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2670</v>
+        <v>2664</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2394">
       <c r="A2394" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2730</v>
+        <v>2670</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2671</v>
+        <v>2730</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2396">
       <c r="A2396" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2691</v>
+        <v>2671</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2397">
@@ -43569,11 +43569,11 @@
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2397" t="n">
@@ -43583,55 +43583,55 @@
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2724</v>
+        <v>2692</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2773</v>
+        <v>2724</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>VIVIANE LEAL DA SILVA</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2400">
       <c r="A2400" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2825</v>
+        <v>2773</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>VIVIANE LEAL DA SILVA</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2401">
@@ -43641,15 +43641,15 @@
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2787</v>
+        <v>2825</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2402">
@@ -43659,33 +43659,33 @@
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2648</v>
+        <v>2787</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2403">
       <c r="A2403" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2666</v>
+        <v>2648</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2404">
@@ -43695,15 +43695,15 @@
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2779</v>
+        <v>2666</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2405">
@@ -43713,11 +43713,11 @@
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2780</v>
+        <v>2779</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2405" t="n">
@@ -43731,33 +43731,33 @@
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2786</v>
+        <v>2780</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2407">
       <c r="A2407" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2660</v>
+        <v>2786</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2408">
@@ -43767,15 +43767,15 @@
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2716</v>
+        <v>2660</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2409">
@@ -43785,11 +43785,11 @@
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2734</v>
+        <v>2716</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2409" t="n">
@@ -43799,19 +43799,19 @@
     <row r="2410">
       <c r="A2410" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2742</v>
+        <v>2734</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2410" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2411">
@@ -43821,15 +43821,15 @@
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2794</v>
+        <v>2742</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2412">
@@ -43839,15 +43839,15 @@
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2795</v>
+        <v>2794</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2413">
@@ -43857,11 +43857,11 @@
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2796</v>
+        <v>2795</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VINICIUS RAMOS DOS P. - FAR (CAMAÇARÍ)</t>
         </is>
       </c>
       <c r="D2413" t="n">
@@ -43875,11 +43875,11 @@
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2797</v>
+        <v>2796</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2414" t="n">
@@ -43893,11 +43893,11 @@
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2798</v>
+        <v>2797</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2415" t="n">
@@ -43907,55 +43907,55 @@
     <row r="2416">
       <c r="A2416" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2668</v>
+        <v>2798</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2416" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2417">
       <c r="A2417" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2690</v>
+        <v>2668</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>38</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2418">
       <c r="A2418" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2696</v>
+        <v>2690</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2418" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2419">
@@ -43965,11 +43965,11 @@
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2419" t="n">
@@ -43983,11 +43983,11 @@
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2420" t="n">
@@ -43997,19 +43997,19 @@
     <row r="2421">
       <c r="A2421" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2775</v>
+        <v>2698</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2422">
@@ -44019,11 +44019,11 @@
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2776</v>
+        <v>2775</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2422" t="n">
@@ -44037,11 +44037,11 @@
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2777</v>
+        <v>2776</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2423" t="n">
@@ -44055,11 +44055,11 @@
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2778</v>
+        <v>2777</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2424" t="n">
@@ -44073,15 +44073,15 @@
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2781</v>
+        <v>2778</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2425" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2426">
@@ -44091,15 +44091,15 @@
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2822</v>
+        <v>2781</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2426" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2427">
@@ -44109,11 +44109,11 @@
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2740</v>
+        <v>2822</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2427" t="n">
@@ -44123,90 +44123,108 @@
     <row r="2428">
       <c r="A2428" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2710</v>
+        <v>2740</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2428" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2429">
       <c r="A2429" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2711</v>
+        <v>2710</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2429" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2430">
       <c r="A2430" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2430" t="n">
-        <v>2712</v>
+        <v>2711</v>
       </c>
       <c r="C2430" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D2430" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2431">
       <c r="A2431" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2431" t="n">
-        <v>2717</v>
+        <v>2712</v>
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
         </is>
       </c>
       <c r="D2431" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2432">
       <c r="A2432" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2432" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2432" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2432" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2433">
+      <c r="A2433" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2433" t="n">
         <v>2801</v>
       </c>
-      <c r="C2432" t="inlineStr">
+      <c r="C2433" t="inlineStr">
         <is>
           <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
-      <c r="D2432" t="n">
+      <c r="D2433" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:01:57
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2433"/>
+  <dimension ref="A1:D2435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43673,55 +43673,55 @@
     <row r="2403">
       <c r="A2403" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2648</v>
+        <v>2839</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>RCA TENA OL PI</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2404">
       <c r="A2404" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2666</v>
+        <v>2840</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>RCA TENA OL MA</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>63</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2405">
       <c r="A2405" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2779</v>
+        <v>2648</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>105</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2406">
@@ -43731,15 +43731,15 @@
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2780</v>
+        <v>2666</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2407">
@@ -43749,51 +43749,51 @@
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2786</v>
+        <v>2779</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2660</v>
+        <v>2780</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>38</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2716</v>
+        <v>2786</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2410">
@@ -43803,51 +43803,51 @@
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2734</v>
+        <v>2660</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2410" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2411">
       <c r="A2411" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2742</v>
+        <v>2716</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2412">
       <c r="A2412" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2794</v>
+        <v>2734</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2413">
@@ -43857,11 +43857,11 @@
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2795</v>
+        <v>2742</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2413" t="n">
@@ -43875,15 +43875,15 @@
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2796</v>
+        <v>2794</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2415">
@@ -43893,11 +43893,11 @@
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2797</v>
+        <v>2795</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
         </is>
       </c>
       <c r="D2415" t="n">
@@ -43911,11 +43911,11 @@
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2798</v>
+        <v>2796</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2416" t="n">
@@ -43925,73 +43925,73 @@
     <row r="2417">
       <c r="A2417" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2668</v>
+        <v>2797</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2418">
       <c r="A2418" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2690</v>
+        <v>2798</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2418" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2419">
       <c r="A2419" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2696</v>
+        <v>2668</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2419" t="n">
-        <v>69</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2420">
       <c r="A2420" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2697</v>
+        <v>2690</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2421">
@@ -44001,11 +44001,11 @@
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2698</v>
+        <v>2696</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2421" t="n">
@@ -44015,37 +44015,37 @@
     <row r="2422">
       <c r="A2422" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2775</v>
+        <v>2697</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2423">
       <c r="A2423" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2776</v>
+        <v>2698</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2424">
@@ -44055,11 +44055,11 @@
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2777</v>
+        <v>2775</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2424" t="n">
@@ -44073,11 +44073,11 @@
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2778</v>
+        <v>2776</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2425" t="n">
@@ -44091,15 +44091,15 @@
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2781</v>
+        <v>2777</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2426" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2427">
@@ -44109,11 +44109,11 @@
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2822</v>
+        <v>2778</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2427" t="n">
@@ -44127,87 +44127,87 @@
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2740</v>
+        <v>2781</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2428" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2429">
       <c r="A2429" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2710</v>
+        <v>2822</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2429" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2430">
       <c r="A2430" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2430" t="n">
-        <v>2711</v>
+        <v>2740</v>
       </c>
       <c r="C2430" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2430" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2431">
       <c r="A2431" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2431" t="n">
-        <v>2712</v>
+        <v>2710</v>
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2431" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2432">
       <c r="A2432" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2432" t="n">
-        <v>2717</v>
+        <v>2711</v>
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D2432" t="n">
-        <v>69</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2433">
@@ -44217,14 +44217,50 @@
         </is>
       </c>
       <c r="B2433" t="n">
+        <v>2712</v>
+      </c>
+      <c r="C2433" t="inlineStr">
+        <is>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
+        </is>
+      </c>
+      <c r="D2433" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2434">
+      <c r="A2434" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2434" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2434" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2434" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2435">
+      <c r="A2435" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2435" t="n">
         <v>2801</v>
       </c>
-      <c r="C2433" t="inlineStr">
+      <c r="C2435" t="inlineStr">
         <is>
           <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
-      <c r="D2433" t="n">
+      <c r="D2435" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:01:46
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -33312,7 +33312,7 @@
       </c>
       <c r="C1827" t="inlineStr">
         <is>
-          <t>PETROLINA-HB  (VALERIA COELHO )</t>
+          <t>PETROLINA-HB  (VAGO/VALERIA COELHO )</t>
         </is>
       </c>
       <c r="D1827" t="n">
@@ -37957,7 +37957,7 @@
       </c>
       <c r="C2085" t="inlineStr">
         <is>
-          <t>LITORAL SUL FARMA (ALANNE CRISTINA)</t>
+          <t>LITORAL SUL FARMA (VAGO/ALANNE CRISTINA)</t>
         </is>
       </c>
       <c r="D2085" t="n">

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:02:55
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2435"/>
+  <dimension ref="A1:D2438"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34698,7 +34698,7 @@
       </c>
       <c r="C1904" t="inlineStr">
         <is>
-          <t>ROSEANE SILVA FERREIRA - FARMA</t>
+          <t>VAGO ROSEANE SILVA FERREIRA - FARMA</t>
         </is>
       </c>
       <c r="D1904" t="n">
@@ -36211,7 +36211,7 @@
       </c>
       <c r="C1988" t="inlineStr">
         <is>
-          <t>GUILHERME MARTINS RAMOS- INATIVO</t>
+          <t>INATIVO- GUILHERME MARTINS RAMOS</t>
         </is>
       </c>
       <c r="D1988" t="n">
@@ -41679,11 +41679,11 @@
         </is>
       </c>
       <c r="B2292" t="n">
-        <v>2747</v>
+        <v>2843</v>
       </c>
       <c r="C2292" t="inlineStr">
         <is>
-          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
+          <t>VAGO FEIRA DE SANTANA II - FARMA</t>
         </is>
       </c>
       <c r="D2292" t="n">
@@ -41697,11 +41697,11 @@
         </is>
       </c>
       <c r="B2293" t="n">
-        <v>2748</v>
+        <v>2747</v>
       </c>
       <c r="C2293" t="inlineStr">
         <is>
-          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
+          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
         </is>
       </c>
       <c r="D2293" t="n">
@@ -41711,73 +41711,73 @@
     <row r="2294">
       <c r="A2294" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2294" t="n">
-        <v>2766</v>
+        <v>2748</v>
       </c>
       <c r="C2294" t="inlineStr">
         <is>
-          <t>SETOR VAGO PEDREIRAS</t>
+          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
         </is>
       </c>
       <c r="D2294" t="n">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2295">
       <c r="A2295" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2295" t="n">
-        <v>2767</v>
+        <v>2766</v>
       </c>
       <c r="C2295" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>SETOR VAGO PEDREIRAS</t>
         </is>
       </c>
       <c r="D2295" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2296">
       <c r="A2296" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2296" t="n">
-        <v>2688</v>
+        <v>2767</v>
       </c>
       <c r="C2296" t="inlineStr">
         <is>
-          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D2296" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2297">
       <c r="A2297" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2297" t="n">
-        <v>2694</v>
+        <v>2688</v>
       </c>
       <c r="C2297" t="inlineStr">
         <is>
-          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
+          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2297" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2298">
@@ -41787,15 +41787,15 @@
         </is>
       </c>
       <c r="B2298" t="n">
-        <v>2714</v>
+        <v>2694</v>
       </c>
       <c r="C2298" t="inlineStr">
         <is>
-          <t>PRISCILA DOS SANTOS LOPES - HB</t>
+          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2298" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2299">
@@ -41805,15 +41805,15 @@
         </is>
       </c>
       <c r="B2299" t="n">
-        <v>2722</v>
+        <v>2714</v>
       </c>
       <c r="C2299" t="inlineStr">
         <is>
-          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
+          <t>PRISCILA DOS SANTOS LOPES - HB</t>
         </is>
       </c>
       <c r="D2299" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2300">
@@ -41823,15 +41823,15 @@
         </is>
       </c>
       <c r="B2300" t="n">
-        <v>2723</v>
+        <v>2722</v>
       </c>
       <c r="C2300" t="inlineStr">
         <is>
-          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
+          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
         </is>
       </c>
       <c r="D2300" t="n">
-        <v>95</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2301">
@@ -41841,15 +41841,15 @@
         </is>
       </c>
       <c r="B2301" t="n">
-        <v>2803</v>
+        <v>2723</v>
       </c>
       <c r="C2301" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
+          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2301" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2302">
@@ -41859,11 +41859,11 @@
         </is>
       </c>
       <c r="B2302" t="n">
-        <v>2804</v>
+        <v>2803</v>
       </c>
       <c r="C2302" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA - HB</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
         </is>
       </c>
       <c r="D2302" t="n">
@@ -41873,19 +41873,19 @@
     <row r="2303">
       <c r="A2303" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2303" t="n">
-        <v>2830</v>
+        <v>2804</v>
       </c>
       <c r="C2303" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 1</t>
+          <t>PAULA CARLA CALDAS MOTA - HB</t>
         </is>
       </c>
       <c r="D2303" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2304">
@@ -41895,11 +41895,11 @@
         </is>
       </c>
       <c r="B2304" t="n">
-        <v>2831</v>
+        <v>2830</v>
       </c>
       <c r="C2304" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 2</t>
+          <t>SETOR VAGO BALSAS 1</t>
         </is>
       </c>
       <c r="D2304" t="n">
@@ -41909,55 +41909,55 @@
     <row r="2305">
       <c r="A2305" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2305" t="n">
-        <v>2647</v>
+        <v>2831</v>
       </c>
       <c r="C2305" t="inlineStr">
         <is>
-          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
+          <t>SETOR VAGO BALSAS 2</t>
         </is>
       </c>
       <c r="D2305" t="n">
-        <v>147</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2306">
       <c r="A2306" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2306" t="n">
-        <v>2661</v>
+        <v>2647</v>
       </c>
       <c r="C2306" t="inlineStr">
         <is>
-          <t>MARIA ISADORA DOS REIS REGO</t>
+          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
         </is>
       </c>
       <c r="D2306" t="n">
-        <v>76</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2307">
       <c r="A2307" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2307" t="n">
-        <v>2686</v>
+        <v>2661</v>
       </c>
       <c r="C2307" t="inlineStr">
         <is>
-          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
+          <t>MARIA ISADORA DOS REIS REGO</t>
         </is>
       </c>
       <c r="D2307" t="n">
-        <v>120</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2308">
@@ -41967,11 +41967,11 @@
         </is>
       </c>
       <c r="B2308" t="n">
-        <v>2687</v>
+        <v>2686</v>
       </c>
       <c r="C2308" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
+          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2308" t="n">
@@ -41981,109 +41981,109 @@
     <row r="2309">
       <c r="A2309" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2309" t="n">
-        <v>2681</v>
+        <v>2687</v>
       </c>
       <c r="C2309" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL PI</t>
+          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
         </is>
       </c>
       <c r="D2309" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2310">
       <c r="A2310" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2310" t="n">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="C2310" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL MA</t>
+          <t>RCA PRINCIPIA OL PI</t>
         </is>
       </c>
       <c r="D2310" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2311" t="n">
-        <v>2826</v>
+        <v>2682</v>
       </c>
       <c r="C2311" t="inlineStr">
         <is>
-          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
+          <t>RCA PRINCIPIA OL MA</t>
         </is>
       </c>
       <c r="D2311" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2312">
       <c r="A2312" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2312" t="n">
-        <v>2677</v>
+        <v>2826</v>
       </c>
       <c r="C2312" t="inlineStr">
         <is>
-          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
+          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
         </is>
       </c>
       <c r="D2312" t="n">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2313">
       <c r="A2313" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2313" t="n">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="C2313" t="inlineStr">
         <is>
-          <t>ADRIEL XERXES BARROS MARTINS</t>
+          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
         </is>
       </c>
       <c r="D2313" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2314">
       <c r="A2314" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2314" t="n">
-        <v>2735</v>
+        <v>2678</v>
       </c>
       <c r="C2314" t="inlineStr">
         <is>
-          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
+          <t>ADRIEL XERXES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D2314" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2315">
@@ -42093,15 +42093,15 @@
         </is>
       </c>
       <c r="B2315" t="n">
-        <v>2736</v>
+        <v>2735</v>
       </c>
       <c r="C2315" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
+          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2315" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2316">
@@ -42111,15 +42111,15 @@
         </is>
       </c>
       <c r="B2316" t="n">
-        <v>2737</v>
+        <v>2736</v>
       </c>
       <c r="C2316" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
+          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2316" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2317">
@@ -42129,15 +42129,15 @@
         </is>
       </c>
       <c r="B2317" t="n">
-        <v>2743</v>
+        <v>2737</v>
       </c>
       <c r="C2317" t="inlineStr">
         <is>
-          <t>VAGO SEABRA - FARMA</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
         </is>
       </c>
       <c r="D2317" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2318">
@@ -42147,11 +42147,11 @@
         </is>
       </c>
       <c r="B2318" t="n">
-        <v>2744</v>
+        <v>2743</v>
       </c>
       <c r="C2318" t="inlineStr">
         <is>
-          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
+          <t>VAGO SEABRA - FARMA</t>
         </is>
       </c>
       <c r="D2318" t="n">
@@ -42165,15 +42165,15 @@
         </is>
       </c>
       <c r="B2319" t="n">
-        <v>2745</v>
+        <v>2744</v>
       </c>
       <c r="C2319" t="inlineStr">
         <is>
-          <t>CIRLANE ARAUJO SOUZA - HB</t>
+          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
         </is>
       </c>
       <c r="D2319" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2320">
@@ -42183,105 +42183,105 @@
         </is>
       </c>
       <c r="B2320" t="n">
-        <v>2783</v>
+        <v>2745</v>
       </c>
       <c r="C2320" t="inlineStr">
         <is>
-          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
+          <t>CIRLANE ARAUJO SOUZA - HB</t>
         </is>
       </c>
       <c r="D2320" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2321">
       <c r="A2321" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2321" t="n">
-        <v>2768</v>
+        <v>2783</v>
       </c>
       <c r="C2321" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2321" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2322">
       <c r="A2322" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2322" t="n">
-        <v>2703</v>
+        <v>2768</v>
       </c>
       <c r="C2322" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2322" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2323">
       <c r="A2323" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2828</v>
+        <v>2703</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>LYERKA MARDANIA RODRIGUES MELO</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2323" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2324">
       <c r="A2324" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2750</v>
+        <v>2828</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>LYERKA MARDANIA RODRIGUES MELO</t>
         </is>
       </c>
       <c r="D2324" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2325">
       <c r="A2325" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2689</v>
+        <v>2750</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2325" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2326">
@@ -42291,69 +42291,69 @@
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2708</v>
+        <v>2689</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2326" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2327">
       <c r="A2327" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2709</v>
+        <v>2708</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2327" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2328">
       <c r="A2328" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2789</v>
+        <v>2709</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
         </is>
       </c>
       <c r="D2328" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2790</v>
+        <v>2789</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2329" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2330">
@@ -42363,11 +42363,11 @@
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2791</v>
+        <v>2790</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>DANIELY PEREIRA PINHEIRO</t>
+          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
         </is>
       </c>
       <c r="D2330" t="n">
@@ -42377,19 +42377,19 @@
     <row r="2331">
       <c r="A2331" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2805</v>
+        <v>2791</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>DANIELY PEREIRA PINHEIRO</t>
         </is>
       </c>
       <c r="D2331" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2332">
@@ -42399,11 +42399,11 @@
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2806</v>
+        <v>2805</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2332" t="n">
@@ -42417,11 +42417,11 @@
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2807</v>
+        <v>2806</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2333" t="n">
@@ -42435,11 +42435,11 @@
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2808</v>
+        <v>2807</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2334" t="n">
@@ -42449,109 +42449,109 @@
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2820</v>
+        <v>2808</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2335" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2336">
       <c r="A2336" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2765</v>
+        <v>2820</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2336" t="n">
-        <v>98</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2337">
       <c r="A2337" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2741</v>
+        <v>2765</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2337" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2338">
       <c r="A2338" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2758</v>
+        <v>2842</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D2338" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2339">
       <c r="A2339" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2659</v>
+        <v>2741</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2339" t="n">
-        <v>100</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2669</v>
+        <v>2758</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>135</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2341">
@@ -42561,141 +42561,141 @@
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2672</v>
+        <v>2659</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2341" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2342">
       <c r="A2342" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2673</v>
+        <v>2669</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2343">
       <c r="A2343" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2676</v>
+        <v>2672</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2343" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2344">
       <c r="A2344" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2344" t="n">
-        <v>2760</v>
+        <v>2673</v>
       </c>
       <c r="C2344" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2344" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2345">
       <c r="A2345" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2345" t="n">
-        <v>2823</v>
+        <v>2676</v>
       </c>
       <c r="C2345" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2345" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2346">
       <c r="A2346" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2346" t="n">
-        <v>2792</v>
+        <v>2760</v>
       </c>
       <c r="C2346" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2346" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2347">
       <c r="A2347" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2347" t="n">
-        <v>2793</v>
+        <v>2823</v>
       </c>
       <c r="C2347" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2347" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2348">
       <c r="A2348" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2802</v>
+        <v>2792</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2348" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2349">
@@ -42705,11 +42705,11 @@
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2656</v>
+        <v>2793</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2349" t="n">
@@ -42719,19 +42719,19 @@
     <row r="2350">
       <c r="A2350" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2657</v>
+        <v>2802</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2350" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2351">
@@ -42741,33 +42741,33 @@
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2658</v>
+        <v>2656</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2351" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2352">
       <c r="A2352" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2729</v>
+        <v>2657</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D2352" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2353">
@@ -42777,33 +42777,33 @@
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2759</v>
+        <v>2658</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2353" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2354">
       <c r="A2354" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2832</v>
+        <v>2729</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2354" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2355">
@@ -42813,11 +42813,11 @@
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2769</v>
+        <v>2759</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2355" t="n">
@@ -42827,73 +42827,73 @@
     <row r="2356">
       <c r="A2356" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2679</v>
+        <v>2832</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
         </is>
       </c>
       <c r="D2356" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2680</v>
+        <v>2769</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2357" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2358">
       <c r="A2358" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2815</v>
+        <v>2679</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2358" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2359">
       <c r="A2359" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2816</v>
+        <v>2680</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2359" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2360">
@@ -42903,159 +42903,159 @@
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2817</v>
+        <v>2815</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2361">
       <c r="A2361" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2701</v>
+        <v>2816</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2361" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2362">
       <c r="A2362" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2644</v>
+        <v>2817</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2362" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2363">
       <c r="A2363" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2645</v>
+        <v>2841</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
         </is>
       </c>
       <c r="D2363" t="n">
-        <v>108</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2364">
       <c r="A2364" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2754</v>
+        <v>2701</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2364" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2365">
       <c r="A2365" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2755</v>
+        <v>2644</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2365" t="n">
-        <v>80</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2665</v>
+        <v>2645</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2366" t="n">
-        <v>141</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2367">
       <c r="A2367" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2667</v>
+        <v>2754</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>114</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2368">
       <c r="A2368" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2727</v>
+        <v>2755</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2368" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2369">
@@ -43065,69 +43065,69 @@
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2728</v>
+        <v>2665</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2369" t="n">
-        <v>120</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2370">
       <c r="A2370" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2833</v>
+        <v>2667</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>ADEILZA PINTO DA SILVA - FARMA</t>
+          <t>GILBERTO MOREIRA MENESES (PLUS HIBRIDO)</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2814</v>
+        <v>2727</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2372">
       <c r="A2372" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2646</v>
+        <v>2728</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2372" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2373">
@@ -43137,11 +43137,11 @@
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2650</v>
+        <v>2833</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>ADEILZA PINTO DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2373" t="n">
@@ -43151,19 +43151,19 @@
     <row r="2374">
       <c r="A2374" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2652</v>
+        <v>2814</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>98</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2375">
@@ -43173,11 +43173,11 @@
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2653</v>
+        <v>2646</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2375" t="n">
@@ -43191,15 +43191,15 @@
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2654</v>
+        <v>2650</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2376" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2377">
@@ -43209,11 +43209,11 @@
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2655</v>
+        <v>2652</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2377" t="n">
@@ -43223,19 +43223,19 @@
     <row r="2378">
       <c r="A2378" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2821</v>
+        <v>2653</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2379">
@@ -43245,11 +43245,11 @@
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2683</v>
+        <v>2654</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2379" t="n">
@@ -43263,11 +43263,11 @@
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2684</v>
+        <v>2655</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2380" t="n">
@@ -43277,73 +43277,73 @@
     <row r="2381">
       <c r="A2381" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2749</v>
+        <v>2821</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>111</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2382">
       <c r="A2382" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2812</v>
+        <v>2683</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>145</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2383">
       <c r="A2383" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2715</v>
+        <v>2684</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2834</v>
+        <v>2749</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>GILVANA DA SILVA MONTELES</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2385">
@@ -43353,11 +43353,11 @@
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2651</v>
+        <v>2812</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2385" t="n">
@@ -43367,127 +43367,127 @@
     <row r="2386">
       <c r="A2386" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2819</v>
+        <v>2715</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2387">
       <c r="A2387" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2835</v>
+        <v>2834</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>ROGÉRIO LIRA DA GAMA</t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2699</v>
+        <v>2651</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2389">
       <c r="A2389" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2706</v>
+        <v>2819</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS BARREIRINHAS</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2707</v>
+        <v>2835</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>EVANESSA DA SILVA E SILVA</t>
+          <t>ROGÉRIO LIRA DA GAMA</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2693</v>
+        <v>2699</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>80</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2705</v>
+        <v>2706</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>SETOR VAGO PLUS BARREIRINHAS</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>146</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2393">
@@ -43497,15 +43497,15 @@
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2664</v>
+        <v>2707</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>EVANESSA DA SILVA E SILVA</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2394">
@@ -43515,51 +43515,51 @@
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2670</v>
+        <v>2693</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2730</v>
+        <v>2705</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>120</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2396">
       <c r="A2396" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2671</v>
+        <v>2664</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2397">
@@ -43569,33 +43569,33 @@
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2691</v>
+        <v>2670</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2692</v>
+        <v>2730</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2399">
@@ -43605,87 +43605,87 @@
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2724</v>
+        <v>2671</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2400">
       <c r="A2400" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2773</v>
+        <v>2691</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>VIVIANE LEAL DA SILVA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2401">
       <c r="A2401" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2825</v>
+        <v>2692</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2402">
       <c r="A2402" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2787</v>
+        <v>2724</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2403">
       <c r="A2403" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2839</v>
+        <v>2773</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>RCA TENA OL PI</t>
+          <t>VIVIANE LEAL DA SILVA</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>69</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2404">
@@ -43695,15 +43695,15 @@
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2840</v>
+        <v>2825</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>RCA TENA OL MA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2405">
@@ -43713,69 +43713,69 @@
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2648</v>
+        <v>2787</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2666</v>
+        <v>2839</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>RCA TENA OL PI</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2407">
       <c r="A2407" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2779</v>
+        <v>2840</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>RCA TENA OL MA</t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>105</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2780</v>
+        <v>2648</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>105</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2409">
@@ -43785,123 +43785,123 @@
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2786</v>
+        <v>2666</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2410">
       <c r="A2410" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2660</v>
+        <v>2779</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2410" t="n">
-        <v>38</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2411">
       <c r="A2411" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2716</v>
+        <v>2780</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2412">
       <c r="A2412" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2734</v>
+        <v>2786</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2413">
       <c r="A2413" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2742</v>
+        <v>2660</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2414">
       <c r="A2414" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2794</v>
+        <v>2716</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2415">
       <c r="A2415" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2795</v>
+        <v>2734</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2415" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2416">
@@ -43911,11 +43911,11 @@
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2796</v>
+        <v>2742</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2416" t="n">
@@ -43929,15 +43929,15 @@
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2797</v>
+        <v>2794</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2418">
@@ -43947,11 +43947,11 @@
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2798</v>
+        <v>2795</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
         </is>
       </c>
       <c r="D2418" t="n">
@@ -43961,145 +43961,145 @@
     <row r="2419">
       <c r="A2419" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2668</v>
+        <v>2796</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2419" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2420">
       <c r="A2420" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2690</v>
+        <v>2797</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2421">
       <c r="A2421" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2696</v>
+        <v>2798</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2422">
       <c r="A2422" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2697</v>
+        <v>2668</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>69</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2423">
       <c r="A2423" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2698</v>
+        <v>2690</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2424">
       <c r="A2424" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2775</v>
+        <v>2696</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2424" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2425">
       <c r="A2425" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2776</v>
+        <v>2697</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2425" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2426">
       <c r="A2426" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2777</v>
+        <v>2698</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2426" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2427">
@@ -44109,11 +44109,11 @@
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2778</v>
+        <v>2775</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2427" t="n">
@@ -44127,15 +44127,15 @@
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2781</v>
+        <v>2776</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2428" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2429">
@@ -44145,11 +44145,11 @@
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2822</v>
+        <v>2777</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2429" t="n">
@@ -44163,11 +44163,11 @@
         </is>
       </c>
       <c r="B2430" t="n">
-        <v>2740</v>
+        <v>2778</v>
       </c>
       <c r="C2430" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2430" t="n">
@@ -44177,37 +44177,37 @@
     <row r="2431">
       <c r="A2431" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2431" t="n">
-        <v>2710</v>
+        <v>2781</v>
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2431" t="n">
-        <v>69</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2432">
       <c r="A2432" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2432" t="n">
-        <v>2711</v>
+        <v>2822</v>
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2432" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2433">
@@ -44217,11 +44217,11 @@
         </is>
       </c>
       <c r="B2433" t="n">
-        <v>2712</v>
+        <v>2740</v>
       </c>
       <c r="C2433" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2433" t="n">
@@ -44235,11 +44235,11 @@
         </is>
       </c>
       <c r="B2434" t="n">
-        <v>2717</v>
+        <v>2710</v>
       </c>
       <c r="C2434" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2434" t="n">
@@ -44249,18 +44249,72 @@
     <row r="2435">
       <c r="A2435" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2435" t="n">
+        <v>2711</v>
+      </c>
+      <c r="C2435" t="inlineStr">
+        <is>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+        </is>
+      </c>
+      <c r="D2435" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2436">
+      <c r="A2436" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2436" t="n">
+        <v>2712</v>
+      </c>
+      <c r="C2436" t="inlineStr">
+        <is>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
+        </is>
+      </c>
+      <c r="D2436" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2437">
+      <c r="A2437" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2437" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2437" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2437" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2438">
+      <c r="A2438" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2438" t="n">
         <v>2801</v>
       </c>
-      <c r="C2435" t="inlineStr">
+      <c r="C2438" t="inlineStr">
         <is>
           <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
-      <c r="D2435" t="n">
+      <c r="D2438" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:01:43
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2438"/>
+  <dimension ref="A1:D2440"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43691,55 +43691,55 @@
     <row r="2404">
       <c r="A2404" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2825</v>
+        <v>2844</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>90</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2405">
       <c r="A2405" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2787</v>
+        <v>2845</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>120</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2839</v>
+        <v>2825</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>RCA TENA OL PI</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2407">
@@ -43749,69 +43749,69 @@
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2840</v>
+        <v>2787</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>RCA TENA OL MA</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2648</v>
+        <v>2839</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>RCA TENA OL PI</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2666</v>
+        <v>2840</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>RCA TENA OL MA</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>63</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2410">
       <c r="A2410" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2779</v>
+        <v>2648</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2410" t="n">
-        <v>105</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2411">
@@ -43821,15 +43821,15 @@
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2780</v>
+        <v>2666</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2412">
@@ -43839,51 +43839,51 @@
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2786</v>
+        <v>2779</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2413">
       <c r="A2413" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2660</v>
+        <v>2780</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>38</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2414">
       <c r="A2414" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2716</v>
+        <v>2786</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2415">
@@ -43893,51 +43893,51 @@
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2734</v>
+        <v>2660</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2415" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2416">
       <c r="A2416" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2742</v>
+        <v>2716</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2416" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2417">
       <c r="A2417" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2794</v>
+        <v>2734</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2418">
@@ -43947,11 +43947,11 @@
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2795</v>
+        <v>2742</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2418" t="n">
@@ -43965,15 +43965,15 @@
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2796</v>
+        <v>2794</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2419" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2420">
@@ -43983,11 +43983,11 @@
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2797</v>
+        <v>2795</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
         </is>
       </c>
       <c r="D2420" t="n">
@@ -44001,11 +44001,11 @@
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2798</v>
+        <v>2796</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2421" t="n">
@@ -44015,73 +44015,73 @@
     <row r="2422">
       <c r="A2422" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2668</v>
+        <v>2797</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2423">
       <c r="A2423" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2690</v>
+        <v>2798</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2424">
       <c r="A2424" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2696</v>
+        <v>2668</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2424" t="n">
-        <v>69</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2425">
       <c r="A2425" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2697</v>
+        <v>2690</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2425" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2426">
@@ -44091,11 +44091,11 @@
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2698</v>
+        <v>2696</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2426" t="n">
@@ -44105,37 +44105,37 @@
     <row r="2427">
       <c r="A2427" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2775</v>
+        <v>2697</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2427" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2428">
       <c r="A2428" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2776</v>
+        <v>2698</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2428" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2429">
@@ -44145,11 +44145,11 @@
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2777</v>
+        <v>2775</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2429" t="n">
@@ -44163,11 +44163,11 @@
         </is>
       </c>
       <c r="B2430" t="n">
-        <v>2778</v>
+        <v>2776</v>
       </c>
       <c r="C2430" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2430" t="n">
@@ -44181,15 +44181,15 @@
         </is>
       </c>
       <c r="B2431" t="n">
-        <v>2781</v>
+        <v>2777</v>
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2431" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2432">
@@ -44199,11 +44199,11 @@
         </is>
       </c>
       <c r="B2432" t="n">
-        <v>2822</v>
+        <v>2778</v>
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2432" t="n">
@@ -44217,87 +44217,87 @@
         </is>
       </c>
       <c r="B2433" t="n">
-        <v>2740</v>
+        <v>2781</v>
       </c>
       <c r="C2433" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2433" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2434">
       <c r="A2434" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2434" t="n">
-        <v>2710</v>
+        <v>2822</v>
       </c>
       <c r="C2434" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2434" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2435">
       <c r="A2435" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2435" t="n">
-        <v>2711</v>
+        <v>2740</v>
       </c>
       <c r="C2435" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2435" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2436">
       <c r="A2436" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2436" t="n">
-        <v>2712</v>
+        <v>2710</v>
       </c>
       <c r="C2436" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2436" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2437">
       <c r="A2437" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2437" t="n">
-        <v>2717</v>
+        <v>2711</v>
       </c>
       <c r="C2437" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D2437" t="n">
-        <v>69</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2438">
@@ -44307,14 +44307,50 @@
         </is>
       </c>
       <c r="B2438" t="n">
+        <v>2712</v>
+      </c>
+      <c r="C2438" t="inlineStr">
+        <is>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
+        </is>
+      </c>
+      <c r="D2438" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2439">
+      <c r="A2439" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2439" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2439" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2439" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2440">
+      <c r="A2440" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2440" t="n">
         <v>2801</v>
       </c>
-      <c r="C2438" t="inlineStr">
+      <c r="C2440" t="inlineStr">
         <is>
           <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
-      <c r="D2438" t="n">
+      <c r="D2440" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:01:12
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -4205,7 +4205,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>FELIPE FERNANDES FONTINELES - HIBRIDO</t>
+          <t>INATIVO - FELIPE FERNANDES FONTINELES</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -40081,7 +40081,7 @@
       </c>
       <c r="C2203" t="inlineStr">
         <is>
-          <t>ANTÔNIO WLAKCSON SERP CAVALCAN-ALIMENTAR</t>
+          <t>INATIVO- ANTÔNIO WLAKCSON SERP CAVALCAN</t>
         </is>
       </c>
       <c r="D2203" t="n">
@@ -44383,7 +44383,7 @@
       </c>
       <c r="C2442" t="inlineStr">
         <is>
-          <t>SETOR VAGO VIANA</t>
+          <t>SETOR VAGO VIANA FARMA</t>
         </is>
       </c>
       <c r="D2442" t="n">

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:01:23
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2442"/>
+  <dimension ref="A1:D2443"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41215,7 +41215,7 @@
       </c>
       <c r="C2266" t="inlineStr">
         <is>
-          <t>VALDECI NASCIMENTO DELGADO JUNIOR</t>
+          <t>SETOR CODÓ VAGO FARMA</t>
         </is>
       </c>
       <c r="D2266" t="n">
@@ -42683,15 +42683,15 @@
     <row r="2348">
       <c r="A2348" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2792</v>
+        <v>2848</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2348" t="n">
@@ -42701,19 +42701,19 @@
     <row r="2349">
       <c r="A2349" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2793</v>
+        <v>2792</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2349" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2350">
@@ -42723,15 +42723,15 @@
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2802</v>
+        <v>2793</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2350" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2351">
@@ -42741,47 +42741,47 @@
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2656</v>
+        <v>2802</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2351" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2352">
       <c r="A2352" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2657</v>
+        <v>2656</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA IMP 01 HNB</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2352" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2353">
       <c r="A2353" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>MARIA APARECIDA IMP 01 HNB</t>
         </is>
       </c>
       <c r="D2353" t="n">
@@ -42791,37 +42791,37 @@
     <row r="2354">
       <c r="A2354" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2729</v>
+        <v>2658</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2354" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2355">
       <c r="A2355" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2759</v>
+        <v>2729</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2355" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2356">
@@ -42831,15 +42831,15 @@
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2832</v>
+        <v>2759</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2356" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2357">
@@ -42849,33 +42849,33 @@
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2769</v>
+        <v>2832</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
         </is>
       </c>
       <c r="D2357" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2358">
       <c r="A2358" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2679</v>
+        <v>2769</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2358" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2359">
@@ -42885,11 +42885,11 @@
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2359" t="n">
@@ -42899,19 +42899,19 @@
     <row r="2360">
       <c r="A2360" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2815</v>
+        <v>2680</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2361">
@@ -42921,15 +42921,15 @@
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2816</v>
+        <v>2815</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2361" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2362">
@@ -42939,11 +42939,11 @@
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2817</v>
+        <v>2816</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2362" t="n">
@@ -42953,37 +42953,37 @@
     <row r="2363">
       <c r="A2363" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2841</v>
+        <v>2817</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2363" t="n">
-        <v>46</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2364">
       <c r="A2364" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2701</v>
+        <v>2841</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
         </is>
       </c>
       <c r="D2364" t="n">
-        <v>90</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2365">
@@ -42993,29 +42993,29 @@
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2644</v>
+        <v>2701</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2365" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2645</v>
+        <v>2644</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2366" t="n">
@@ -43029,15 +43029,15 @@
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2754</v>
+        <v>2645</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2368">
@@ -43047,33 +43047,33 @@
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2755</v>
+        <v>2754</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2368" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2369">
       <c r="A2369" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2665</v>
+        <v>2755</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2369" t="n">
-        <v>141</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2370">
@@ -43083,15 +43083,15 @@
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2667</v>
+        <v>2665</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>VAGO AÇAILÂNDIA HNB</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>114</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2371">
@@ -43101,15 +43101,15 @@
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2727</v>
+        <v>2667</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>VAGO AÇAILÂNDIA HNB</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2372">
@@ -43119,11 +43119,11 @@
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2728</v>
+        <v>2727</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2372" t="n">
@@ -43133,55 +43133,55 @@
     <row r="2373">
       <c r="A2373" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2833</v>
+        <v>2728</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>ADEILZA PINTO DA SILVA - FARMA</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2374">
       <c r="A2374" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2814</v>
+        <v>2833</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>ADEILZA PINTO DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>39</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2375">
       <c r="A2375" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2646</v>
+        <v>2814</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2375" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2376">
@@ -43191,11 +43191,11 @@
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2650</v>
+        <v>2646</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2376" t="n">
@@ -43209,15 +43209,15 @@
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2652</v>
+        <v>2650</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2377" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2378">
@@ -43227,15 +43227,15 @@
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2379">
@@ -43245,15 +43245,15 @@
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2654</v>
+        <v>2653</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2379" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2380">
@@ -43263,51 +43263,51 @@
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2655</v>
+        <v>2654</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2380" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2381">
       <c r="A2381" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2821</v>
+        <v>2655</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>69</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2382">
       <c r="A2382" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2683</v>
+        <v>2821</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2383">
@@ -43317,33 +43317,33 @@
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2749</v>
+        <v>2684</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2385">
@@ -43353,33 +43353,33 @@
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2812</v>
+        <v>2749</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2385" t="n">
-        <v>145</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2386">
       <c r="A2386" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2715</v>
+        <v>2812</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>90</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2387">
@@ -43389,105 +43389,105 @@
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2834</v>
+        <v>2715</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>GILVANA MONTELES U. SANTOS HNB</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2651</v>
+        <v>2834</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>GILVANA MONTELES U. SANTOS HNB</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>145</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2389">
       <c r="A2389" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2819</v>
+        <v>2651</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2835</v>
+        <v>2819</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>ROGÉRIO LIRA DA GAMA</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>116</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2699</v>
+        <v>2835</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>ROGÉRIO LIRA DA GAMA</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>95</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2706</v>
+        <v>2699</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>VAGO BARREIRINHAS HNB</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2393">
@@ -43497,11 +43497,11 @@
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2707</v>
+        <v>2706</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>VAGO BACABAL HNB</t>
+          <t>VAGO BARREIRINHAS HNB</t>
         </is>
       </c>
       <c r="D2393" t="n">
@@ -43515,15 +43515,15 @@
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2846</v>
+        <v>2707</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>VAGO BACABAL HNB</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2395">
@@ -43533,11 +43533,11 @@
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2847</v>
+        <v>2846</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>WERBERTTY</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D2395" t="n">
@@ -43547,127 +43547,127 @@
     <row r="2396">
       <c r="A2396" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2693</v>
+        <v>2847</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>WERBERTTY</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2397">
       <c r="A2397" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2705</v>
+        <v>2693</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>146</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2664</v>
+        <v>2705</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>90</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2670</v>
+        <v>2664</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2400">
       <c r="A2400" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2730</v>
+        <v>2670</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2401">
       <c r="A2401" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2671</v>
+        <v>2730</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2402">
       <c r="A2402" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2691</v>
+        <v>2671</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2403">
@@ -43677,11 +43677,11 @@
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2403" t="n">
@@ -43691,55 +43691,55 @@
     <row r="2404">
       <c r="A2404" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2724</v>
+        <v>2692</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2405">
       <c r="A2405" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2773</v>
+        <v>2724</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>TIMON 01 HNB</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2844</v>
+        <v>2773</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
+          <t>TIMON 01 HNB</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>132</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2407">
@@ -43749,11 +43749,11 @@
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2845</v>
+        <v>2844</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
+          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
         </is>
       </c>
       <c r="D2407" t="n">
@@ -43763,19 +43763,19 @@
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2825</v>
+        <v>2845</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>90</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2409">
@@ -43785,51 +43785,51 @@
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2787</v>
+        <v>2825</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2410">
       <c r="A2410" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2839</v>
+        <v>2787</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>RCA TENA OL PI</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2410" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2411">
       <c r="A2411" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2840</v>
+        <v>2839</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>RCA TENA OL MA</t>
+          <t>RCA TENA OL PI</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2412">
@@ -43839,33 +43839,33 @@
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2648</v>
+        <v>2840</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>RCA TENA OL MA</t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2413">
       <c r="A2413" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2666</v>
+        <v>2648</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2414">
@@ -43875,15 +43875,15 @@
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2779</v>
+        <v>2666</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2415">
@@ -43893,11 +43893,11 @@
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2780</v>
+        <v>2779</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2415" t="n">
@@ -43911,33 +43911,33 @@
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2786</v>
+        <v>2780</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2416" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2417">
       <c r="A2417" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2660</v>
+        <v>2786</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2418">
@@ -43947,15 +43947,15 @@
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2716</v>
+        <v>2660</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2418" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2419">
@@ -43965,11 +43965,11 @@
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2734</v>
+        <v>2716</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2419" t="n">
@@ -43979,19 +43979,19 @@
     <row r="2420">
       <c r="A2420" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2742</v>
+        <v>2734</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2421">
@@ -44001,15 +44001,15 @@
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2794</v>
+        <v>2742</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2422">
@@ -44019,15 +44019,15 @@
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2795</v>
+        <v>2794</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2423">
@@ -44037,11 +44037,11 @@
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2796</v>
+        <v>2795</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
         </is>
       </c>
       <c r="D2423" t="n">
@@ -44055,11 +44055,11 @@
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2797</v>
+        <v>2796</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2424" t="n">
@@ -44073,11 +44073,11 @@
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2798</v>
+        <v>2797</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2425" t="n">
@@ -44087,55 +44087,55 @@
     <row r="2426">
       <c r="A2426" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2668</v>
+        <v>2798</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2426" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2427">
       <c r="A2427" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2690</v>
+        <v>2668</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2427" t="n">
-        <v>38</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2428">
       <c r="A2428" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2696</v>
+        <v>2690</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2428" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2429">
@@ -44145,11 +44145,11 @@
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2429" t="n">
@@ -44163,11 +44163,11 @@
         </is>
       </c>
       <c r="B2430" t="n">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="C2430" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2430" t="n">
@@ -44177,19 +44177,19 @@
     <row r="2431">
       <c r="A2431" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2431" t="n">
-        <v>2775</v>
+        <v>2698</v>
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2431" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2432">
@@ -44199,11 +44199,11 @@
         </is>
       </c>
       <c r="B2432" t="n">
-        <v>2776</v>
+        <v>2775</v>
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2432" t="n">
@@ -44217,11 +44217,11 @@
         </is>
       </c>
       <c r="B2433" t="n">
-        <v>2777</v>
+        <v>2776</v>
       </c>
       <c r="C2433" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2433" t="n">
@@ -44235,11 +44235,11 @@
         </is>
       </c>
       <c r="B2434" t="n">
-        <v>2778</v>
+        <v>2777</v>
       </c>
       <c r="C2434" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2434" t="n">
@@ -44253,15 +44253,15 @@
         </is>
       </c>
       <c r="B2435" t="n">
-        <v>2781</v>
+        <v>2778</v>
       </c>
       <c r="C2435" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2435" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2436">
@@ -44271,15 +44271,15 @@
         </is>
       </c>
       <c r="B2436" t="n">
-        <v>2822</v>
+        <v>2781</v>
       </c>
       <c r="C2436" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2436" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2437">
@@ -44289,11 +44289,11 @@
         </is>
       </c>
       <c r="B2437" t="n">
-        <v>2740</v>
+        <v>2822</v>
       </c>
       <c r="C2437" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2437" t="n">
@@ -44303,90 +44303,108 @@
     <row r="2438">
       <c r="A2438" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2438" t="n">
-        <v>2710</v>
+        <v>2740</v>
       </c>
       <c r="C2438" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2438" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2439">
       <c r="A2439" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2439" t="n">
-        <v>2711</v>
+        <v>2710</v>
       </c>
       <c r="C2439" t="inlineStr">
         <is>
-          <t>CARLOS CHAPADINHA</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2439" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2440">
       <c r="A2440" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2440" t="n">
-        <v>2712</v>
+        <v>2711</v>
       </c>
       <c r="C2440" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>CARLOS CHAPADINHA</t>
         </is>
       </c>
       <c r="D2440" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2441">
       <c r="A2441" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2441" t="n">
-        <v>2717</v>
+        <v>2712</v>
       </c>
       <c r="C2441" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
         </is>
       </c>
       <c r="D2441" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2442">
       <c r="A2442" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2442" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2442" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2442" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2443">
+      <c r="A2443" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2443" t="n">
         <v>2801</v>
       </c>
-      <c r="C2442" t="inlineStr">
+      <c r="C2443" t="inlineStr">
         <is>
           <t>SETOR VAGO VIANA FARMA</t>
         </is>
       </c>
-      <c r="D2442" t="n">
+      <c r="D2443" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 17:35:07
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2443"/>
+  <dimension ref="A1:D2444"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41575,7 +41575,7 @@
       </c>
       <c r="C2286" t="inlineStr">
         <is>
-          <t>JOELTON MUNIZ DE SOUZA - HB</t>
+          <t>VAGO JOELTON MUNIZ DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2286" t="n">
@@ -43457,55 +43457,55 @@
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2835</v>
+        <v>2849</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>ROGÉRIO LIRA DA GAMA</t>
+          <t>MULTI PE (PEDRO HENRIQUE VIERA)</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>116</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2699</v>
+        <v>2835</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>ROGÉRIO LIRA DA GAMA</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>95</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2706</v>
+        <v>2699</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>VAGO BARREIRINHAS HNB</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2394">
@@ -43515,11 +43515,11 @@
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2707</v>
+        <v>2706</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>VAGO BACABAL HNB</t>
+          <t>VAGO BARREIRINHAS HNB</t>
         </is>
       </c>
       <c r="D2394" t="n">
@@ -43533,15 +43533,15 @@
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2846</v>
+        <v>2707</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>VAGO BACABAL HNB</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2396">
@@ -43551,11 +43551,11 @@
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2847</v>
+        <v>2846</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>WERBERTTY</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D2396" t="n">
@@ -43565,127 +43565,127 @@
     <row r="2397">
       <c r="A2397" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2693</v>
+        <v>2847</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>WERBERTTY</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2705</v>
+        <v>2693</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>146</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2664</v>
+        <v>2705</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>90</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2400">
       <c r="A2400" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2670</v>
+        <v>2664</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2401">
       <c r="A2401" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2730</v>
+        <v>2670</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2402">
       <c r="A2402" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2671</v>
+        <v>2730</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2403">
       <c r="A2403" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2691</v>
+        <v>2671</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2404">
@@ -43695,11 +43695,11 @@
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2404" t="n">
@@ -43709,55 +43709,55 @@
     <row r="2405">
       <c r="A2405" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2724</v>
+        <v>2692</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2773</v>
+        <v>2724</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>TIMON 01 HNB</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2407">
       <c r="A2407" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2844</v>
+        <v>2773</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
+          <t>TIMON 01 HNB</t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>132</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2408">
@@ -43767,11 +43767,11 @@
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2845</v>
+        <v>2844</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
+          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
         </is>
       </c>
       <c r="D2408" t="n">
@@ -43781,19 +43781,19 @@
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2825</v>
+        <v>2845</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>90</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2410">
@@ -43803,51 +43803,51 @@
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2787</v>
+        <v>2825</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2410" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2411">
       <c r="A2411" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2839</v>
+        <v>2787</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>RCA TENA OL PI</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2412">
       <c r="A2412" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2840</v>
+        <v>2839</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>RCA TENA OL MA</t>
+          <t>RCA TENA OL PI</t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2413">
@@ -43857,33 +43857,33 @@
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2648</v>
+        <v>2840</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>RCA TENA OL MA</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2414">
       <c r="A2414" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2666</v>
+        <v>2648</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2415">
@@ -43893,15 +43893,15 @@
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2779</v>
+        <v>2666</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2415" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2416">
@@ -43911,11 +43911,11 @@
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2780</v>
+        <v>2779</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2416" t="n">
@@ -43929,33 +43929,33 @@
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2786</v>
+        <v>2780</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2418">
       <c r="A2418" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2660</v>
+        <v>2786</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2418" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2419">
@@ -43965,15 +43965,15 @@
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2716</v>
+        <v>2660</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2419" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2420">
@@ -43983,11 +43983,11 @@
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2734</v>
+        <v>2716</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2420" t="n">
@@ -43997,19 +43997,19 @@
     <row r="2421">
       <c r="A2421" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2742</v>
+        <v>2734</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2422">
@@ -44019,15 +44019,15 @@
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2794</v>
+        <v>2742</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2423">
@@ -44037,15 +44037,15 @@
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2795</v>
+        <v>2794</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2424">
@@ -44055,11 +44055,11 @@
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2796</v>
+        <v>2795</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
         </is>
       </c>
       <c r="D2424" t="n">
@@ -44073,11 +44073,11 @@
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2797</v>
+        <v>2796</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2425" t="n">
@@ -44091,11 +44091,11 @@
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2798</v>
+        <v>2797</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2426" t="n">
@@ -44105,55 +44105,55 @@
     <row r="2427">
       <c r="A2427" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2668</v>
+        <v>2798</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2427" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2428">
       <c r="A2428" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2690</v>
+        <v>2668</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2428" t="n">
-        <v>38</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2429">
       <c r="A2429" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2696</v>
+        <v>2690</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2429" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2430">
@@ -44163,11 +44163,11 @@
         </is>
       </c>
       <c r="B2430" t="n">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="C2430" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2430" t="n">
@@ -44181,11 +44181,11 @@
         </is>
       </c>
       <c r="B2431" t="n">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2431" t="n">
@@ -44195,19 +44195,19 @@
     <row r="2432">
       <c r="A2432" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2432" t="n">
-        <v>2775</v>
+        <v>2698</v>
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2432" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2433">
@@ -44217,11 +44217,11 @@
         </is>
       </c>
       <c r="B2433" t="n">
-        <v>2776</v>
+        <v>2775</v>
       </c>
       <c r="C2433" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2433" t="n">
@@ -44235,11 +44235,11 @@
         </is>
       </c>
       <c r="B2434" t="n">
-        <v>2777</v>
+        <v>2776</v>
       </c>
       <c r="C2434" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2434" t="n">
@@ -44253,11 +44253,11 @@
         </is>
       </c>
       <c r="B2435" t="n">
-        <v>2778</v>
+        <v>2777</v>
       </c>
       <c r="C2435" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2435" t="n">
@@ -44271,15 +44271,15 @@
         </is>
       </c>
       <c r="B2436" t="n">
-        <v>2781</v>
+        <v>2778</v>
       </c>
       <c r="C2436" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2436" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2437">
@@ -44289,15 +44289,15 @@
         </is>
       </c>
       <c r="B2437" t="n">
-        <v>2822</v>
+        <v>2781</v>
       </c>
       <c r="C2437" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2437" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2438">
@@ -44307,11 +44307,11 @@
         </is>
       </c>
       <c r="B2438" t="n">
-        <v>2740</v>
+        <v>2822</v>
       </c>
       <c r="C2438" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2438" t="n">
@@ -44321,90 +44321,108 @@
     <row r="2439">
       <c r="A2439" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2439" t="n">
-        <v>2710</v>
+        <v>2740</v>
       </c>
       <c r="C2439" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2439" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2440">
       <c r="A2440" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2440" t="n">
-        <v>2711</v>
+        <v>2710</v>
       </c>
       <c r="C2440" t="inlineStr">
         <is>
-          <t>CARLOS CHAPADINHA</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2440" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2441">
       <c r="A2441" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2441" t="n">
-        <v>2712</v>
+        <v>2711</v>
       </c>
       <c r="C2441" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>CARLOS CHAPADINHA</t>
         </is>
       </c>
       <c r="D2441" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2442">
       <c r="A2442" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2442" t="n">
-        <v>2717</v>
+        <v>2712</v>
       </c>
       <c r="C2442" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
         </is>
       </c>
       <c r="D2442" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2443">
       <c r="A2443" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2443" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2443" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2443" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2444">
+      <c r="A2444" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2444" t="n">
         <v>2801</v>
       </c>
-      <c r="C2443" t="inlineStr">
+      <c r="C2444" t="inlineStr">
         <is>
           <t>SETOR VAGO VIANA FARMA</t>
         </is>
       </c>
-      <c r="D2443" t="n">
+      <c r="D2444" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:00:36
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2444"/>
+  <dimension ref="A1:D2446"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37849,7 +37849,7 @@
       </c>
       <c r="C2079" t="inlineStr">
         <is>
-          <t>VAGO COLINAS</t>
+          <t>VAGO COLINAS HNB</t>
         </is>
       </c>
       <c r="D2079" t="n">
@@ -39667,7 +39667,7 @@
       </c>
       <c r="C2180" t="inlineStr">
         <is>
-          <t>VAGO BALSAS 01</t>
+          <t>VAGO BALSAS 01 HNB</t>
         </is>
       </c>
       <c r="D2180" t="n">
@@ -40801,7 +40801,7 @@
       </c>
       <c r="C2243" t="inlineStr">
         <is>
-          <t>GRAVATA- HB  (VAGO/FABIO INACIO)</t>
+          <t>GRAVATA- HB  (MIGUEL VELOSO)</t>
         </is>
       </c>
       <c r="D2243" t="n">
@@ -40891,7 +40891,7 @@
       </c>
       <c r="C2248" t="inlineStr">
         <is>
-          <t>VAGO CARUTAPERA</t>
+          <t>VAGO CARUTAPERA HNB</t>
         </is>
       </c>
       <c r="D2248" t="n">
@@ -41333,19 +41333,19 @@
     <row r="2273">
       <c r="A2273" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2273" t="n">
-        <v>2799</v>
+        <v>2850</v>
       </c>
       <c r="C2273" t="inlineStr">
         <is>
-          <t>VOLFRAMIO DALFREDO ALMEIDA</t>
+          <t>FERNANDO DE QUEIROZ COSTA - FARMA</t>
         </is>
       </c>
       <c r="D2273" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2274">
@@ -41355,33 +41355,33 @@
         </is>
       </c>
       <c r="B2274" t="n">
-        <v>2719</v>
+        <v>2799</v>
       </c>
       <c r="C2274" t="inlineStr">
         <is>
-          <t>SETOR SÃO RDO NONATO VAGO  (DEDICADA)</t>
+          <t>VOLFRAMIO DALFREDO ALMEIDA</t>
         </is>
       </c>
       <c r="D2274" t="n">
-        <v>39</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2275">
       <c r="A2275" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2275" t="n">
-        <v>2731</v>
+        <v>2719</v>
       </c>
       <c r="C2275" t="inlineStr">
         <is>
-          <t>VAGO ANDERSON A. S. - FARMA (CAMAÇARI)</t>
+          <t>SETOR SÃO RDO NONATO VAGO  (DEDICADA)</t>
         </is>
       </c>
       <c r="D2275" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2276">
@@ -41391,15 +41391,15 @@
         </is>
       </c>
       <c r="B2276" t="n">
-        <v>2732</v>
+        <v>2731</v>
       </c>
       <c r="C2276" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN DE JESUS - HB</t>
+          <t>VAGO ANDERSON A. S. - FARMA (CAMAÇARI)</t>
         </is>
       </c>
       <c r="D2276" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2277">
@@ -41409,51 +41409,51 @@
         </is>
       </c>
       <c r="B2277" t="n">
-        <v>2733</v>
+        <v>2732</v>
       </c>
       <c r="C2277" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAGO CENTRO CAROLINE LEMOS - FARMA </t>
+          <t>VAGO BRENO ALLAN DE JESUS - HB</t>
         </is>
       </c>
       <c r="D2277" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2278">
       <c r="A2278" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2278" t="n">
-        <v>2752</v>
+        <v>2733</v>
       </c>
       <c r="C2278" t="inlineStr">
         <is>
-          <t>SETOR BAIXADA PLUS (ELILTON ROMEU)</t>
+          <t xml:space="preserve">VAGO CENTRO CAROLINE LEMOS - FARMA </t>
         </is>
       </c>
       <c r="D2278" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2279">
       <c r="A2279" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2279" t="n">
-        <v>2662</v>
+        <v>2752</v>
       </c>
       <c r="C2279" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
+          <t>SETOR BAIXADA PLUS (ELILTON ROMEU)</t>
         </is>
       </c>
       <c r="D2279" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2280">
@@ -41463,15 +41463,15 @@
         </is>
       </c>
       <c r="B2280" t="n">
-        <v>2663</v>
+        <v>2662</v>
       </c>
       <c r="C2280" t="inlineStr">
         <is>
-          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
         </is>
       </c>
       <c r="D2280" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2281">
@@ -41481,15 +41481,15 @@
         </is>
       </c>
       <c r="B2281" t="n">
-        <v>2685</v>
+        <v>2663</v>
       </c>
       <c r="C2281" t="inlineStr">
         <is>
-          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
+          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
         </is>
       </c>
       <c r="D2281" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2282">
@@ -41499,15 +41499,15 @@
         </is>
       </c>
       <c r="B2282" t="n">
-        <v>2718</v>
+        <v>2685</v>
       </c>
       <c r="C2282" t="inlineStr">
         <is>
-          <t>KALILLA FERREIRA COSTA - FARMA</t>
+          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2282" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2283">
@@ -41517,15 +41517,15 @@
         </is>
       </c>
       <c r="B2283" t="n">
-        <v>2674</v>
+        <v>2718</v>
       </c>
       <c r="C2283" t="inlineStr">
         <is>
-          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
+          <t>KALILLA FERREIRA COSTA - FARMA</t>
         </is>
       </c>
       <c r="D2283" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2284">
@@ -41535,15 +41535,15 @@
         </is>
       </c>
       <c r="B2284" t="n">
-        <v>2753</v>
+        <v>2674</v>
       </c>
       <c r="C2284" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA - HB</t>
+          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
         </is>
       </c>
       <c r="D2284" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2285">
@@ -41553,15 +41553,15 @@
         </is>
       </c>
       <c r="B2285" t="n">
-        <v>2772</v>
+        <v>2753</v>
       </c>
       <c r="C2285" t="inlineStr">
         <is>
-          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA - HB</t>
         </is>
       </c>
       <c r="D2285" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2286">
@@ -41571,51 +41571,51 @@
         </is>
       </c>
       <c r="B2286" t="n">
-        <v>2827</v>
+        <v>2772</v>
       </c>
       <c r="C2286" t="inlineStr">
         <is>
-          <t>VAGO JOELTON MUNIZ DE SOUZA - HB</t>
+          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2286" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2287">
       <c r="A2287" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2287" t="n">
-        <v>2756</v>
+        <v>2827</v>
       </c>
       <c r="C2287" t="inlineStr">
         <is>
-          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
+          <t>VAGO JOELTON MUNIZ DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2287" t="n">
-        <v>39</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2288">
       <c r="A2288" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2288" t="n">
-        <v>2813</v>
+        <v>2756</v>
       </c>
       <c r="C2288" t="inlineStr">
         <is>
-          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
+          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
         </is>
       </c>
       <c r="D2288" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2289">
@@ -41625,15 +41625,15 @@
         </is>
       </c>
       <c r="B2289" t="n">
-        <v>2738</v>
+        <v>2813</v>
       </c>
       <c r="C2289" t="inlineStr">
         <is>
-          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
+          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
         </is>
       </c>
       <c r="D2289" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2290">
@@ -41643,11 +41643,11 @@
         </is>
       </c>
       <c r="B2290" t="n">
-        <v>2739</v>
+        <v>2738</v>
       </c>
       <c r="C2290" t="inlineStr">
         <is>
-          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
+          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2290" t="n">
@@ -41661,33 +41661,33 @@
         </is>
       </c>
       <c r="B2291" t="n">
-        <v>2824</v>
+        <v>2739</v>
       </c>
       <c r="C2291" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2291" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2292">
       <c r="A2292" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2292" t="n">
-        <v>2843</v>
+        <v>2824</v>
       </c>
       <c r="C2292" t="inlineStr">
         <is>
-          <t>VAGO FEIRA DE SANTANA II - FARMA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D2292" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2293">
@@ -41697,11 +41697,11 @@
         </is>
       </c>
       <c r="B2293" t="n">
-        <v>2747</v>
+        <v>2843</v>
       </c>
       <c r="C2293" t="inlineStr">
         <is>
-          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
+          <t>VAGO FEIRA DE SANTANA II - FARMA</t>
         </is>
       </c>
       <c r="D2293" t="n">
@@ -41715,11 +41715,11 @@
         </is>
       </c>
       <c r="B2294" t="n">
-        <v>2748</v>
+        <v>2747</v>
       </c>
       <c r="C2294" t="inlineStr">
         <is>
-          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
+          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
         </is>
       </c>
       <c r="D2294" t="n">
@@ -41729,73 +41729,73 @@
     <row r="2295">
       <c r="A2295" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2295" t="n">
-        <v>2766</v>
+        <v>2748</v>
       </c>
       <c r="C2295" t="inlineStr">
         <is>
-          <t>SETOR VAGO PEDREIRAS</t>
+          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
         </is>
       </c>
       <c r="D2295" t="n">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2296">
       <c r="A2296" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2296" t="n">
-        <v>2767</v>
+        <v>2766</v>
       </c>
       <c r="C2296" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>SETOR VAGO PEDREIRAS</t>
         </is>
       </c>
       <c r="D2296" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2297">
       <c r="A2297" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2297" t="n">
-        <v>2688</v>
+        <v>2767</v>
       </c>
       <c r="C2297" t="inlineStr">
         <is>
-          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D2297" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2298">
       <c r="A2298" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2298" t="n">
-        <v>2694</v>
+        <v>2688</v>
       </c>
       <c r="C2298" t="inlineStr">
         <is>
-          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
+          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2298" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2299">
@@ -41805,15 +41805,15 @@
         </is>
       </c>
       <c r="B2299" t="n">
-        <v>2714</v>
+        <v>2694</v>
       </c>
       <c r="C2299" t="inlineStr">
         <is>
-          <t>PRISCILA DOS SANTOS LOPES - HB</t>
+          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2299" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2300">
@@ -41823,15 +41823,15 @@
         </is>
       </c>
       <c r="B2300" t="n">
-        <v>2722</v>
+        <v>2714</v>
       </c>
       <c r="C2300" t="inlineStr">
         <is>
-          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
+          <t>PRISCILA DOS SANTOS LOPES - HB</t>
         </is>
       </c>
       <c r="D2300" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2301">
@@ -41841,15 +41841,15 @@
         </is>
       </c>
       <c r="B2301" t="n">
-        <v>2723</v>
+        <v>2722</v>
       </c>
       <c r="C2301" t="inlineStr">
         <is>
-          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
+          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
         </is>
       </c>
       <c r="D2301" t="n">
-        <v>95</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2302">
@@ -41859,15 +41859,15 @@
         </is>
       </c>
       <c r="B2302" t="n">
-        <v>2803</v>
+        <v>2723</v>
       </c>
       <c r="C2302" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
+          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2302" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2303">
@@ -41877,11 +41877,11 @@
         </is>
       </c>
       <c r="B2303" t="n">
-        <v>2804</v>
+        <v>2803</v>
       </c>
       <c r="C2303" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA - HB</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
         </is>
       </c>
       <c r="D2303" t="n">
@@ -41891,19 +41891,19 @@
     <row r="2304">
       <c r="A2304" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2304" t="n">
-        <v>2830</v>
+        <v>2804</v>
       </c>
       <c r="C2304" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 1</t>
+          <t>PAULA CARLA CALDAS MOTA - HB</t>
         </is>
       </c>
       <c r="D2304" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2305">
@@ -41913,11 +41913,11 @@
         </is>
       </c>
       <c r="B2305" t="n">
-        <v>2831</v>
+        <v>2830</v>
       </c>
       <c r="C2305" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 2</t>
+          <t>SETOR VAGO BALSAS 1</t>
         </is>
       </c>
       <c r="D2305" t="n">
@@ -41927,55 +41927,55 @@
     <row r="2306">
       <c r="A2306" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2306" t="n">
-        <v>2647</v>
+        <v>2831</v>
       </c>
       <c r="C2306" t="inlineStr">
         <is>
-          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
+          <t>SETOR VAGO BALSAS 2</t>
         </is>
       </c>
       <c r="D2306" t="n">
-        <v>147</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2307">
       <c r="A2307" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2307" t="n">
-        <v>2661</v>
+        <v>2647</v>
       </c>
       <c r="C2307" t="inlineStr">
         <is>
-          <t>MARIA ISADORA DOS REIS REGO</t>
+          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
         </is>
       </c>
       <c r="D2307" t="n">
-        <v>76</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2308">
       <c r="A2308" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2308" t="n">
-        <v>2686</v>
+        <v>2661</v>
       </c>
       <c r="C2308" t="inlineStr">
         <is>
-          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
+          <t>MARIA ISADORA DOS REIS REGO</t>
         </is>
       </c>
       <c r="D2308" t="n">
-        <v>120</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2309">
@@ -41985,11 +41985,11 @@
         </is>
       </c>
       <c r="B2309" t="n">
-        <v>2687</v>
+        <v>2686</v>
       </c>
       <c r="C2309" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
+          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2309" t="n">
@@ -41999,109 +41999,109 @@
     <row r="2310">
       <c r="A2310" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2310" t="n">
-        <v>2681</v>
+        <v>2687</v>
       </c>
       <c r="C2310" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL PI</t>
+          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
         </is>
       </c>
       <c r="D2310" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2311" t="n">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="C2311" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL MA</t>
+          <t>RCA PRINCIPIA OL PI</t>
         </is>
       </c>
       <c r="D2311" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2312">
       <c r="A2312" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2312" t="n">
-        <v>2826</v>
+        <v>2682</v>
       </c>
       <c r="C2312" t="inlineStr">
         <is>
-          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
+          <t>RCA PRINCIPIA OL MA</t>
         </is>
       </c>
       <c r="D2312" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2313">
       <c r="A2313" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2313" t="n">
-        <v>2677</v>
+        <v>2826</v>
       </c>
       <c r="C2313" t="inlineStr">
         <is>
-          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
+          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
         </is>
       </c>
       <c r="D2313" t="n">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2314">
       <c r="A2314" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2314" t="n">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="C2314" t="inlineStr">
         <is>
-          <t>ADRIEL XERXES BARROS MARTINS</t>
+          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
         </is>
       </c>
       <c r="D2314" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2315">
       <c r="A2315" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2315" t="n">
-        <v>2735</v>
+        <v>2678</v>
       </c>
       <c r="C2315" t="inlineStr">
         <is>
-          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
+          <t>ADRIEL XERXES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D2315" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2316">
@@ -42111,15 +42111,15 @@
         </is>
       </c>
       <c r="B2316" t="n">
-        <v>2736</v>
+        <v>2735</v>
       </c>
       <c r="C2316" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
+          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2316" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2317">
@@ -42129,15 +42129,15 @@
         </is>
       </c>
       <c r="B2317" t="n">
-        <v>2737</v>
+        <v>2736</v>
       </c>
       <c r="C2317" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
+          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2317" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2318">
@@ -42147,15 +42147,15 @@
         </is>
       </c>
       <c r="B2318" t="n">
-        <v>2743</v>
+        <v>2737</v>
       </c>
       <c r="C2318" t="inlineStr">
         <is>
-          <t>VAGO SEABRA - FARMA</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
         </is>
       </c>
       <c r="D2318" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2319">
@@ -42165,11 +42165,11 @@
         </is>
       </c>
       <c r="B2319" t="n">
-        <v>2744</v>
+        <v>2743</v>
       </c>
       <c r="C2319" t="inlineStr">
         <is>
-          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
+          <t>VAGO SEABRA - FARMA</t>
         </is>
       </c>
       <c r="D2319" t="n">
@@ -42183,15 +42183,15 @@
         </is>
       </c>
       <c r="B2320" t="n">
-        <v>2745</v>
+        <v>2744</v>
       </c>
       <c r="C2320" t="inlineStr">
         <is>
-          <t>CIRLANE ARAUJO SOUZA - HB</t>
+          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
         </is>
       </c>
       <c r="D2320" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2321">
@@ -42201,105 +42201,105 @@
         </is>
       </c>
       <c r="B2321" t="n">
-        <v>2783</v>
+        <v>2745</v>
       </c>
       <c r="C2321" t="inlineStr">
         <is>
-          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
+          <t>CIRLANE ARAUJO SOUZA - HB</t>
         </is>
       </c>
       <c r="D2321" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2322">
       <c r="A2322" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2322" t="n">
-        <v>2768</v>
+        <v>2783</v>
       </c>
       <c r="C2322" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2322" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2323">
       <c r="A2323" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2703</v>
+        <v>2768</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2323" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2324">
       <c r="A2324" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2828</v>
+        <v>2703</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>LYERKA MARDANIA RODRIGUES MELO</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2324" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2325">
       <c r="A2325" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2750</v>
+        <v>2828</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>LYERKA MARDANIA RODRIGUES MELO</t>
         </is>
       </c>
       <c r="D2325" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2326">
       <c r="A2326" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2689</v>
+        <v>2750</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2326" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2327">
@@ -42309,69 +42309,69 @@
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2708</v>
+        <v>2689</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2327" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2328">
       <c r="A2328" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2709</v>
+        <v>2708</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2328" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2789</v>
+        <v>2709</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
         </is>
       </c>
       <c r="D2329" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2330">
       <c r="A2330" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2790</v>
+        <v>2789</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>VAGO STA INES 01 HNB</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2330" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2331">
@@ -42381,11 +42381,11 @@
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2791</v>
+        <v>2790</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>DANIELY SLZ 01</t>
+          <t>VAGO STA INES 01 HNB</t>
         </is>
       </c>
       <c r="D2331" t="n">
@@ -42395,19 +42395,19 @@
     <row r="2332">
       <c r="A2332" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2805</v>
+        <v>2791</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>DANIELY SLZ 01</t>
         </is>
       </c>
       <c r="D2332" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2333">
@@ -42417,11 +42417,11 @@
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2806</v>
+        <v>2805</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2333" t="n">
@@ -42435,11 +42435,11 @@
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2807</v>
+        <v>2806</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2334" t="n">
@@ -42453,11 +42453,11 @@
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2808</v>
+        <v>2807</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2335" t="n">
@@ -42467,127 +42467,127 @@
     <row r="2336">
       <c r="A2336" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2820</v>
+        <v>2808</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2336" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2337">
       <c r="A2337" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2765</v>
+        <v>2820</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2337" t="n">
-        <v>98</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2338">
       <c r="A2338" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2842</v>
+        <v>2851</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2338" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2339">
       <c r="A2339" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2741</v>
+        <v>2765</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2339" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2758</v>
+        <v>2842</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2341">
       <c r="A2341" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2659</v>
+        <v>2741</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2341" t="n">
-        <v>100</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2342">
       <c r="A2342" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2669</v>
+        <v>2758</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>135</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2343">
@@ -42597,159 +42597,159 @@
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2672</v>
+        <v>2659</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2343" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2344">
       <c r="A2344" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2344" t="n">
-        <v>2673</v>
+        <v>2669</v>
       </c>
       <c r="C2344" t="inlineStr">
         <is>
-          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2344" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2345">
       <c r="A2345" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2345" t="n">
-        <v>2676</v>
+        <v>2672</v>
       </c>
       <c r="C2345" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2345" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2346">
       <c r="A2346" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2346" t="n">
-        <v>2760</v>
+        <v>2673</v>
       </c>
       <c r="C2346" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2346" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2347">
       <c r="A2347" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2347" t="n">
-        <v>2823</v>
+        <v>2676</v>
       </c>
       <c r="C2347" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2347" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2348">
       <c r="A2348" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2848</v>
+        <v>2760</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2348" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2349">
       <c r="A2349" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2792</v>
+        <v>2823</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2349" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2350">
       <c r="A2350" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2793</v>
+        <v>2848</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2350" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2351">
       <c r="A2351" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2802</v>
+        <v>2792</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2351" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2352">
@@ -42759,11 +42759,11 @@
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2656</v>
+        <v>2793</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2352" t="n">
@@ -42773,19 +42773,19 @@
     <row r="2353">
       <c r="A2353" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2657</v>
+        <v>2802</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA IMP 01 HNB</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2353" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2354">
@@ -42795,33 +42795,33 @@
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2658</v>
+        <v>2656</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2354" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2355">
       <c r="A2355" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2729</v>
+        <v>2657</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>MARIA APARECIDA IMP 01 HNB</t>
         </is>
       </c>
       <c r="D2355" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2356">
@@ -42831,33 +42831,33 @@
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2759</v>
+        <v>2658</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2356" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2832</v>
+        <v>2729</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2357" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2358">
@@ -42867,11 +42867,11 @@
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2769</v>
+        <v>2759</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2358" t="n">
@@ -42881,73 +42881,73 @@
     <row r="2359">
       <c r="A2359" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2679</v>
+        <v>2832</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
         </is>
       </c>
       <c r="D2359" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2360">
       <c r="A2360" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2680</v>
+        <v>2769</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2361">
       <c r="A2361" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2815</v>
+        <v>2679</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2361" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2362">
       <c r="A2362" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2816</v>
+        <v>2680</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2362" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2363">
@@ -42957,105 +42957,105 @@
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2817</v>
+        <v>2815</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2363" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2364">
       <c r="A2364" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2841</v>
+        <v>2816</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2364" t="n">
-        <v>46</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2365">
       <c r="A2365" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2701</v>
+        <v>2817</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2365" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2644</v>
+        <v>2841</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
         </is>
       </c>
       <c r="D2366" t="n">
-        <v>108</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2367">
       <c r="A2367" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2645</v>
+        <v>2701</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2368">
       <c r="A2368" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2754</v>
+        <v>2644</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2368" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2369">
@@ -43065,51 +43065,51 @@
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2755</v>
+        <v>2645</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2369" t="n">
-        <v>80</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2370">
       <c r="A2370" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2665</v>
+        <v>2754</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>141</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2667</v>
+        <v>2755</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>VAGO AÇAILÂNDIA HNB</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2372">
@@ -43119,15 +43119,15 @@
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2727</v>
+        <v>2665</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2372" t="n">
-        <v>120</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2373">
@@ -43137,51 +43137,51 @@
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2728</v>
+        <v>2667</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>VAGO AÇAILÂNDIA HNB</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2374">
       <c r="A2374" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2833</v>
+        <v>2727</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>ADEILZA PINTO DA SILVA - FARMA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2375">
       <c r="A2375" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2814</v>
+        <v>2728</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2375" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2376">
@@ -43191,11 +43191,11 @@
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2646</v>
+        <v>2833</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>ADEILZA PINTO DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2376" t="n">
@@ -43205,19 +43205,19 @@
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2650</v>
+        <v>2814</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2377" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2378">
@@ -43227,15 +43227,15 @@
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2652</v>
+        <v>2646</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2379">
@@ -43245,11 +43245,11 @@
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2653</v>
+        <v>2650</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2379" t="n">
@@ -43263,15 +43263,15 @@
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2654</v>
+        <v>2652</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2380" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2381">
@@ -43281,33 +43281,33 @@
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2655</v>
+        <v>2653</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2382">
       <c r="A2382" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2821</v>
+        <v>2654</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>69</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2383">
@@ -43317,231 +43317,231 @@
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2683</v>
+        <v>2655</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2684</v>
+        <v>2821</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2385">
       <c r="A2385" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2749</v>
+        <v>2683</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2385" t="n">
-        <v>111</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2386">
       <c r="A2386" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2812</v>
+        <v>2684</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>145</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2387">
       <c r="A2387" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2715</v>
+        <v>2749</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>90</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2834</v>
+        <v>2812</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>GILVANA MONTELES U. SANTOS HNB</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>114</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2389">
       <c r="A2389" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2651</v>
+        <v>2715</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>145</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2819</v>
+        <v>2834</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>GILVANA MONTELES U. SANTOS HNB</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2849</v>
+        <v>2651</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>MULTI PE (PEDRO HENRIQUE VIERA)</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>72</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2835</v>
+        <v>2819</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>ROGÉRIO LIRA DA GAMA</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>116</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2699</v>
+        <v>2849</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>MULTI PE (PEDRO HENRIQUE VIERA)</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>95</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2394">
       <c r="A2394" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2706</v>
+        <v>2835</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>VAGO BARREIRINHAS HNB</t>
+          <t>ROGÉRIO LIRA DA GAMA</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2707</v>
+        <v>2699</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>VAGO BACABAL HNB</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2396">
@@ -43551,15 +43551,15 @@
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2846</v>
+        <v>2706</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>VAGO BARREIRINHAS HNB</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2397">
@@ -43569,87 +43569,87 @@
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2847</v>
+        <v>2707</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>WERBERTTY</t>
+          <t>VAGO BACABAL HNB</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2693</v>
+        <v>2846</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2705</v>
+        <v>2847</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>WERBERTTY</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>146</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2400">
       <c r="A2400" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2664</v>
+        <v>2693</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2401">
       <c r="A2401" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2670</v>
+        <v>2705</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>69</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2402">
@@ -43659,195 +43659,195 @@
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2730</v>
+        <v>2664</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2403">
       <c r="A2403" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2671</v>
+        <v>2670</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2404">
       <c r="A2404" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2691</v>
+        <v>2730</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2405">
       <c r="A2405" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2692</v>
+        <v>2671</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2724</v>
+        <v>2691</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2407">
       <c r="A2407" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2773</v>
+        <v>2692</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>TIMON 01 HNB</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2844</v>
+        <v>2724</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>132</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2845</v>
+        <v>2773</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
+          <t>TIMON 01 HNB</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>132</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2410">
       <c r="A2410" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2825</v>
+        <v>2844</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
         </is>
       </c>
       <c r="D2410" t="n">
-        <v>90</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2411">
       <c r="A2411" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2787</v>
+        <v>2845</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>120</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2412">
       <c r="A2412" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2839</v>
+        <v>2825</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>RCA TENA OL PI</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2413">
@@ -43857,69 +43857,69 @@
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2840</v>
+        <v>2787</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>RCA TENA OL MA</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2414">
       <c r="A2414" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2648</v>
+        <v>2839</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>RCA TENA OL PI</t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2415">
       <c r="A2415" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2666</v>
+        <v>2840</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>RCA TENA OL MA</t>
         </is>
       </c>
       <c r="D2415" t="n">
-        <v>63</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2416">
       <c r="A2416" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2779</v>
+        <v>2648</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2416" t="n">
-        <v>105</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2417">
@@ -43929,15 +43929,15 @@
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2780</v>
+        <v>2666</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2418">
@@ -43947,51 +43947,51 @@
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2786</v>
+        <v>2779</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2418" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2419">
       <c r="A2419" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2660</v>
+        <v>2780</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2419" t="n">
-        <v>38</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2420">
       <c r="A2420" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2716</v>
+        <v>2786</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2421">
@@ -44001,51 +44001,51 @@
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2734</v>
+        <v>2660</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2422">
       <c r="A2422" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2742</v>
+        <v>2716</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2423">
       <c r="A2423" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2794</v>
+        <v>2734</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2424">
@@ -44055,11 +44055,11 @@
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2795</v>
+        <v>2742</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2424" t="n">
@@ -44073,15 +44073,15 @@
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2796</v>
+        <v>2794</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
         </is>
       </c>
       <c r="D2425" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2426">
@@ -44091,11 +44091,11 @@
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2797</v>
+        <v>2795</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
         </is>
       </c>
       <c r="D2426" t="n">
@@ -44109,11 +44109,11 @@
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2798</v>
+        <v>2796</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2427" t="n">
@@ -44123,73 +44123,73 @@
     <row r="2428">
       <c r="A2428" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2668</v>
+        <v>2797</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2428" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2429">
       <c r="A2429" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2690</v>
+        <v>2798</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2429" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2430">
       <c r="A2430" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2430" t="n">
-        <v>2696</v>
+        <v>2668</v>
       </c>
       <c r="C2430" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2430" t="n">
-        <v>69</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2431">
       <c r="A2431" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2431" t="n">
-        <v>2697</v>
+        <v>2690</v>
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2431" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2432">
@@ -44199,11 +44199,11 @@
         </is>
       </c>
       <c r="B2432" t="n">
-        <v>2698</v>
+        <v>2696</v>
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2432" t="n">
@@ -44213,37 +44213,37 @@
     <row r="2433">
       <c r="A2433" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2433" t="n">
-        <v>2775</v>
+        <v>2697</v>
       </c>
       <c r="C2433" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2433" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2434">
       <c r="A2434" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2434" t="n">
-        <v>2776</v>
+        <v>2698</v>
       </c>
       <c r="C2434" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2434" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2435">
@@ -44253,11 +44253,11 @@
         </is>
       </c>
       <c r="B2435" t="n">
-        <v>2777</v>
+        <v>2775</v>
       </c>
       <c r="C2435" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2435" t="n">
@@ -44271,11 +44271,11 @@
         </is>
       </c>
       <c r="B2436" t="n">
-        <v>2778</v>
+        <v>2776</v>
       </c>
       <c r="C2436" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2436" t="n">
@@ -44289,15 +44289,15 @@
         </is>
       </c>
       <c r="B2437" t="n">
-        <v>2781</v>
+        <v>2777</v>
       </c>
       <c r="C2437" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2437" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2438">
@@ -44307,11 +44307,11 @@
         </is>
       </c>
       <c r="B2438" t="n">
-        <v>2822</v>
+        <v>2778</v>
       </c>
       <c r="C2438" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2438" t="n">
@@ -44325,87 +44325,87 @@
         </is>
       </c>
       <c r="B2439" t="n">
-        <v>2740</v>
+        <v>2781</v>
       </c>
       <c r="C2439" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2439" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2440">
       <c r="A2440" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2440" t="n">
-        <v>2710</v>
+        <v>2822</v>
       </c>
       <c r="C2440" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2440" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2441">
       <c r="A2441" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2441" t="n">
-        <v>2711</v>
+        <v>2740</v>
       </c>
       <c r="C2441" t="inlineStr">
         <is>
-          <t>CARLOS CHAPADINHA</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2441" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2442">
       <c r="A2442" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2442" t="n">
-        <v>2712</v>
+        <v>2710</v>
       </c>
       <c r="C2442" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2442" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2443">
       <c r="A2443" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2443" t="n">
-        <v>2717</v>
+        <v>2711</v>
       </c>
       <c r="C2443" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>CARLOS CHAPADINHA</t>
         </is>
       </c>
       <c r="D2443" t="n">
-        <v>69</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2444">
@@ -44415,14 +44415,50 @@
         </is>
       </c>
       <c r="B2444" t="n">
+        <v>2712</v>
+      </c>
+      <c r="C2444" t="inlineStr">
+        <is>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
+        </is>
+      </c>
+      <c r="D2444" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2445">
+      <c r="A2445" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2445" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2445" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2445" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2446">
+      <c r="A2446" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2446" t="n">
         <v>2801</v>
       </c>
-      <c r="C2444" t="inlineStr">
+      <c r="C2446" t="inlineStr">
         <is>
           <t>SETOR VAGO VIANA FARMA</t>
         </is>
       </c>
-      <c r="D2444" t="n">
+      <c r="D2446" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:01:28
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2446"/>
+  <dimension ref="A1:D2447"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36679,7 +36679,7 @@
       </c>
       <c r="C2014" t="inlineStr">
         <is>
-          <t>ANTONIA ANGELICA SILVA LOPES-INATIVO</t>
+          <t>KENNEDY ANDERSON VIEIRA DA SILVA CARACO</t>
         </is>
       </c>
       <c r="D2014" t="n">
@@ -41557,7 +41557,7 @@
       </c>
       <c r="C2285" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA - HB</t>
+          <t>VAGO PATRICIA DOS S. NONATO OLIVEIRA-HB</t>
         </is>
       </c>
       <c r="D2285" t="n">
@@ -41845,7 +41845,7 @@
       </c>
       <c r="C2301" t="inlineStr">
         <is>
-          <t>ISALTINO BISPO DE OLIVEIRA JUNIOR - FARM</t>
+          <t>VAGO ISALTINO BISPO DE O. JUNIOR - FARM</t>
         </is>
       </c>
       <c r="D2301" t="n">
@@ -42237,11 +42237,11 @@
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2768</v>
+        <v>2852</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
         </is>
       </c>
       <c r="D2323" t="n">
@@ -42251,73 +42251,73 @@
     <row r="2324">
       <c r="A2324" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2703</v>
+        <v>2768</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2324" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2325">
       <c r="A2325" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2828</v>
+        <v>2703</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>LYERKA MARDANIA RODRIGUES MELO</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2325" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2326">
       <c r="A2326" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2750</v>
+        <v>2828</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>LYERKA MARDANIA RODRIGUES MELO</t>
         </is>
       </c>
       <c r="D2326" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2327">
       <c r="A2327" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2689</v>
+        <v>2750</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2327" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2328">
@@ -42327,69 +42327,69 @@
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2708</v>
+        <v>2689</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2328" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2709</v>
+        <v>2708</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2329" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2330">
       <c r="A2330" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2789</v>
+        <v>2709</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
         </is>
       </c>
       <c r="D2330" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2331">
       <c r="A2331" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2790</v>
+        <v>2789</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>VAGO STA INES 01 HNB</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2331" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2332">
@@ -42399,11 +42399,11 @@
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2791</v>
+        <v>2790</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>DANIELY SLZ 01</t>
+          <t>VAGO STA INES 01 HNB</t>
         </is>
       </c>
       <c r="D2332" t="n">
@@ -42413,19 +42413,19 @@
     <row r="2333">
       <c r="A2333" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2805</v>
+        <v>2791</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>DANIELY SLZ 01</t>
         </is>
       </c>
       <c r="D2333" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2334">
@@ -42435,11 +42435,11 @@
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2806</v>
+        <v>2805</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2334" t="n">
@@ -42453,11 +42453,11 @@
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2807</v>
+        <v>2806</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2335" t="n">
@@ -42471,11 +42471,11 @@
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2808</v>
+        <v>2807</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2336" t="n">
@@ -42485,73 +42485,73 @@
     <row r="2337">
       <c r="A2337" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2820</v>
+        <v>2808</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2337" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2338">
       <c r="A2338" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2851</v>
+        <v>2820</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2338" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2339">
       <c r="A2339" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2765</v>
+        <v>2851</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2339" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2842</v>
+        <v>2765</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2341">
@@ -42561,33 +42561,33 @@
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2741</v>
+        <v>2842</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D2341" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2342">
       <c r="A2342" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2758</v>
+        <v>2741</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2343">
@@ -42597,51 +42597,51 @@
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2659</v>
+        <v>2758</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2343" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2344">
       <c r="A2344" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2344" t="n">
-        <v>2669</v>
+        <v>2659</v>
       </c>
       <c r="C2344" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2344" t="n">
-        <v>135</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2345">
       <c r="A2345" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2345" t="n">
-        <v>2672</v>
+        <v>2669</v>
       </c>
       <c r="C2345" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2345" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2346">
@@ -42651,11 +42651,11 @@
         </is>
       </c>
       <c r="B2346" t="n">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="C2346" t="inlineStr">
         <is>
-          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2346" t="n">
@@ -42665,19 +42665,19 @@
     <row r="2347">
       <c r="A2347" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2347" t="n">
-        <v>2676</v>
+        <v>2673</v>
       </c>
       <c r="C2347" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2347" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2348">
@@ -42687,33 +42687,33 @@
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2760</v>
+        <v>2676</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2348" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2349">
       <c r="A2349" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2823</v>
+        <v>2760</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2349" t="n">
-        <v>80</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2350">
@@ -42723,29 +42723,29 @@
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2848</v>
+        <v>2823</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2350" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2351">
       <c r="A2351" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2792</v>
+        <v>2848</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2351" t="n">
@@ -42755,19 +42755,19 @@
     <row r="2352">
       <c r="A2352" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2793</v>
+        <v>2792</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2352" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2353">
@@ -42777,15 +42777,15 @@
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2802</v>
+        <v>2793</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2353" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2354">
@@ -42795,47 +42795,47 @@
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2656</v>
+        <v>2802</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2354" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2355">
       <c r="A2355" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2657</v>
+        <v>2656</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA IMP 01 HNB</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2355" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2356">
       <c r="A2356" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>MARIA APARECIDA IMP 01 HNB</t>
         </is>
       </c>
       <c r="D2356" t="n">
@@ -42845,37 +42845,37 @@
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2729</v>
+        <v>2658</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2357" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2358">
       <c r="A2358" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2759</v>
+        <v>2729</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2358" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2359">
@@ -42885,15 +42885,15 @@
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2832</v>
+        <v>2759</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2359" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2360">
@@ -42903,33 +42903,33 @@
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2769</v>
+        <v>2832</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2361">
       <c r="A2361" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2679</v>
+        <v>2769</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2361" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2362">
@@ -42939,11 +42939,11 @@
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2362" t="n">
@@ -42953,19 +42953,19 @@
     <row r="2363">
       <c r="A2363" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2815</v>
+        <v>2680</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2363" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2364">
@@ -42975,15 +42975,15 @@
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2816</v>
+        <v>2815</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2364" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2365">
@@ -42993,11 +42993,11 @@
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2817</v>
+        <v>2816</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2365" t="n">
@@ -43007,37 +43007,37 @@
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2841</v>
+        <v>2817</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2366" t="n">
-        <v>46</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2367">
       <c r="A2367" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2701</v>
+        <v>2841</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>90</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2368">
@@ -43047,29 +43047,29 @@
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2644</v>
+        <v>2701</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2368" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2369">
       <c r="A2369" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2645</v>
+        <v>2644</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2369" t="n">
@@ -43083,15 +43083,15 @@
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2754</v>
+        <v>2645</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2371">
@@ -43101,33 +43101,33 @@
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2755</v>
+        <v>2754</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2372">
       <c r="A2372" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2665</v>
+        <v>2755</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2372" t="n">
-        <v>141</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2373">
@@ -43137,15 +43137,15 @@
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2667</v>
+        <v>2665</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>VAGO AÇAILÂNDIA HNB</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>114</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2374">
@@ -43155,15 +43155,15 @@
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2727</v>
+        <v>2667</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>VAGO AÇAILÂNDIA HNB</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2375">
@@ -43173,11 +43173,11 @@
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2728</v>
+        <v>2727</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2375" t="n">
@@ -43187,55 +43187,55 @@
     <row r="2376">
       <c r="A2376" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2833</v>
+        <v>2728</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>ADEILZA PINTO DA SILVA - FARMA</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2376" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2814</v>
+        <v>2833</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>ADEILZA PINTO DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2377" t="n">
-        <v>39</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2378">
       <c r="A2378" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2646</v>
+        <v>2814</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2379">
@@ -43245,11 +43245,11 @@
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2650</v>
+        <v>2646</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2379" t="n">
@@ -43263,15 +43263,15 @@
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2652</v>
+        <v>2650</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2380" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2381">
@@ -43281,15 +43281,15 @@
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2382">
@@ -43299,15 +43299,15 @@
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2654</v>
+        <v>2653</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2383">
@@ -43317,51 +43317,51 @@
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2655</v>
+        <v>2654</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2821</v>
+        <v>2655</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>69</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2385">
       <c r="A2385" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2683</v>
+        <v>2821</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2385" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2386">
@@ -43371,33 +43371,33 @@
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2387">
       <c r="A2387" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2749</v>
+        <v>2684</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2388">
@@ -43407,33 +43407,33 @@
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2812</v>
+        <v>2749</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>145</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2389">
       <c r="A2389" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2715</v>
+        <v>2812</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>90</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2390">
@@ -43443,123 +43443,123 @@
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2834</v>
+        <v>2715</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>GILVANA MONTELES U. SANTOS HNB</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2651</v>
+        <v>2834</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>GILVANA MONTELES U. SANTOS HNB</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>145</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2819</v>
+        <v>2651</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2849</v>
+        <v>2819</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>MULTI PE (PEDRO HENRIQUE VIERA)</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2394">
       <c r="A2394" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2835</v>
+        <v>2849</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>ROGÉRIO LIRA DA GAMA</t>
+          <t>MULTI PE (PEDRO HENRIQUE VIERA)</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>116</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2699</v>
+        <v>2835</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>ROGÉRIO LIRA DA GAMA</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>95</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2396">
       <c r="A2396" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2706</v>
+        <v>2699</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>VAGO BARREIRINHAS HNB</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2397">
@@ -43569,11 +43569,11 @@
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2707</v>
+        <v>2706</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>VAGO BACABAL HNB</t>
+          <t>VAGO BARREIRINHAS HNB</t>
         </is>
       </c>
       <c r="D2397" t="n">
@@ -43587,15 +43587,15 @@
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2846</v>
+        <v>2707</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>VAGO BACABAL HNB</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2399">
@@ -43605,11 +43605,11 @@
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2847</v>
+        <v>2846</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>WERBERTTY</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D2399" t="n">
@@ -43619,127 +43619,127 @@
     <row r="2400">
       <c r="A2400" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2693</v>
+        <v>2847</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>WERBERTTY</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2401">
       <c r="A2401" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2705</v>
+        <v>2693</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>146</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2402">
       <c r="A2402" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2664</v>
+        <v>2705</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>90</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2403">
       <c r="A2403" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2670</v>
+        <v>2664</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2404">
       <c r="A2404" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2730</v>
+        <v>2670</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2405">
       <c r="A2405" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2671</v>
+        <v>2730</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2691</v>
+        <v>2671</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2407">
@@ -43749,11 +43749,11 @@
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2407" t="n">
@@ -43763,55 +43763,55 @@
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2724</v>
+        <v>2692</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2773</v>
+        <v>2724</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>TIMON 01 HNB</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2410">
       <c r="A2410" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2844</v>
+        <v>2773</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
+          <t>TIMON 01 HNB</t>
         </is>
       </c>
       <c r="D2410" t="n">
-        <v>132</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2411">
@@ -43821,11 +43821,11 @@
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2845</v>
+        <v>2844</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
+          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
         </is>
       </c>
       <c r="D2411" t="n">
@@ -43835,19 +43835,19 @@
     <row r="2412">
       <c r="A2412" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2825</v>
+        <v>2845</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>90</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2413">
@@ -43857,51 +43857,51 @@
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2787</v>
+        <v>2825</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2414">
       <c r="A2414" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2839</v>
+        <v>2787</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>RCA TENA OL PI</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2415">
       <c r="A2415" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2840</v>
+        <v>2839</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>RCA TENA OL MA</t>
+          <t>RCA TENA OL PI</t>
         </is>
       </c>
       <c r="D2415" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2416">
@@ -43911,33 +43911,33 @@
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2648</v>
+        <v>2840</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>RCA TENA OL MA</t>
         </is>
       </c>
       <c r="D2416" t="n">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2417">
       <c r="A2417" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2666</v>
+        <v>2648</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>63</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2418">
@@ -43947,15 +43947,15 @@
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2779</v>
+        <v>2666</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2418" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2419">
@@ -43965,11 +43965,11 @@
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2780</v>
+        <v>2779</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D2419" t="n">
@@ -43983,33 +43983,33 @@
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2786</v>
+        <v>2780</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2421">
       <c r="A2421" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2660</v>
+        <v>2786</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2422">
@@ -44019,15 +44019,15 @@
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2716</v>
+        <v>2660</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2423">
@@ -44037,11 +44037,11 @@
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2734</v>
+        <v>2716</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2423" t="n">
@@ -44051,19 +44051,19 @@
     <row r="2424">
       <c r="A2424" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2742</v>
+        <v>2734</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2424" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2425">
@@ -44073,15 +44073,15 @@
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2794</v>
+        <v>2742</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>DEISIELLE JESUS DA SILVA - HB (JACOBINA)</t>
+          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
         </is>
       </c>
       <c r="D2425" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2426">
@@ -44091,15 +44091,15 @@
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2795</v>
+        <v>2794</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
+          <t>VAGO DEISIELLE J. SILVA - HB JACOBINA</t>
         </is>
       </c>
       <c r="D2426" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2427">
@@ -44109,11 +44109,11 @@
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2796</v>
+        <v>2795</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
         </is>
       </c>
       <c r="D2427" t="n">
@@ -44127,11 +44127,11 @@
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2797</v>
+        <v>2796</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>ESDRAS A. SANTOS SANTANA-FAR (PAULO AFO)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2428" t="n">
@@ -44145,11 +44145,11 @@
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2798</v>
+        <v>2797</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>VAGO ESDRAS A. SANTOS-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2429" t="n">
@@ -44159,55 +44159,55 @@
     <row r="2430">
       <c r="A2430" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2430" t="n">
-        <v>2668</v>
+        <v>2798</v>
       </c>
       <c r="C2430" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2430" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2431">
       <c r="A2431" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2431" t="n">
-        <v>2690</v>
+        <v>2668</v>
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2431" t="n">
-        <v>38</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2432">
       <c r="A2432" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2432" t="n">
-        <v>2696</v>
+        <v>2690</v>
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2432" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2433">
@@ -44217,11 +44217,11 @@
         </is>
       </c>
       <c r="B2433" t="n">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="C2433" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2433" t="n">
@@ -44235,11 +44235,11 @@
         </is>
       </c>
       <c r="B2434" t="n">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="C2434" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2434" t="n">
@@ -44249,19 +44249,19 @@
     <row r="2435">
       <c r="A2435" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2435" t="n">
-        <v>2775</v>
+        <v>2698</v>
       </c>
       <c r="C2435" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2435" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2436">
@@ -44271,11 +44271,11 @@
         </is>
       </c>
       <c r="B2436" t="n">
-        <v>2776</v>
+        <v>2775</v>
       </c>
       <c r="C2436" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2436" t="n">
@@ -44289,11 +44289,11 @@
         </is>
       </c>
       <c r="B2437" t="n">
-        <v>2777</v>
+        <v>2776</v>
       </c>
       <c r="C2437" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2437" t="n">
@@ -44307,11 +44307,11 @@
         </is>
       </c>
       <c r="B2438" t="n">
-        <v>2778</v>
+        <v>2777</v>
       </c>
       <c r="C2438" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2438" t="n">
@@ -44325,15 +44325,15 @@
         </is>
       </c>
       <c r="B2439" t="n">
-        <v>2781</v>
+        <v>2778</v>
       </c>
       <c r="C2439" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2439" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2440">
@@ -44343,15 +44343,15 @@
         </is>
       </c>
       <c r="B2440" t="n">
-        <v>2822</v>
+        <v>2781</v>
       </c>
       <c r="C2440" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2440" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2441">
@@ -44361,11 +44361,11 @@
         </is>
       </c>
       <c r="B2441" t="n">
-        <v>2740</v>
+        <v>2822</v>
       </c>
       <c r="C2441" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2441" t="n">
@@ -44375,90 +44375,108 @@
     <row r="2442">
       <c r="A2442" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2442" t="n">
-        <v>2710</v>
+        <v>2740</v>
       </c>
       <c r="C2442" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2442" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2443">
       <c r="A2443" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2443" t="n">
-        <v>2711</v>
+        <v>2710</v>
       </c>
       <c r="C2443" t="inlineStr">
         <is>
-          <t>CARLOS CHAPADINHA</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2443" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2444">
       <c r="A2444" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2444" t="n">
-        <v>2712</v>
+        <v>2711</v>
       </c>
       <c r="C2444" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>CARLOS CHAPADINHA</t>
         </is>
       </c>
       <c r="D2444" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2445">
       <c r="A2445" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2445" t="n">
-        <v>2717</v>
+        <v>2712</v>
       </c>
       <c r="C2445" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
         </is>
       </c>
       <c r="D2445" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2446">
       <c r="A2446" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2446" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2446" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2446" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2447">
+      <c r="A2447" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2447" t="n">
         <v>2801</v>
       </c>
-      <c r="C2446" t="inlineStr">
+      <c r="C2447" t="inlineStr">
         <is>
           <t>SETOR VAGO VIANA FARMA</t>
         </is>
       </c>
-      <c r="D2446" t="n">
+      <c r="D2447" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:02:07
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2447"/>
+  <dimension ref="A1:D2448"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4205,7 +4205,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>INATIVO - FELIPE FERNANDES FONTINELES</t>
+          <t>SAMARA ALVES DA SILVA</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -27592,7 +27592,7 @@
         </is>
       </c>
       <c r="D1509" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="1510">
@@ -27736,7 +27736,7 @@
         </is>
       </c>
       <c r="D1517" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="1518">
@@ -33064,7 +33064,7 @@
         </is>
       </c>
       <c r="D1813" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="1814">
@@ -33082,7 +33082,7 @@
         </is>
       </c>
       <c r="D1814" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="1815">
@@ -33820,7 +33820,7 @@
         </is>
       </c>
       <c r="D1855" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="1856">
@@ -35166,7 +35166,7 @@
       </c>
       <c r="C1930" t="inlineStr">
         <is>
-          <t>GUILHERME FERREIRA DE SOUSA (DEDICADA)</t>
+          <t>GUILHERME FERREIRA DE SOUSA</t>
         </is>
       </c>
       <c r="D1930" t="n">
@@ -35765,7 +35765,7 @@
         </is>
       </c>
       <c r="D1963" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="1964">
@@ -36287,7 +36287,7 @@
         </is>
       </c>
       <c r="D1992" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="1993">
@@ -36467,7 +36467,7 @@
         </is>
       </c>
       <c r="D2002" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2003">
@@ -36611,7 +36611,7 @@
         </is>
       </c>
       <c r="D2010" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2011">
@@ -37961,7 +37961,7 @@
         </is>
       </c>
       <c r="D2085" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2086">
@@ -38479,7 +38479,7 @@
       </c>
       <c r="C2114" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS FARMA SUPERVI</t>
+          <t>INATIVO PAULO CESAR D. LEMOS FARMA SUP</t>
         </is>
       </c>
       <c r="D2114" t="n">
@@ -38879,7 +38879,7 @@
         </is>
       </c>
       <c r="D2136" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2137">
@@ -40247,7 +40247,7 @@
         </is>
       </c>
       <c r="D2212" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2213">
@@ -40261,7 +40261,7 @@
       </c>
       <c r="C2213" t="inlineStr">
         <is>
-          <t>SALGUEIRO - HB  (DEBORA ALVES )</t>
+          <t>SALGUEIRO - HB  (LUCIENE ALVES )</t>
         </is>
       </c>
       <c r="D2213" t="n">
@@ -40427,7 +40427,7 @@
         </is>
       </c>
       <c r="D2222" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2223">
@@ -40877,7 +40877,7 @@
         </is>
       </c>
       <c r="D2247" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2248">
@@ -40991,127 +40991,127 @@
     <row r="2254">
       <c r="A2254" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2254" t="n">
-        <v>2598</v>
+        <v>2534</v>
       </c>
       <c r="C2254" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - FARMA</t>
+          <t>MARCIA JORDANIA COSTA DE ARAUJO</t>
         </is>
       </c>
       <c r="D2254" t="n">
-        <v>83</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2255">
       <c r="A2255" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2255" t="n">
-        <v>2534</v>
+        <v>2369</v>
       </c>
       <c r="C2255" t="inlineStr">
         <is>
-          <t>MARCIA JORDANIA COSTA DE ARAUJO</t>
+          <t>RCA GLOBO PLUS PI</t>
         </is>
       </c>
       <c r="D2255" t="n">
-        <v>114</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2256">
       <c r="A2256" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2256" t="n">
-        <v>2369</v>
+        <v>2409</v>
       </c>
       <c r="C2256" t="inlineStr">
         <is>
-          <t>RCA GLOBO PLUS PI</t>
+          <t>VAGO ANDRE BORGES DOURADO - FARMA</t>
         </is>
       </c>
       <c r="D2256" t="n">
-        <v>26</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2257">
       <c r="A2257" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2257" t="n">
-        <v>2409</v>
+        <v>2495</v>
       </c>
       <c r="C2257" t="inlineStr">
         <is>
-          <t>VAGO ANDRE BORGES DOURADO - FARMA</t>
+          <t>INATIVO- JOSE NERTAN COSTA SABINO</t>
         </is>
       </c>
       <c r="D2257" t="n">
-        <v>95</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2258">
       <c r="A2258" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2258" t="n">
-        <v>2495</v>
+        <v>2504</v>
       </c>
       <c r="C2258" t="inlineStr">
         <is>
-          <t>INATIVO- JOSE NERTAN COSTA SABINO</t>
+          <t>KAYRO RAFAEL DE JESUS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2258" t="n">
-        <v>46</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2259">
       <c r="A2259" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2259" t="n">
-        <v>2504</v>
+        <v>2359</v>
       </c>
       <c r="C2259" t="inlineStr">
         <is>
-          <t>KAYRO RAFAEL DE JESUS OLIVEIRA</t>
+          <t>JOAO CARLOS OLIVEIRA RODRIGUES</t>
         </is>
       </c>
       <c r="D2259" t="n">
-        <v>39</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2260">
       <c r="A2260" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2260" t="n">
-        <v>2359</v>
+        <v>2486</v>
       </c>
       <c r="C2260" t="inlineStr">
         <is>
-          <t>JOAO CARLOS OLIVEIRA RODRIGUES</t>
+          <t>PATRICIA SOUSA SANTOS</t>
         </is>
       </c>
       <c r="D2260" t="n">
-        <v>69</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2261">
@@ -41121,15 +41121,15 @@
         </is>
       </c>
       <c r="B2261" t="n">
-        <v>2486</v>
+        <v>2521</v>
       </c>
       <c r="C2261" t="inlineStr">
         <is>
-          <t>PATRICIA SOUSA SANTOS</t>
+          <t>OSMANYEL MENEZES VIEIRA</t>
         </is>
       </c>
       <c r="D2261" t="n">
-        <v>141</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2262">
@@ -41139,11 +41139,11 @@
         </is>
       </c>
       <c r="B2262" t="n">
-        <v>2521</v>
+        <v>2540</v>
       </c>
       <c r="C2262" t="inlineStr">
         <is>
-          <t>OSMANYEL MENEZES VIEIRA</t>
+          <t>ZALMIR PAIXAO MENDES JUNIOR</t>
         </is>
       </c>
       <c r="D2262" t="n">
@@ -41157,11 +41157,11 @@
         </is>
       </c>
       <c r="B2263" t="n">
-        <v>2540</v>
+        <v>2704</v>
       </c>
       <c r="C2263" t="inlineStr">
         <is>
-          <t>ZALMIR PAIXAO MENDES JUNIOR</t>
+          <t>DEDICADA MA (EVALDO)</t>
         </is>
       </c>
       <c r="D2263" t="n">
@@ -41171,109 +41171,109 @@
     <row r="2264">
       <c r="A2264" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2264" t="n">
-        <v>2704</v>
+        <v>2725</v>
       </c>
       <c r="C2264" t="inlineStr">
         <is>
-          <t>DEDICADA MA (EVALDO)</t>
+          <t>VAGO MARIA APARECIDA D. FRAGA - FARMA</t>
         </is>
       </c>
       <c r="D2264" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2265">
       <c r="A2265" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2265" t="n">
-        <v>2725</v>
+        <v>2726</v>
       </c>
       <c r="C2265" t="inlineStr">
         <is>
-          <t>VAGO MARIA APARECIDA D. FRAGA - FARMA</t>
+          <t>SETOR CODÓ VAGO FARMA</t>
         </is>
       </c>
       <c r="D2265" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2266">
       <c r="A2266" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2266" t="n">
-        <v>2726</v>
+        <v>2757</v>
       </c>
       <c r="C2266" t="inlineStr">
         <is>
-          <t>SETOR CODÓ VAGO FARMA</t>
+          <t>FERNANDA MASCARENHAS CEDRAZ - FARMA</t>
         </is>
       </c>
       <c r="D2266" t="n">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2267">
       <c r="A2267" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2267" t="n">
-        <v>2757</v>
+        <v>2810</v>
       </c>
       <c r="C2267" t="inlineStr">
         <is>
-          <t>FERNANDA MASCARENHAS CEDRAZ - FARMA</t>
+          <t>SILVESTRA COSTA NUNES</t>
         </is>
       </c>
       <c r="D2267" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2268">
       <c r="A2268" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2268" t="n">
-        <v>2810</v>
+        <v>2829</v>
       </c>
       <c r="C2268" t="inlineStr">
         <is>
-          <t>SILVESTRA COSTA NUNES</t>
+          <t>LAIS ANDRADE VIRIATO - FARMA</t>
         </is>
       </c>
       <c r="D2268" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2269">
       <c r="A2269" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2269" t="n">
-        <v>2829</v>
+        <v>2836</v>
       </c>
       <c r="C2269" t="inlineStr">
         <is>
-          <t>LAIS ANDRADE VIRIATO - FARMA</t>
+          <t>MARIA EDUARDA SILVA SANTOS</t>
         </is>
       </c>
       <c r="D2269" t="n">
-        <v>95</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2270">
@@ -41283,11 +41283,11 @@
         </is>
       </c>
       <c r="B2270" t="n">
-        <v>2836</v>
+        <v>2837</v>
       </c>
       <c r="C2270" t="inlineStr">
         <is>
-          <t>MARIA EDUARDA SILVA SANTOS</t>
+          <t>MERCYA BERCE NASCIMENTO DE MESQUITA</t>
         </is>
       </c>
       <c r="D2270" t="n">
@@ -41297,55 +41297,55 @@
     <row r="2271">
       <c r="A2271" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2271" t="n">
-        <v>2837</v>
+        <v>2838</v>
       </c>
       <c r="C2271" t="inlineStr">
         <is>
-          <t>MERCYA BERCE NASCIMENTO DE MESQUITA</t>
+          <t>CAIO LUA MENDES DE ARAUJO</t>
         </is>
       </c>
       <c r="D2271" t="n">
-        <v>108</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2272">
       <c r="A2272" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2272" t="n">
-        <v>2838</v>
+        <v>2850</v>
       </c>
       <c r="C2272" t="inlineStr">
         <is>
-          <t>CAIO LUA MENDES DE ARAUJO</t>
+          <t>FERNANDO DE QUEIROZ COSTA - FARMA</t>
         </is>
       </c>
       <c r="D2272" t="n">
-        <v>80</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2273">
       <c r="A2273" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2273" t="n">
-        <v>2850</v>
+        <v>2799</v>
       </c>
       <c r="C2273" t="inlineStr">
         <is>
-          <t>FERNANDO DE QUEIROZ COSTA - FARMA</t>
+          <t>VOLFRAMIO DALFREDO ALMEIDA</t>
         </is>
       </c>
       <c r="D2273" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2274">
@@ -41355,33 +41355,33 @@
         </is>
       </c>
       <c r="B2274" t="n">
-        <v>2799</v>
+        <v>2719</v>
       </c>
       <c r="C2274" t="inlineStr">
         <is>
-          <t>VOLFRAMIO DALFREDO ALMEIDA</t>
+          <t>SETOR SÃO RDO NONATO VAGO  (DEDICADA)</t>
         </is>
       </c>
       <c r="D2274" t="n">
-        <v>69</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2275">
       <c r="A2275" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2275" t="n">
-        <v>2719</v>
+        <v>2731</v>
       </c>
       <c r="C2275" t="inlineStr">
         <is>
-          <t>SETOR SÃO RDO NONATO VAGO  (DEDICADA)</t>
+          <t>VAGO ANDERSON A. S. - FARMA (CAMAÇARI)</t>
         </is>
       </c>
       <c r="D2275" t="n">
-        <v>39</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2276">
@@ -41391,15 +41391,15 @@
         </is>
       </c>
       <c r="B2276" t="n">
-        <v>2731</v>
+        <v>2732</v>
       </c>
       <c r="C2276" t="inlineStr">
         <is>
-          <t>VAGO ANDERSON A. S. - FARMA (CAMAÇARI)</t>
+          <t>VAGO BRENO ALLAN DE JESUS - HB</t>
         </is>
       </c>
       <c r="D2276" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2277">
@@ -41409,51 +41409,51 @@
         </is>
       </c>
       <c r="B2277" t="n">
-        <v>2732</v>
+        <v>2733</v>
       </c>
       <c r="C2277" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN DE JESUS - HB</t>
+          <t xml:space="preserve">VAGO CENTRO CAROLINE LEMOS - FARMA </t>
         </is>
       </c>
       <c r="D2277" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2278">
       <c r="A2278" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2278" t="n">
-        <v>2733</v>
+        <v>2752</v>
       </c>
       <c r="C2278" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAGO CENTRO CAROLINE LEMOS - FARMA </t>
+          <t>SETOR BAIXADA PLUS (ELILTON ROMEU)</t>
         </is>
       </c>
       <c r="D2278" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2279">
       <c r="A2279" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2279" t="n">
-        <v>2752</v>
+        <v>2662</v>
       </c>
       <c r="C2279" t="inlineStr">
         <is>
-          <t>SETOR BAIXADA PLUS (ELILTON ROMEU)</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
         </is>
       </c>
       <c r="D2279" t="n">
-        <v>114</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2280">
@@ -41463,15 +41463,15 @@
         </is>
       </c>
       <c r="B2280" t="n">
-        <v>2662</v>
+        <v>2663</v>
       </c>
       <c r="C2280" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
+          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
         </is>
       </c>
       <c r="D2280" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2281">
@@ -41481,15 +41481,15 @@
         </is>
       </c>
       <c r="B2281" t="n">
-        <v>2663</v>
+        <v>2685</v>
       </c>
       <c r="C2281" t="inlineStr">
         <is>
-          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
+          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2281" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2282">
@@ -41499,15 +41499,15 @@
         </is>
       </c>
       <c r="B2282" t="n">
-        <v>2685</v>
+        <v>2718</v>
       </c>
       <c r="C2282" t="inlineStr">
         <is>
-          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
+          <t>KALILLA FERREIRA COSTA - FARMA</t>
         </is>
       </c>
       <c r="D2282" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2283">
@@ -41517,15 +41517,15 @@
         </is>
       </c>
       <c r="B2283" t="n">
-        <v>2718</v>
+        <v>2674</v>
       </c>
       <c r="C2283" t="inlineStr">
         <is>
-          <t>KALILLA FERREIRA COSTA - FARMA</t>
+          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
         </is>
       </c>
       <c r="D2283" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2284">
@@ -41535,15 +41535,15 @@
         </is>
       </c>
       <c r="B2284" t="n">
-        <v>2674</v>
+        <v>2753</v>
       </c>
       <c r="C2284" t="inlineStr">
         <is>
-          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
+          <t>VAGO PATRICIA DOS S. NONATO OLIVEIRA-HB</t>
         </is>
       </c>
       <c r="D2284" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2285">
@@ -41553,15 +41553,15 @@
         </is>
       </c>
       <c r="B2285" t="n">
-        <v>2753</v>
+        <v>2772</v>
       </c>
       <c r="C2285" t="inlineStr">
         <is>
-          <t>VAGO PATRICIA DOS S. NONATO OLIVEIRA-HB</t>
+          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2285" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2286">
@@ -41571,51 +41571,51 @@
         </is>
       </c>
       <c r="B2286" t="n">
-        <v>2772</v>
+        <v>2827</v>
       </c>
       <c r="C2286" t="inlineStr">
         <is>
-          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
+          <t>VAGO JOELTON MUNIZ DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2286" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2287">
       <c r="A2287" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2287" t="n">
-        <v>2827</v>
+        <v>2756</v>
       </c>
       <c r="C2287" t="inlineStr">
         <is>
-          <t>VAGO JOELTON MUNIZ DE SOUZA - HB</t>
+          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
         </is>
       </c>
       <c r="D2287" t="n">
-        <v>98</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2288">
       <c r="A2288" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2288" t="n">
-        <v>2756</v>
+        <v>2813</v>
       </c>
       <c r="C2288" t="inlineStr">
         <is>
-          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
+          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
         </is>
       </c>
       <c r="D2288" t="n">
-        <v>39</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2289">
@@ -41625,15 +41625,15 @@
         </is>
       </c>
       <c r="B2289" t="n">
-        <v>2813</v>
+        <v>2738</v>
       </c>
       <c r="C2289" t="inlineStr">
         <is>
-          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
+          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2289" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2290">
@@ -41643,11 +41643,11 @@
         </is>
       </c>
       <c r="B2290" t="n">
-        <v>2738</v>
+        <v>2739</v>
       </c>
       <c r="C2290" t="inlineStr">
         <is>
-          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
+          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2290" t="n">
@@ -41661,33 +41661,33 @@
         </is>
       </c>
       <c r="B2291" t="n">
-        <v>2739</v>
+        <v>2824</v>
       </c>
       <c r="C2291" t="inlineStr">
         <is>
-          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D2291" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2292">
       <c r="A2292" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2292" t="n">
-        <v>2824</v>
+        <v>2843</v>
       </c>
       <c r="C2292" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>VAGO FEIRA DE SANTANA II - FARMA</t>
         </is>
       </c>
       <c r="D2292" t="n">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2293">
@@ -41697,11 +41697,11 @@
         </is>
       </c>
       <c r="B2293" t="n">
-        <v>2843</v>
+        <v>2747</v>
       </c>
       <c r="C2293" t="inlineStr">
         <is>
-          <t>VAGO FEIRA DE SANTANA II - FARMA</t>
+          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
         </is>
       </c>
       <c r="D2293" t="n">
@@ -41715,11 +41715,11 @@
         </is>
       </c>
       <c r="B2294" t="n">
-        <v>2747</v>
+        <v>2748</v>
       </c>
       <c r="C2294" t="inlineStr">
         <is>
-          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
+          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
         </is>
       </c>
       <c r="D2294" t="n">
@@ -41729,73 +41729,73 @@
     <row r="2295">
       <c r="A2295" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2295" t="n">
-        <v>2748</v>
+        <v>2766</v>
       </c>
       <c r="C2295" t="inlineStr">
         <is>
-          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
+          <t>SETOR VAGO PEDREIRAS</t>
         </is>
       </c>
       <c r="D2295" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2296">
       <c r="A2296" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2296" t="n">
-        <v>2766</v>
+        <v>2767</v>
       </c>
       <c r="C2296" t="inlineStr">
         <is>
-          <t>SETOR VAGO PEDREIRAS</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D2296" t="n">
-        <v>120</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2297">
       <c r="A2297" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2297" t="n">
-        <v>2767</v>
+        <v>2688</v>
       </c>
       <c r="C2297" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2297" t="n">
-        <v>39</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2298">
       <c r="A2298" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2298" t="n">
-        <v>2688</v>
+        <v>2694</v>
       </c>
       <c r="C2298" t="inlineStr">
         <is>
-          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
+          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2298" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2299">
@@ -41805,15 +41805,15 @@
         </is>
       </c>
       <c r="B2299" t="n">
-        <v>2694</v>
+        <v>2714</v>
       </c>
       <c r="C2299" t="inlineStr">
         <is>
-          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
+          <t>PRISCILA DOS SANTOS LOPES - HB</t>
         </is>
       </c>
       <c r="D2299" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2300">
@@ -41823,15 +41823,15 @@
         </is>
       </c>
       <c r="B2300" t="n">
-        <v>2714</v>
+        <v>2722</v>
       </c>
       <c r="C2300" t="inlineStr">
         <is>
-          <t>PRISCILA DOS SANTOS LOPES - HB</t>
+          <t>VAGO ISALTINO BISPO DE O. JUNIOR - FARM</t>
         </is>
       </c>
       <c r="D2300" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2301">
@@ -41841,15 +41841,15 @@
         </is>
       </c>
       <c r="B2301" t="n">
-        <v>2722</v>
+        <v>2723</v>
       </c>
       <c r="C2301" t="inlineStr">
         <is>
-          <t>VAGO ISALTINO BISPO DE O. JUNIOR - FARM</t>
+          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2301" t="n">
-        <v>50</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2302">
@@ -41859,15 +41859,15 @@
         </is>
       </c>
       <c r="B2302" t="n">
-        <v>2723</v>
+        <v>2803</v>
       </c>
       <c r="C2302" t="inlineStr">
         <is>
-          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
         </is>
       </c>
       <c r="D2302" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2303">
@@ -41877,11 +41877,11 @@
         </is>
       </c>
       <c r="B2303" t="n">
-        <v>2803</v>
+        <v>2804</v>
       </c>
       <c r="C2303" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
+          <t>PAULA CARLA CALDAS MOTA - HB</t>
         </is>
       </c>
       <c r="D2303" t="n">
@@ -41891,19 +41891,19 @@
     <row r="2304">
       <c r="A2304" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2304" t="n">
-        <v>2804</v>
+        <v>2830</v>
       </c>
       <c r="C2304" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA - HB</t>
+          <t>SETOR VAGO BALSAS 1</t>
         </is>
       </c>
       <c r="D2304" t="n">
-        <v>98</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2305">
@@ -41913,11 +41913,11 @@
         </is>
       </c>
       <c r="B2305" t="n">
-        <v>2830</v>
+        <v>2831</v>
       </c>
       <c r="C2305" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 1</t>
+          <t>SETOR VAGO BALSAS 2</t>
         </is>
       </c>
       <c r="D2305" t="n">
@@ -41927,55 +41927,55 @@
     <row r="2306">
       <c r="A2306" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2306" t="n">
-        <v>2831</v>
+        <v>2647</v>
       </c>
       <c r="C2306" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 2</t>
+          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
         </is>
       </c>
       <c r="D2306" t="n">
-        <v>120</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2307">
       <c r="A2307" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2307" t="n">
-        <v>2647</v>
+        <v>2661</v>
       </c>
       <c r="C2307" t="inlineStr">
         <is>
-          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
+          <t>MARIA ISADORA DOS REIS REGO</t>
         </is>
       </c>
       <c r="D2307" t="n">
-        <v>147</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2308">
       <c r="A2308" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2308" t="n">
-        <v>2661</v>
+        <v>2686</v>
       </c>
       <c r="C2308" t="inlineStr">
         <is>
-          <t>MARIA ISADORA DOS REIS REGO</t>
+          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2308" t="n">
-        <v>76</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2309">
@@ -41985,11 +41985,11 @@
         </is>
       </c>
       <c r="B2309" t="n">
-        <v>2686</v>
+        <v>2687</v>
       </c>
       <c r="C2309" t="inlineStr">
         <is>
-          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
+          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
         </is>
       </c>
       <c r="D2309" t="n">
@@ -41999,109 +41999,109 @@
     <row r="2310">
       <c r="A2310" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2310" t="n">
-        <v>2687</v>
+        <v>2681</v>
       </c>
       <c r="C2310" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
+          <t>RCA PRINCIPIA OL PI</t>
         </is>
       </c>
       <c r="D2310" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2311" t="n">
-        <v>2681</v>
+        <v>2682</v>
       </c>
       <c r="C2311" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL PI</t>
+          <t>RCA PRINCIPIA OL MA</t>
         </is>
       </c>
       <c r="D2311" t="n">
-        <v>69</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2312">
       <c r="A2312" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2312" t="n">
-        <v>2682</v>
+        <v>2826</v>
       </c>
       <c r="C2312" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL MA</t>
+          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
         </is>
       </c>
       <c r="D2312" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2313">
       <c r="A2313" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2313" t="n">
-        <v>2826</v>
+        <v>2677</v>
       </c>
       <c r="C2313" t="inlineStr">
         <is>
-          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
+          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
         </is>
       </c>
       <c r="D2313" t="n">
-        <v>95</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2314">
       <c r="A2314" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2314" t="n">
-        <v>2677</v>
+        <v>2678</v>
       </c>
       <c r="C2314" t="inlineStr">
         <is>
-          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
+          <t>ADRIEL XERXES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D2314" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2315">
       <c r="A2315" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2315" t="n">
-        <v>2678</v>
+        <v>2735</v>
       </c>
       <c r="C2315" t="inlineStr">
         <is>
-          <t>ADRIEL XERXES BARROS MARTINS</t>
+          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2315" t="n">
-        <v>69</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2316">
@@ -42111,15 +42111,15 @@
         </is>
       </c>
       <c r="B2316" t="n">
-        <v>2735</v>
+        <v>2736</v>
       </c>
       <c r="C2316" t="inlineStr">
         <is>
-          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
+          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2316" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2317">
@@ -42129,15 +42129,15 @@
         </is>
       </c>
       <c r="B2317" t="n">
-        <v>2736</v>
+        <v>2737</v>
       </c>
       <c r="C2317" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
         </is>
       </c>
       <c r="D2317" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2318">
@@ -42147,15 +42147,15 @@
         </is>
       </c>
       <c r="B2318" t="n">
-        <v>2737</v>
+        <v>2743</v>
       </c>
       <c r="C2318" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
+          <t>VAGO SEABRA - FARMA</t>
         </is>
       </c>
       <c r="D2318" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2319">
@@ -42165,11 +42165,11 @@
         </is>
       </c>
       <c r="B2319" t="n">
-        <v>2743</v>
+        <v>2744</v>
       </c>
       <c r="C2319" t="inlineStr">
         <is>
-          <t>VAGO SEABRA - FARMA</t>
+          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
         </is>
       </c>
       <c r="D2319" t="n">
@@ -42183,15 +42183,15 @@
         </is>
       </c>
       <c r="B2320" t="n">
-        <v>2744</v>
+        <v>2745</v>
       </c>
       <c r="C2320" t="inlineStr">
         <is>
-          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
+          <t>CIRLANE ARAUJO SOUZA - HB</t>
         </is>
       </c>
       <c r="D2320" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2321">
@@ -42201,33 +42201,33 @@
         </is>
       </c>
       <c r="B2321" t="n">
-        <v>2745</v>
+        <v>2783</v>
       </c>
       <c r="C2321" t="inlineStr">
         <is>
-          <t>CIRLANE ARAUJO SOUZA - HB</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2321" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2322">
       <c r="A2322" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2322" t="n">
-        <v>2783</v>
+        <v>2852</v>
       </c>
       <c r="C2322" t="inlineStr">
         <is>
-          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
+          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
         </is>
       </c>
       <c r="D2322" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2323">
@@ -42237,11 +42237,11 @@
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2852</v>
+        <v>2768</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2323" t="n">
@@ -42251,73 +42251,73 @@
     <row r="2324">
       <c r="A2324" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2768</v>
+        <v>2703</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2324" t="n">
-        <v>69</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2325">
       <c r="A2325" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2703</v>
+        <v>2828</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>LYERKA MARDANIA RODRIGUES MELO</t>
         </is>
       </c>
       <c r="D2325" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2326">
       <c r="A2326" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2828</v>
+        <v>2750</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>LYERKA MARDANIA RODRIGUES MELO</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2326" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2327">
       <c r="A2327" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2750</v>
+        <v>2689</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2327" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2328">
@@ -42327,69 +42327,69 @@
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2689</v>
+        <v>2708</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2328" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2708</v>
+        <v>2709</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>BRUNO TEIXEIRA TORRES</t>
         </is>
       </c>
       <c r="D2329" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2330">
       <c r="A2330" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2709</v>
+        <v>2789</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES (DEDICADA)</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2330" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2331">
       <c r="A2331" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2789</v>
+        <v>2790</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>VAGO STA INES 01 HNB</t>
         </is>
       </c>
       <c r="D2331" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2332">
@@ -42399,11 +42399,11 @@
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2790</v>
+        <v>2791</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>VAGO STA INES 01 HNB</t>
+          <t>DANIELY SLZ 01</t>
         </is>
       </c>
       <c r="D2332" t="n">
@@ -42413,19 +42413,19 @@
     <row r="2333">
       <c r="A2333" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2791</v>
+        <v>2805</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>DANIELY SLZ 01</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2333" t="n">
-        <v>114</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2334">
@@ -42435,11 +42435,11 @@
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2805</v>
+        <v>2806</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2334" t="n">
@@ -42453,11 +42453,11 @@
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2806</v>
+        <v>2807</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2335" t="n">
@@ -42471,11 +42471,11 @@
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2807</v>
+        <v>2808</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2336" t="n">
@@ -42485,73 +42485,73 @@
     <row r="2337">
       <c r="A2337" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2808</v>
+        <v>2820</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2337" t="n">
-        <v>104</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2338">
       <c r="A2338" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2820</v>
+        <v>2851</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2338" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2339">
       <c r="A2339" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2851</v>
+        <v>2765</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2339" t="n">
-        <v>69</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2765</v>
+        <v>2842</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>98</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2341">
@@ -42561,33 +42561,33 @@
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2842</v>
+        <v>2741</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2341" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2342">
       <c r="A2342" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2741</v>
+        <v>2758</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2343">
@@ -42597,11 +42597,11 @@
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2758</v>
+        <v>2854</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>JONILSON SANTANA SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2343" t="n">
@@ -44073,15 +44073,15 @@
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2742</v>
+        <v>2853</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS C. AZEVEDO - FARMA</t>
+          <t>H - ROBERTO SOARES OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2425" t="n">
-        <v>95</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2426">
@@ -44091,15 +44091,15 @@
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2794</v>
+        <v>2742</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>VAGO DEISIELLE J. SILVA - HB JACOBINA</t>
+          <t>VAGO MARCUS VINICIUS - FARMA JACOBINA</t>
         </is>
       </c>
       <c r="D2426" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2427">
@@ -44109,15 +44109,15 @@
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2795</v>
+        <v>2794</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
+          <t>VAGO DEISIELLE J. SILVA - HB JACOBINA</t>
         </is>
       </c>
       <c r="D2427" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2428">
@@ -44127,11 +44127,11 @@
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2796</v>
+        <v>2795</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
         </is>
       </c>
       <c r="D2428" t="n">
@@ -44145,11 +44145,11 @@
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2797</v>
+        <v>2796</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>VAGO ESDRAS A. SANTOS-FAR (PAULO AFO)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2429" t="n">
@@ -44163,11 +44163,11 @@
         </is>
       </c>
       <c r="B2430" t="n">
-        <v>2798</v>
+        <v>2797</v>
       </c>
       <c r="C2430" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>VAGO ESDRAS A. SANTOS-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2430" t="n">
@@ -44177,55 +44177,55 @@
     <row r="2431">
       <c r="A2431" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2431" t="n">
-        <v>2668</v>
+        <v>2798</v>
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2431" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2432">
       <c r="A2432" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2432" t="n">
-        <v>2690</v>
+        <v>2668</v>
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2432" t="n">
-        <v>38</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2433">
       <c r="A2433" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2433" t="n">
-        <v>2696</v>
+        <v>2690</v>
       </c>
       <c r="C2433" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2433" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2434">
@@ -44235,11 +44235,11 @@
         </is>
       </c>
       <c r="B2434" t="n">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="C2434" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2434" t="n">
@@ -44253,11 +44253,11 @@
         </is>
       </c>
       <c r="B2435" t="n">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="C2435" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2435" t="n">
@@ -44267,19 +44267,19 @@
     <row r="2436">
       <c r="A2436" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2436" t="n">
-        <v>2775</v>
+        <v>2698</v>
       </c>
       <c r="C2436" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2436" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2437">
@@ -44289,11 +44289,11 @@
         </is>
       </c>
       <c r="B2437" t="n">
-        <v>2776</v>
+        <v>2775</v>
       </c>
       <c r="C2437" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2437" t="n">
@@ -44307,11 +44307,11 @@
         </is>
       </c>
       <c r="B2438" t="n">
-        <v>2777</v>
+        <v>2776</v>
       </c>
       <c r="C2438" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2438" t="n">
@@ -44325,11 +44325,11 @@
         </is>
       </c>
       <c r="B2439" t="n">
-        <v>2778</v>
+        <v>2777</v>
       </c>
       <c r="C2439" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2439" t="n">
@@ -44343,15 +44343,15 @@
         </is>
       </c>
       <c r="B2440" t="n">
-        <v>2781</v>
+        <v>2778</v>
       </c>
       <c r="C2440" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2440" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2441">
@@ -44361,15 +44361,15 @@
         </is>
       </c>
       <c r="B2441" t="n">
-        <v>2822</v>
+        <v>2781</v>
       </c>
       <c r="C2441" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2441" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2442">
@@ -44379,11 +44379,11 @@
         </is>
       </c>
       <c r="B2442" t="n">
-        <v>2740</v>
+        <v>2822</v>
       </c>
       <c r="C2442" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2442" t="n">
@@ -44393,90 +44393,108 @@
     <row r="2443">
       <c r="A2443" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2443" t="n">
-        <v>2710</v>
+        <v>2740</v>
       </c>
       <c r="C2443" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2443" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2444">
       <c r="A2444" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2444" t="n">
-        <v>2711</v>
+        <v>2710</v>
       </c>
       <c r="C2444" t="inlineStr">
         <is>
-          <t>CARLOS CHAPADINHA</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2444" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2445">
       <c r="A2445" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2445" t="n">
-        <v>2712</v>
+        <v>2711</v>
       </c>
       <c r="C2445" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>CARLOS CHAPADINHA</t>
         </is>
       </c>
       <c r="D2445" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2446">
       <c r="A2446" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2446" t="n">
-        <v>2717</v>
+        <v>2712</v>
       </c>
       <c r="C2446" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
         </is>
       </c>
       <c r="D2446" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2447">
       <c r="A2447" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2447" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2447" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2447" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2448">
+      <c r="A2448" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2448" t="n">
         <v>2801</v>
       </c>
-      <c r="C2447" t="inlineStr">
+      <c r="C2448" t="inlineStr">
         <is>
           <t>SETOR VAGO VIANA FARMA</t>
         </is>
       </c>
-      <c r="D2447" t="n">
+      <c r="D2448" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:02:43
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -14110,7 +14110,7 @@
         </is>
       </c>
       <c r="D760" t="n">
-        <v>120</v>
+        <v>58</v>
       </c>
     </row>
     <row r="761">
@@ -44077,7 +44077,7 @@
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>H - ROBERTO SOARES OLIVEIRA JUNIOR</t>
+          <t>H-ROBERTO SOARES OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2425" t="n">

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:02:26
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -3201,7 +3201,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>138</v>
+        <v>43</v>
       </c>
     </row>
     <row r="155">
@@ -30742,7 +30742,7 @@
         </is>
       </c>
       <c r="D1684" t="n">
-        <v>138</v>
+        <v>43</v>
       </c>
     </row>
     <row r="1685">
@@ -32668,7 +32668,7 @@
         </is>
       </c>
       <c r="D1791" t="n">
-        <v>138</v>
+        <v>43</v>
       </c>
     </row>
     <row r="1792">
@@ -36823,7 +36823,7 @@
       </c>
       <c r="C2022" t="inlineStr">
         <is>
-          <t>ELIELTON PINHEIRO HNB</t>
+          <t>ELILTON PINHEIRO HNB</t>
         </is>
       </c>
       <c r="D2022" t="n">

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:01:55
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2448"/>
+  <dimension ref="A1:D2450"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5145,7 +5145,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>138</v>
+        <v>116</v>
       </c>
     </row>
     <row r="263">
@@ -18970,7 +18970,7 @@
         </is>
       </c>
       <c r="D1030" t="n">
-        <v>138</v>
+        <v>116</v>
       </c>
     </row>
     <row r="1031">
@@ -39689,7 +39689,7 @@
         </is>
       </c>
       <c r="D2181" t="n">
-        <v>138</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2182">
@@ -41261,7 +41261,7 @@
     <row r="2269">
       <c r="A2269" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2269" t="n">
@@ -41279,7 +41279,7 @@
     <row r="2270">
       <c r="A2270" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2270" t="n">
@@ -41445,15 +41445,15 @@
         </is>
       </c>
       <c r="B2279" t="n">
-        <v>2662</v>
+        <v>2856</v>
       </c>
       <c r="C2279" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
+          <t>ALDA SOUZA ROCHA CERQUEIRA - TLV</t>
         </is>
       </c>
       <c r="D2279" t="n">
-        <v>50</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2280">
@@ -41463,15 +41463,15 @@
         </is>
       </c>
       <c r="B2280" t="n">
-        <v>2663</v>
+        <v>2662</v>
       </c>
       <c r="C2280" t="inlineStr">
         <is>
-          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
         </is>
       </c>
       <c r="D2280" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2281">
@@ -41481,15 +41481,15 @@
         </is>
       </c>
       <c r="B2281" t="n">
-        <v>2685</v>
+        <v>2663</v>
       </c>
       <c r="C2281" t="inlineStr">
         <is>
-          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
+          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
         </is>
       </c>
       <c r="D2281" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2282">
@@ -41499,15 +41499,15 @@
         </is>
       </c>
       <c r="B2282" t="n">
-        <v>2718</v>
+        <v>2685</v>
       </c>
       <c r="C2282" t="inlineStr">
         <is>
-          <t>KALILLA FERREIRA COSTA - FARMA</t>
+          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2282" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2283">
@@ -41517,15 +41517,15 @@
         </is>
       </c>
       <c r="B2283" t="n">
-        <v>2674</v>
+        <v>2718</v>
       </c>
       <c r="C2283" t="inlineStr">
         <is>
-          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
+          <t>KALILLA FERREIRA COSTA - FARMA</t>
         </is>
       </c>
       <c r="D2283" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2284">
@@ -41535,15 +41535,15 @@
         </is>
       </c>
       <c r="B2284" t="n">
-        <v>2753</v>
+        <v>2674</v>
       </c>
       <c r="C2284" t="inlineStr">
         <is>
-          <t>VAGO PATRICIA DOS S. NONATO OLIVEIRA-HB</t>
+          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
         </is>
       </c>
       <c r="D2284" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2285">
@@ -41553,15 +41553,15 @@
         </is>
       </c>
       <c r="B2285" t="n">
-        <v>2772</v>
+        <v>2753</v>
       </c>
       <c r="C2285" t="inlineStr">
         <is>
-          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
+          <t>VAGO PATRICIA DOS S. NONATO OLIVEIRA-HB</t>
         </is>
       </c>
       <c r="D2285" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2286">
@@ -41571,51 +41571,51 @@
         </is>
       </c>
       <c r="B2286" t="n">
-        <v>2827</v>
+        <v>2772</v>
       </c>
       <c r="C2286" t="inlineStr">
         <is>
-          <t>VAGO JOELTON MUNIZ DE SOUZA - HB</t>
+          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2286" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2287">
       <c r="A2287" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2287" t="n">
-        <v>2756</v>
+        <v>2827</v>
       </c>
       <c r="C2287" t="inlineStr">
         <is>
-          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
+          <t>VAGO JOELTON MUNIZ DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2287" t="n">
-        <v>39</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2288">
       <c r="A2288" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2288" t="n">
-        <v>2813</v>
+        <v>2756</v>
       </c>
       <c r="C2288" t="inlineStr">
         <is>
-          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
+          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
         </is>
       </c>
       <c r="D2288" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2289">
@@ -41625,15 +41625,15 @@
         </is>
       </c>
       <c r="B2289" t="n">
-        <v>2738</v>
+        <v>2813</v>
       </c>
       <c r="C2289" t="inlineStr">
         <is>
-          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
+          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
         </is>
       </c>
       <c r="D2289" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2290">
@@ -41643,11 +41643,11 @@
         </is>
       </c>
       <c r="B2290" t="n">
-        <v>2739</v>
+        <v>2738</v>
       </c>
       <c r="C2290" t="inlineStr">
         <is>
-          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
+          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2290" t="n">
@@ -41661,33 +41661,33 @@
         </is>
       </c>
       <c r="B2291" t="n">
-        <v>2824</v>
+        <v>2739</v>
       </c>
       <c r="C2291" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2291" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2292">
       <c r="A2292" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2292" t="n">
-        <v>2843</v>
+        <v>2824</v>
       </c>
       <c r="C2292" t="inlineStr">
         <is>
-          <t>VAGO FEIRA DE SANTANA II - FARMA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D2292" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2293">
@@ -41697,11 +41697,11 @@
         </is>
       </c>
       <c r="B2293" t="n">
-        <v>2747</v>
+        <v>2843</v>
       </c>
       <c r="C2293" t="inlineStr">
         <is>
-          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
+          <t>VAGO FEIRA DE SANTANA II - FARMA</t>
         </is>
       </c>
       <c r="D2293" t="n">
@@ -41715,11 +41715,11 @@
         </is>
       </c>
       <c r="B2294" t="n">
-        <v>2748</v>
+        <v>2747</v>
       </c>
       <c r="C2294" t="inlineStr">
         <is>
-          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
+          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
         </is>
       </c>
       <c r="D2294" t="n">
@@ -41729,73 +41729,73 @@
     <row r="2295">
       <c r="A2295" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2295" t="n">
-        <v>2766</v>
+        <v>2748</v>
       </c>
       <c r="C2295" t="inlineStr">
         <is>
-          <t>SETOR VAGO PEDREIRAS</t>
+          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
         </is>
       </c>
       <c r="D2295" t="n">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2296">
       <c r="A2296" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2296" t="n">
-        <v>2767</v>
+        <v>2766</v>
       </c>
       <c r="C2296" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>SETOR VAGO PEDREIRAS</t>
         </is>
       </c>
       <c r="D2296" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2297">
       <c r="A2297" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2297" t="n">
-        <v>2688</v>
+        <v>2767</v>
       </c>
       <c r="C2297" t="inlineStr">
         <is>
-          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D2297" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2298">
       <c r="A2298" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2298" t="n">
-        <v>2694</v>
+        <v>2688</v>
       </c>
       <c r="C2298" t="inlineStr">
         <is>
-          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
+          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2298" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2299">
@@ -41805,15 +41805,15 @@
         </is>
       </c>
       <c r="B2299" t="n">
-        <v>2714</v>
+        <v>2694</v>
       </c>
       <c r="C2299" t="inlineStr">
         <is>
-          <t>PRISCILA DOS SANTOS LOPES - HB</t>
+          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2299" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2300">
@@ -41823,15 +41823,15 @@
         </is>
       </c>
       <c r="B2300" t="n">
-        <v>2722</v>
+        <v>2714</v>
       </c>
       <c r="C2300" t="inlineStr">
         <is>
-          <t>VAGO ISALTINO BISPO DE O. JUNIOR - FARM</t>
+          <t>PRISCILA DOS SANTOS LOPES - HB</t>
         </is>
       </c>
       <c r="D2300" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2301">
@@ -41841,15 +41841,15 @@
         </is>
       </c>
       <c r="B2301" t="n">
-        <v>2723</v>
+        <v>2722</v>
       </c>
       <c r="C2301" t="inlineStr">
         <is>
-          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
+          <t>VAGO ISALTINO BISPO DE O. JUNIOR - FARM</t>
         </is>
       </c>
       <c r="D2301" t="n">
-        <v>95</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2302">
@@ -41859,15 +41859,15 @@
         </is>
       </c>
       <c r="B2302" t="n">
-        <v>2803</v>
+        <v>2723</v>
       </c>
       <c r="C2302" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
+          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2302" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2303">
@@ -41877,11 +41877,11 @@
         </is>
       </c>
       <c r="B2303" t="n">
-        <v>2804</v>
+        <v>2803</v>
       </c>
       <c r="C2303" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA - HB</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
         </is>
       </c>
       <c r="D2303" t="n">
@@ -41891,19 +41891,19 @@
     <row r="2304">
       <c r="A2304" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2304" t="n">
-        <v>2830</v>
+        <v>2804</v>
       </c>
       <c r="C2304" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 1</t>
+          <t>PAULA CARLA CALDAS MOTA - HB</t>
         </is>
       </c>
       <c r="D2304" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2305">
@@ -41913,11 +41913,11 @@
         </is>
       </c>
       <c r="B2305" t="n">
-        <v>2831</v>
+        <v>2830</v>
       </c>
       <c r="C2305" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 2</t>
+          <t>SETOR VAGO BALSAS 1</t>
         </is>
       </c>
       <c r="D2305" t="n">
@@ -41927,55 +41927,55 @@
     <row r="2306">
       <c r="A2306" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2306" t="n">
-        <v>2647</v>
+        <v>2831</v>
       </c>
       <c r="C2306" t="inlineStr">
         <is>
-          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
+          <t>SETOR VAGO BALSAS 2</t>
         </is>
       </c>
       <c r="D2306" t="n">
-        <v>148</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2307">
       <c r="A2307" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2307" t="n">
-        <v>2661</v>
+        <v>2647</v>
       </c>
       <c r="C2307" t="inlineStr">
         <is>
-          <t>MARIA ISADORA DOS REIS REGO</t>
+          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
         </is>
       </c>
       <c r="D2307" t="n">
-        <v>76</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2308">
       <c r="A2308" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2308" t="n">
-        <v>2686</v>
+        <v>2661</v>
       </c>
       <c r="C2308" t="inlineStr">
         <is>
-          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
+          <t>MARIA ISADORA DOS REIS REGO</t>
         </is>
       </c>
       <c r="D2308" t="n">
-        <v>120</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2309">
@@ -41985,11 +41985,11 @@
         </is>
       </c>
       <c r="B2309" t="n">
-        <v>2687</v>
+        <v>2686</v>
       </c>
       <c r="C2309" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
+          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2309" t="n">
@@ -41999,109 +41999,109 @@
     <row r="2310">
       <c r="A2310" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2310" t="n">
-        <v>2681</v>
+        <v>2687</v>
       </c>
       <c r="C2310" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL PI</t>
+          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
         </is>
       </c>
       <c r="D2310" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2311" t="n">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="C2311" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL MA</t>
+          <t>RCA PRINCIPIA OL PI</t>
         </is>
       </c>
       <c r="D2311" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2312">
       <c r="A2312" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2312" t="n">
-        <v>2826</v>
+        <v>2682</v>
       </c>
       <c r="C2312" t="inlineStr">
         <is>
-          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
+          <t>RCA PRINCIPIA OL MA</t>
         </is>
       </c>
       <c r="D2312" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2313">
       <c r="A2313" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2313" t="n">
-        <v>2677</v>
+        <v>2826</v>
       </c>
       <c r="C2313" t="inlineStr">
         <is>
-          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
+          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
         </is>
       </c>
       <c r="D2313" t="n">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2314">
       <c r="A2314" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2314" t="n">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="C2314" t="inlineStr">
         <is>
-          <t>ADRIEL XERXES BARROS MARTINS</t>
+          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
         </is>
       </c>
       <c r="D2314" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2315">
       <c r="A2315" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2315" t="n">
-        <v>2735</v>
+        <v>2678</v>
       </c>
       <c r="C2315" t="inlineStr">
         <is>
-          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
+          <t>ADRIEL XERXES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D2315" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2316">
@@ -42111,15 +42111,15 @@
         </is>
       </c>
       <c r="B2316" t="n">
-        <v>2736</v>
+        <v>2735</v>
       </c>
       <c r="C2316" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
+          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2316" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2317">
@@ -42129,15 +42129,15 @@
         </is>
       </c>
       <c r="B2317" t="n">
-        <v>2737</v>
+        <v>2736</v>
       </c>
       <c r="C2317" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
+          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2317" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2318">
@@ -42147,15 +42147,15 @@
         </is>
       </c>
       <c r="B2318" t="n">
-        <v>2743</v>
+        <v>2737</v>
       </c>
       <c r="C2318" t="inlineStr">
         <is>
-          <t>VAGO SEABRA - FARMA</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
         </is>
       </c>
       <c r="D2318" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2319">
@@ -42165,11 +42165,11 @@
         </is>
       </c>
       <c r="B2319" t="n">
-        <v>2744</v>
+        <v>2743</v>
       </c>
       <c r="C2319" t="inlineStr">
         <is>
-          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
+          <t>VAGO SEABRA - FARMA</t>
         </is>
       </c>
       <c r="D2319" t="n">
@@ -42183,15 +42183,15 @@
         </is>
       </c>
       <c r="B2320" t="n">
-        <v>2745</v>
+        <v>2744</v>
       </c>
       <c r="C2320" t="inlineStr">
         <is>
-          <t>CIRLANE ARAUJO SOUZA - HB</t>
+          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
         </is>
       </c>
       <c r="D2320" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2321">
@@ -42201,33 +42201,33 @@
         </is>
       </c>
       <c r="B2321" t="n">
-        <v>2783</v>
+        <v>2745</v>
       </c>
       <c r="C2321" t="inlineStr">
         <is>
-          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
+          <t>CIRLANE ARAUJO SOUZA - HB</t>
         </is>
       </c>
       <c r="D2321" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2322">
       <c r="A2322" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2322" t="n">
-        <v>2852</v>
+        <v>2783</v>
       </c>
       <c r="C2322" t="inlineStr">
         <is>
-          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2322" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2323">
@@ -42237,11 +42237,11 @@
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2768</v>
+        <v>2852</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
         </is>
       </c>
       <c r="D2323" t="n">
@@ -42251,73 +42251,73 @@
     <row r="2324">
       <c r="A2324" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2703</v>
+        <v>2768</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2324" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2325">
       <c r="A2325" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2828</v>
+        <v>2703</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>LYERKA MARDANIA RODRIGUES MELO</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2325" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2326">
       <c r="A2326" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2750</v>
+        <v>2828</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>LYERKA MARDANIA RODRIGUES MELO</t>
         </is>
       </c>
       <c r="D2326" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2327">
       <c r="A2327" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2689</v>
+        <v>2750</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2327" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2328">
@@ -42327,69 +42327,69 @@
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2708</v>
+        <v>2689</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2328" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2709</v>
+        <v>2708</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2329" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2330">
       <c r="A2330" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2789</v>
+        <v>2709</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>BRUNO TEIXEIRA TORRES</t>
         </is>
       </c>
       <c r="D2330" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2331">
       <c r="A2331" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2790</v>
+        <v>2789</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>VAGO STA INES 01 HNB</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2331" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2332">
@@ -42399,11 +42399,11 @@
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2791</v>
+        <v>2790</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>DANIELY SLZ 01</t>
+          <t>VAGO STA INES 01 HNB</t>
         </is>
       </c>
       <c r="D2332" t="n">
@@ -42413,19 +42413,19 @@
     <row r="2333">
       <c r="A2333" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2805</v>
+        <v>2791</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>DANIELY SLZ 01</t>
         </is>
       </c>
       <c r="D2333" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2334">
@@ -42435,11 +42435,11 @@
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2806</v>
+        <v>2805</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2334" t="n">
@@ -42453,11 +42453,11 @@
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2807</v>
+        <v>2806</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2335" t="n">
@@ -42471,11 +42471,11 @@
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2808</v>
+        <v>2807</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2336" t="n">
@@ -42485,73 +42485,73 @@
     <row r="2337">
       <c r="A2337" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2820</v>
+        <v>2808</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2337" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2338">
       <c r="A2338" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2851</v>
+        <v>2820</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2338" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2339">
       <c r="A2339" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2765</v>
+        <v>2851</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2339" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2842</v>
+        <v>2765</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2341">
@@ -42561,33 +42561,33 @@
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2741</v>
+        <v>2842</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D2341" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2342">
       <c r="A2342" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2758</v>
+        <v>2741</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2343">
@@ -42597,11 +42597,11 @@
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2854</v>
+        <v>2758</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>JONILSON SANTANA SANTOS - FARMA</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2343" t="n">
@@ -42615,51 +42615,51 @@
         </is>
       </c>
       <c r="B2344" t="n">
-        <v>2659</v>
+        <v>2854</v>
       </c>
       <c r="C2344" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>JONILSON SANTANA SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2344" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2345">
       <c r="A2345" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2345" t="n">
-        <v>2669</v>
+        <v>2659</v>
       </c>
       <c r="C2345" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2345" t="n">
-        <v>135</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2346">
       <c r="A2346" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2346" t="n">
-        <v>2672</v>
+        <v>2669</v>
       </c>
       <c r="C2346" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2346" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2347">
@@ -42669,11 +42669,11 @@
         </is>
       </c>
       <c r="B2347" t="n">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="C2347" t="inlineStr">
         <is>
-          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2347" t="n">
@@ -42683,19 +42683,19 @@
     <row r="2348">
       <c r="A2348" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2676</v>
+        <v>2673</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2348" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2349">
@@ -42705,33 +42705,33 @@
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2760</v>
+        <v>2676</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2349" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2350">
       <c r="A2350" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2823</v>
+        <v>2760</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2350" t="n">
-        <v>80</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2351">
@@ -42741,29 +42741,29 @@
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2848</v>
+        <v>2823</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2351" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2352">
       <c r="A2352" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2792</v>
+        <v>2848</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2352" t="n">
@@ -42773,19 +42773,19 @@
     <row r="2353">
       <c r="A2353" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2793</v>
+        <v>2792</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2353" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2354">
@@ -42795,15 +42795,15 @@
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2802</v>
+        <v>2793</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2354" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2355">
@@ -42813,47 +42813,47 @@
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2656</v>
+        <v>2802</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2355" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2356">
       <c r="A2356" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2657</v>
+        <v>2656</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA IMP 01 HNB</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2356" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>MARIA APARECIDA IMP 01 HNB</t>
         </is>
       </c>
       <c r="D2357" t="n">
@@ -42863,37 +42863,37 @@
     <row r="2358">
       <c r="A2358" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2729</v>
+        <v>2658</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2358" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2359">
       <c r="A2359" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2759</v>
+        <v>2729</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2359" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2360">
@@ -42903,15 +42903,15 @@
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2832</v>
+        <v>2759</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2361">
@@ -42921,33 +42921,33 @@
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2769</v>
+        <v>2832</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
         </is>
       </c>
       <c r="D2361" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2362">
       <c r="A2362" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2679</v>
+        <v>2769</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2362" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2363">
@@ -42957,11 +42957,11 @@
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2363" t="n">
@@ -42971,19 +42971,19 @@
     <row r="2364">
       <c r="A2364" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2815</v>
+        <v>2680</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2364" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2365">
@@ -42993,15 +42993,15 @@
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2816</v>
+        <v>2815</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2365" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2366">
@@ -43011,11 +43011,11 @@
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2817</v>
+        <v>2816</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2366" t="n">
@@ -43025,37 +43025,37 @@
     <row r="2367">
       <c r="A2367" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2841</v>
+        <v>2817</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>46</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2368">
       <c r="A2368" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2701</v>
+        <v>2841</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
         </is>
       </c>
       <c r="D2368" t="n">
-        <v>90</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2369">
@@ -43065,29 +43065,29 @@
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2644</v>
+        <v>2701</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2369" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2370">
       <c r="A2370" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2645</v>
+        <v>2644</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2370" t="n">
@@ -43101,15 +43101,15 @@
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2754</v>
+        <v>2645</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2372">
@@ -43119,33 +43119,33 @@
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2755</v>
+        <v>2754</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2372" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2373">
       <c r="A2373" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2665</v>
+        <v>2755</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>141</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2374">
@@ -43155,15 +43155,15 @@
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2667</v>
+        <v>2665</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>VAGO AÇAILÂNDIA HNB</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>114</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2375">
@@ -43173,15 +43173,15 @@
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2727</v>
+        <v>2667</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>VAGO AÇAILÂNDIA HNB</t>
         </is>
       </c>
       <c r="D2375" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2376">
@@ -43191,11 +43191,11 @@
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2728</v>
+        <v>2727</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2376" t="n">
@@ -43205,55 +43205,55 @@
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2833</v>
+        <v>2728</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>ADEILZA PINTO DA SILVA - FARMA</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2377" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2378">
       <c r="A2378" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2814</v>
+        <v>2833</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>ADEILZA PINTO DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>39</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2379">
       <c r="A2379" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2646</v>
+        <v>2814</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2379" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2380">
@@ -43263,15 +43263,15 @@
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2650</v>
+        <v>2855</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>DESIREE BARROS DE CARVALHO - CCM</t>
         </is>
       </c>
       <c r="D2380" t="n">
-        <v>95</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2381">
@@ -43281,15 +43281,15 @@
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2652</v>
+        <v>2646</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2382">
@@ -43299,11 +43299,11 @@
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2653</v>
+        <v>2650</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2382" t="n">
@@ -43317,15 +43317,15 @@
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2654</v>
+        <v>2652</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2384">
@@ -43335,33 +43335,33 @@
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2655</v>
+        <v>2653</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2385">
       <c r="A2385" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2821</v>
+        <v>2654</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2385" t="n">
-        <v>69</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2386">
@@ -43371,231 +43371,231 @@
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2683</v>
+        <v>2655</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2387">
       <c r="A2387" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2684</v>
+        <v>2821</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2749</v>
+        <v>2683</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>111</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2389">
       <c r="A2389" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2812</v>
+        <v>2684</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>145</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2715</v>
+        <v>2749</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>90</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2834</v>
+        <v>2812</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>GILVANA MONTELES U. SANTOS HNB</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>114</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2651</v>
+        <v>2715</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>145</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2819</v>
+        <v>2834</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>GILVANA MONTELES U. SANTOS HNB</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2394">
       <c r="A2394" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2849</v>
+        <v>2651</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>MULTI PE (PEDRO HENRIQUE VIERA)</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>72</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2835</v>
+        <v>2819</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>ROGÉRIO LIRA DA GAMA</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>116</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2396">
       <c r="A2396" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2699</v>
+        <v>2849</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>MULTI PE (PEDRO HENRIQUE VIERA)</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>95</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2397">
       <c r="A2397" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2706</v>
+        <v>2835</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>VAGO BARREIRINHAS HNB</t>
+          <t>ROGÉRIO LIRA DA GAMA</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2707</v>
+        <v>2699</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>VAGO BACABAL HNB</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2399">
@@ -43605,15 +43605,15 @@
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2846</v>
+        <v>2706</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>VAGO BARREIRINHAS HNB</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2400">
@@ -43623,87 +43623,87 @@
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2847</v>
+        <v>2707</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>WERBERTTY</t>
+          <t>VAGO BACABAL HNB</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2401">
       <c r="A2401" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2693</v>
+        <v>2846</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2402">
       <c r="A2402" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2705</v>
+        <v>2847</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>FRANCISCO WERBERTTY DA SILVA MORAIS</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>146</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2403">
       <c r="A2403" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2664</v>
+        <v>2693</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2404">
       <c r="A2404" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2670</v>
+        <v>2705</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>69</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2405">
@@ -43713,195 +43713,195 @@
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2730</v>
+        <v>2664</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2671</v>
+        <v>2670</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2407">
       <c r="A2407" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2691</v>
+        <v>2730</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2692</v>
+        <v>2671</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2724</v>
+        <v>2691</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2410">
       <c r="A2410" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2773</v>
+        <v>2692</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>TIMON 01 HNB</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2410" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2411">
       <c r="A2411" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2844</v>
+        <v>2724</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>132</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2412">
       <c r="A2412" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2845</v>
+        <v>2773</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
+          <t>TIMON 01 HNB</t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>132</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2413">
       <c r="A2413" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2825</v>
+        <v>2844</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>90</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2414">
       <c r="A2414" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2787</v>
+        <v>2845</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>120</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2415">
       <c r="A2415" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2839</v>
+        <v>2825</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>RCA TENA OL PI</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2415" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2416">
@@ -43911,69 +43911,69 @@
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2840</v>
+        <v>2787</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>RCA TENA OL MA</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2416" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2417">
       <c r="A2417" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2648</v>
+        <v>2839</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>RCA TENA OL PI</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2418">
       <c r="A2418" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2666</v>
+        <v>2840</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>RCA TENA OL MA</t>
         </is>
       </c>
       <c r="D2418" t="n">
-        <v>63</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2419">
       <c r="A2419" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2779</v>
+        <v>2648</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2419" t="n">
-        <v>105</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2420">
@@ -43983,15 +43983,15 @@
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2780</v>
+        <v>2666</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2421">
@@ -44001,51 +44001,51 @@
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2786</v>
+        <v>2779</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO - TLV</t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2422">
       <c r="A2422" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2660</v>
+        <v>2780</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>38</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2423">
       <c r="A2423" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2716</v>
+        <v>2786</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2424">
@@ -44055,51 +44055,51 @@
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2734</v>
+        <v>2660</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2424" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2425">
       <c r="A2425" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2853</v>
+        <v>2716</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>H-ROBERTO SOARES OLIVEIRA JUNIOR</t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2425" t="n">
-        <v>53</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2426">
       <c r="A2426" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2742</v>
+        <v>2734</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS - FARMA JACOBINA</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2426" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2427">
@@ -44109,15 +44109,15 @@
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2794</v>
+        <v>2853</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>VAGO DEISIELLE J. SILVA - HB JACOBINA</t>
+          <t>H-ROBERTO SOARES OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2427" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2428">
@@ -44127,11 +44127,11 @@
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2795</v>
+        <v>2742</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
+          <t>VAGO MARCUS VINICIUS - FARMA JACOBINA</t>
         </is>
       </c>
       <c r="D2428" t="n">
@@ -44145,15 +44145,15 @@
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2796</v>
+        <v>2794</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VAGO DEISIELLE J. SILVA - HB JACOBINA</t>
         </is>
       </c>
       <c r="D2429" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2430">
@@ -44163,11 +44163,11 @@
         </is>
       </c>
       <c r="B2430" t="n">
-        <v>2797</v>
+        <v>2795</v>
       </c>
       <c r="C2430" t="inlineStr">
         <is>
-          <t>VAGO ESDRAS A. SANTOS-FAR (PAULO AFO)</t>
+          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
         </is>
       </c>
       <c r="D2430" t="n">
@@ -44181,11 +44181,11 @@
         </is>
       </c>
       <c r="B2431" t="n">
-        <v>2798</v>
+        <v>2796</v>
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2431" t="n">
@@ -44195,73 +44195,73 @@
     <row r="2432">
       <c r="A2432" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2432" t="n">
-        <v>2668</v>
+        <v>2797</v>
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>VAGO ESDRAS A. SANTOS-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2432" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2433">
       <c r="A2433" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2433" t="n">
-        <v>2690</v>
+        <v>2798</v>
       </c>
       <c r="C2433" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2433" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2434">
       <c r="A2434" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2434" t="n">
-        <v>2696</v>
+        <v>2668</v>
       </c>
       <c r="C2434" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2434" t="n">
-        <v>69</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2435">
       <c r="A2435" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2435" t="n">
-        <v>2697</v>
+        <v>2690</v>
       </c>
       <c r="C2435" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2435" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2436">
@@ -44271,11 +44271,11 @@
         </is>
       </c>
       <c r="B2436" t="n">
-        <v>2698</v>
+        <v>2696</v>
       </c>
       <c r="C2436" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2436" t="n">
@@ -44285,37 +44285,37 @@
     <row r="2437">
       <c r="A2437" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2437" t="n">
-        <v>2775</v>
+        <v>2697</v>
       </c>
       <c r="C2437" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2437" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2438">
       <c r="A2438" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2438" t="n">
-        <v>2776</v>
+        <v>2698</v>
       </c>
       <c r="C2438" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2438" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2439">
@@ -44325,11 +44325,11 @@
         </is>
       </c>
       <c r="B2439" t="n">
-        <v>2777</v>
+        <v>2775</v>
       </c>
       <c r="C2439" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2439" t="n">
@@ -44343,11 +44343,11 @@
         </is>
       </c>
       <c r="B2440" t="n">
-        <v>2778</v>
+        <v>2776</v>
       </c>
       <c r="C2440" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2440" t="n">
@@ -44361,15 +44361,15 @@
         </is>
       </c>
       <c r="B2441" t="n">
-        <v>2781</v>
+        <v>2777</v>
       </c>
       <c r="C2441" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2441" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2442">
@@ -44379,11 +44379,11 @@
         </is>
       </c>
       <c r="B2442" t="n">
-        <v>2822</v>
+        <v>2778</v>
       </c>
       <c r="C2442" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2442" t="n">
@@ -44397,87 +44397,87 @@
         </is>
       </c>
       <c r="B2443" t="n">
-        <v>2740</v>
+        <v>2781</v>
       </c>
       <c r="C2443" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2443" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2444">
       <c r="A2444" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2444" t="n">
-        <v>2710</v>
+        <v>2822</v>
       </c>
       <c r="C2444" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2444" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2445">
       <c r="A2445" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2445" t="n">
-        <v>2711</v>
+        <v>2740</v>
       </c>
       <c r="C2445" t="inlineStr">
         <is>
-          <t>CARLOS CHAPADINHA</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2445" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2446">
       <c r="A2446" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2446" t="n">
-        <v>2712</v>
+        <v>2710</v>
       </c>
       <c r="C2446" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2446" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2447">
       <c r="A2447" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2447" t="n">
-        <v>2717</v>
+        <v>2711</v>
       </c>
       <c r="C2447" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>CARLOS CHAPADINHA</t>
         </is>
       </c>
       <c r="D2447" t="n">
-        <v>69</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2448">
@@ -44487,14 +44487,50 @@
         </is>
       </c>
       <c r="B2448" t="n">
+        <v>2712</v>
+      </c>
+      <c r="C2448" t="inlineStr">
+        <is>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
+        </is>
+      </c>
+      <c r="D2448" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2449">
+      <c r="A2449" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2449" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2449" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2449" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2450">
+      <c r="A2450" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2450" t="n">
         <v>2801</v>
       </c>
-      <c r="C2448" t="inlineStr">
+      <c r="C2450" t="inlineStr">
         <is>
           <t>SETOR VAGO VIANA FARMA</t>
         </is>
       </c>
-      <c r="D2448" t="n">
+      <c r="D2450" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:01:27
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2450"/>
+  <dimension ref="A1:D2451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42017,109 +42017,109 @@
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2311" t="n">
-        <v>2681</v>
+        <v>2857</v>
       </c>
       <c r="C2311" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL PI</t>
+          <t>H-VALQUIRIO OLIVEIRA SOUSA</t>
         </is>
       </c>
       <c r="D2311" t="n">
-        <v>69</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2312">
       <c r="A2312" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2312" t="n">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="C2312" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL MA</t>
+          <t>RCA PRINCIPIA OL PI</t>
         </is>
       </c>
       <c r="D2312" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2313">
       <c r="A2313" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2313" t="n">
-        <v>2826</v>
+        <v>2682</v>
       </c>
       <c r="C2313" t="inlineStr">
         <is>
-          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
+          <t>RCA PRINCIPIA OL MA</t>
         </is>
       </c>
       <c r="D2313" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2314">
       <c r="A2314" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2314" t="n">
-        <v>2677</v>
+        <v>2826</v>
       </c>
       <c r="C2314" t="inlineStr">
         <is>
-          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
+          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
         </is>
       </c>
       <c r="D2314" t="n">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2315">
       <c r="A2315" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2315" t="n">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="C2315" t="inlineStr">
         <is>
-          <t>ADRIEL XERXES BARROS MARTINS</t>
+          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
         </is>
       </c>
       <c r="D2315" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2316">
       <c r="A2316" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2316" t="n">
-        <v>2735</v>
+        <v>2678</v>
       </c>
       <c r="C2316" t="inlineStr">
         <is>
-          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
+          <t>ADRIEL XERXES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D2316" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2317">
@@ -42129,15 +42129,15 @@
         </is>
       </c>
       <c r="B2317" t="n">
-        <v>2736</v>
+        <v>2735</v>
       </c>
       <c r="C2317" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
+          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2317" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2318">
@@ -42147,15 +42147,15 @@
         </is>
       </c>
       <c r="B2318" t="n">
-        <v>2737</v>
+        <v>2736</v>
       </c>
       <c r="C2318" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
+          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2318" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2319">
@@ -42165,15 +42165,15 @@
         </is>
       </c>
       <c r="B2319" t="n">
-        <v>2743</v>
+        <v>2737</v>
       </c>
       <c r="C2319" t="inlineStr">
         <is>
-          <t>VAGO SEABRA - FARMA</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
         </is>
       </c>
       <c r="D2319" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2320">
@@ -42183,11 +42183,11 @@
         </is>
       </c>
       <c r="B2320" t="n">
-        <v>2744</v>
+        <v>2743</v>
       </c>
       <c r="C2320" t="inlineStr">
         <is>
-          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
+          <t>VAGO SEABRA - FARMA</t>
         </is>
       </c>
       <c r="D2320" t="n">
@@ -42201,15 +42201,15 @@
         </is>
       </c>
       <c r="B2321" t="n">
-        <v>2745</v>
+        <v>2744</v>
       </c>
       <c r="C2321" t="inlineStr">
         <is>
-          <t>CIRLANE ARAUJO SOUZA - HB</t>
+          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
         </is>
       </c>
       <c r="D2321" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2322">
@@ -42219,33 +42219,33 @@
         </is>
       </c>
       <c r="B2322" t="n">
-        <v>2783</v>
+        <v>2745</v>
       </c>
       <c r="C2322" t="inlineStr">
         <is>
-          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
+          <t>CIRLANE ARAUJO SOUZA - HB</t>
         </is>
       </c>
       <c r="D2322" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2323">
       <c r="A2323" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2852</v>
+        <v>2783</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2323" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2324">
@@ -42255,11 +42255,11 @@
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2768</v>
+        <v>2852</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
         </is>
       </c>
       <c r="D2324" t="n">
@@ -42269,73 +42269,73 @@
     <row r="2325">
       <c r="A2325" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2703</v>
+        <v>2768</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2325" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2326">
       <c r="A2326" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2828</v>
+        <v>2703</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>LYERKA MARDANIA RODRIGUES MELO</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2326" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2327">
       <c r="A2327" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2750</v>
+        <v>2828</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>LYERKA MARDANIA RODRIGUES MELO</t>
         </is>
       </c>
       <c r="D2327" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2328">
       <c r="A2328" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2689</v>
+        <v>2750</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2328" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2329">
@@ -42345,69 +42345,69 @@
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2708</v>
+        <v>2689</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2329" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2330">
       <c r="A2330" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2709</v>
+        <v>2708</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2330" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2331">
       <c r="A2331" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2789</v>
+        <v>2709</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>BRUNO TEIXEIRA TORRES</t>
         </is>
       </c>
       <c r="D2331" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2332">
       <c r="A2332" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2790</v>
+        <v>2789</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>VAGO STA INES 01 HNB</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2332" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2333">
@@ -42417,11 +42417,11 @@
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2791</v>
+        <v>2790</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>DANIELY SLZ 01</t>
+          <t>VAGO STA INES 01 HNB</t>
         </is>
       </c>
       <c r="D2333" t="n">
@@ -42431,19 +42431,19 @@
     <row r="2334">
       <c r="A2334" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2805</v>
+        <v>2791</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>DANIELY SLZ 01</t>
         </is>
       </c>
       <c r="D2334" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2335">
@@ -42453,11 +42453,11 @@
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2806</v>
+        <v>2805</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2335" t="n">
@@ -42471,11 +42471,11 @@
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2807</v>
+        <v>2806</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2336" t="n">
@@ -42489,11 +42489,11 @@
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2808</v>
+        <v>2807</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2337" t="n">
@@ -42503,73 +42503,73 @@
     <row r="2338">
       <c r="A2338" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2820</v>
+        <v>2808</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2338" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2339">
       <c r="A2339" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2851</v>
+        <v>2820</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2339" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2765</v>
+        <v>2851</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2341">
       <c r="A2341" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2842</v>
+        <v>2765</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2341" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2342">
@@ -42579,33 +42579,33 @@
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2741</v>
+        <v>2842</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2343">
       <c r="A2343" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2758</v>
+        <v>2741</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2343" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2344">
@@ -42615,11 +42615,11 @@
         </is>
       </c>
       <c r="B2344" t="n">
-        <v>2854</v>
+        <v>2758</v>
       </c>
       <c r="C2344" t="inlineStr">
         <is>
-          <t>JONILSON SANTANA SANTOS - FARMA</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2344" t="n">
@@ -42633,51 +42633,51 @@
         </is>
       </c>
       <c r="B2345" t="n">
-        <v>2659</v>
+        <v>2854</v>
       </c>
       <c r="C2345" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>JONILSON SANTANA SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2345" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2346">
       <c r="A2346" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2346" t="n">
-        <v>2669</v>
+        <v>2659</v>
       </c>
       <c r="C2346" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2346" t="n">
-        <v>135</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2347">
       <c r="A2347" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2347" t="n">
-        <v>2672</v>
+        <v>2669</v>
       </c>
       <c r="C2347" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2347" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2348">
@@ -42687,11 +42687,11 @@
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2348" t="n">
@@ -42701,19 +42701,19 @@
     <row r="2349">
       <c r="A2349" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2676</v>
+        <v>2673</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2349" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2350">
@@ -42723,33 +42723,33 @@
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2760</v>
+        <v>2676</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2350" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2351">
       <c r="A2351" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2823</v>
+        <v>2760</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2351" t="n">
-        <v>80</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2352">
@@ -42759,29 +42759,29 @@
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2848</v>
+        <v>2823</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2352" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2353">
       <c r="A2353" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2792</v>
+        <v>2848</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2353" t="n">
@@ -42791,19 +42791,19 @@
     <row r="2354">
       <c r="A2354" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2793</v>
+        <v>2792</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2354" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2355">
@@ -42813,15 +42813,15 @@
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2802</v>
+        <v>2793</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2355" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2356">
@@ -42831,47 +42831,47 @@
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2656</v>
+        <v>2802</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2356" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2657</v>
+        <v>2656</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA IMP 01 HNB</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2357" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2358">
       <c r="A2358" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>MARIA APARECIDA IMP 01 HNB</t>
         </is>
       </c>
       <c r="D2358" t="n">
@@ -42881,37 +42881,37 @@
     <row r="2359">
       <c r="A2359" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2729</v>
+        <v>2658</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2359" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2360">
       <c r="A2360" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2759</v>
+        <v>2729</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2361">
@@ -42921,15 +42921,15 @@
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2832</v>
+        <v>2759</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2361" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2362">
@@ -42939,33 +42939,33 @@
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2769</v>
+        <v>2832</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
         </is>
       </c>
       <c r="D2362" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2363">
       <c r="A2363" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2679</v>
+        <v>2769</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2363" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2364">
@@ -42975,11 +42975,11 @@
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2364" t="n">
@@ -42989,19 +42989,19 @@
     <row r="2365">
       <c r="A2365" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2815</v>
+        <v>2680</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2365" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2366">
@@ -43011,15 +43011,15 @@
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2816</v>
+        <v>2815</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2366" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2367">
@@ -43029,11 +43029,11 @@
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2817</v>
+        <v>2816</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2367" t="n">
@@ -43043,37 +43043,37 @@
     <row r="2368">
       <c r="A2368" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2841</v>
+        <v>2817</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2368" t="n">
-        <v>46</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2369">
       <c r="A2369" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2701</v>
+        <v>2841</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
         </is>
       </c>
       <c r="D2369" t="n">
-        <v>90</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2370">
@@ -43083,29 +43083,29 @@
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2644</v>
+        <v>2701</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2645</v>
+        <v>2644</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2371" t="n">
@@ -43119,15 +43119,15 @@
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2754</v>
+        <v>2645</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2372" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2373">
@@ -43137,33 +43137,33 @@
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2755</v>
+        <v>2754</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2374">
       <c r="A2374" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2665</v>
+        <v>2755</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>141</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2375">
@@ -43173,15 +43173,15 @@
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2667</v>
+        <v>2665</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>VAGO AÇAILÂNDIA HNB</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2375" t="n">
-        <v>114</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2376">
@@ -43191,15 +43191,15 @@
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2727</v>
+        <v>2667</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>VAGO AÇAILÂNDIA HNB</t>
         </is>
       </c>
       <c r="D2376" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2377">
@@ -43209,11 +43209,11 @@
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2728</v>
+        <v>2727</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2377" t="n">
@@ -43223,55 +43223,55 @@
     <row r="2378">
       <c r="A2378" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2833</v>
+        <v>2728</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>ADEILZA PINTO DA SILVA - FARMA</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2379">
       <c r="A2379" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2814</v>
+        <v>2833</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>ADEILZA PINTO DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2379" t="n">
-        <v>39</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2380">
       <c r="A2380" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2855</v>
+        <v>2814</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>DESIREE BARROS DE CARVALHO - CCM</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2380" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2381">
@@ -43281,15 +43281,15 @@
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2646</v>
+        <v>2855</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>DESIREE BARROS DE CARVALHO - CCM</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>95</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2382">
@@ -43299,11 +43299,11 @@
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2650</v>
+        <v>2646</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2382" t="n">
@@ -43317,15 +43317,15 @@
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2652</v>
+        <v>2650</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2384">
@@ -43335,15 +43335,15 @@
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2385">
@@ -43353,15 +43353,15 @@
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2654</v>
+        <v>2653</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2385" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2386">
@@ -43371,51 +43371,51 @@
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2655</v>
+        <v>2654</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2387">
       <c r="A2387" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2821</v>
+        <v>2655</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>69</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2683</v>
+        <v>2821</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2389">
@@ -43425,33 +43425,33 @@
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2749</v>
+        <v>2684</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2391">
@@ -43461,33 +43461,33 @@
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2812</v>
+        <v>2749</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>145</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2715</v>
+        <v>2812</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>90</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2393">
@@ -43497,123 +43497,123 @@
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2834</v>
+        <v>2715</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>GILVANA MONTELES U. SANTOS HNB</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2394">
       <c r="A2394" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2651</v>
+        <v>2834</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>GILVANA MONTELES U. SANTOS HNB</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>145</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2819</v>
+        <v>2651</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2396">
       <c r="A2396" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2849</v>
+        <v>2819</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>MULTI PE (PEDRO HENRIQUE VIERA)</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2397">
       <c r="A2397" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2835</v>
+        <v>2849</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>ROGÉRIO LIRA DA GAMA</t>
+          <t>MULTI PE (PEDRO HENRIQUE VIERA)</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>116</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2699</v>
+        <v>2835</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>ROGÉRIO LIRA DA GAMA</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>95</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2706</v>
+        <v>2699</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>VAGO BARREIRINHAS HNB</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2400">
@@ -43623,11 +43623,11 @@
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2707</v>
+        <v>2706</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>VAGO BACABAL HNB</t>
+          <t>VAGO BARREIRINHAS HNB</t>
         </is>
       </c>
       <c r="D2400" t="n">
@@ -43641,15 +43641,15 @@
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2846</v>
+        <v>2707</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>VAGO BACABAL HNB</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2402">
@@ -43659,11 +43659,11 @@
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2847</v>
+        <v>2846</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>FRANCISCO WERBERTTY DA SILVA MORAIS</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D2402" t="n">
@@ -43673,127 +43673,127 @@
     <row r="2403">
       <c r="A2403" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2693</v>
+        <v>2847</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>FRANCISCO WERBERTTY DA SILVA MORAIS</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2404">
       <c r="A2404" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2705</v>
+        <v>2693</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>146</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2405">
       <c r="A2405" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2664</v>
+        <v>2705</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>90</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2670</v>
+        <v>2664</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2407">
       <c r="A2407" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2730</v>
+        <v>2670</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2671</v>
+        <v>2730</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2691</v>
+        <v>2671</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2410">
@@ -43803,11 +43803,11 @@
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2410" t="n">
@@ -43817,55 +43817,55 @@
     <row r="2411">
       <c r="A2411" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2724</v>
+        <v>2692</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2412">
       <c r="A2412" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2773</v>
+        <v>2724</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>TIMON 01 HNB</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2413">
       <c r="A2413" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2844</v>
+        <v>2773</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
+          <t>TIMON 01 HNB</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>132</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2414">
@@ -43875,11 +43875,11 @@
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2845</v>
+        <v>2844</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
+          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
         </is>
       </c>
       <c r="D2414" t="n">
@@ -43889,19 +43889,19 @@
     <row r="2415">
       <c r="A2415" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2825</v>
+        <v>2845</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
         </is>
       </c>
       <c r="D2415" t="n">
-        <v>90</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2416">
@@ -43911,51 +43911,51 @@
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2787</v>
+        <v>2825</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2416" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2417">
       <c r="A2417" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2839</v>
+        <v>2787</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>RCA TENA OL PI</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2418">
       <c r="A2418" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2840</v>
+        <v>2839</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>RCA TENA OL MA</t>
+          <t>RCA TENA OL PI</t>
         </is>
       </c>
       <c r="D2418" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2419">
@@ -43965,33 +43965,33 @@
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2648</v>
+        <v>2840</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>RCA TENA OL MA</t>
         </is>
       </c>
       <c r="D2419" t="n">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2420">
       <c r="A2420" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2666</v>
+        <v>2648</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>63</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2421">
@@ -44001,15 +44001,15 @@
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2779</v>
+        <v>2666</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO - TLV</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2422">
@@ -44019,11 +44019,11 @@
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2780</v>
+        <v>2779</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO - TLV</t>
         </is>
       </c>
       <c r="D2422" t="n">
@@ -44037,33 +44037,33 @@
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2786</v>
+        <v>2780</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2424">
       <c r="A2424" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2660</v>
+        <v>2786</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2424" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2425">
@@ -44073,15 +44073,15 @@
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2716</v>
+        <v>2660</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2425" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2426">
@@ -44091,11 +44091,11 @@
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2734</v>
+        <v>2716</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2426" t="n">
@@ -44105,19 +44105,19 @@
     <row r="2427">
       <c r="A2427" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2853</v>
+        <v>2734</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>H-ROBERTO SOARES OLIVEIRA JUNIOR</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2427" t="n">
-        <v>53</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2428">
@@ -44127,15 +44127,15 @@
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2742</v>
+        <v>2853</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS - FARMA JACOBINA</t>
+          <t>H-ROBERTO SOARES OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2428" t="n">
-        <v>95</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2429">
@@ -44145,15 +44145,15 @@
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2794</v>
+        <v>2742</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>VAGO DEISIELLE J. SILVA - HB JACOBINA</t>
+          <t>VAGO MARCUS VINICIUS - FARMA JACOBINA</t>
         </is>
       </c>
       <c r="D2429" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2430">
@@ -44163,15 +44163,15 @@
         </is>
       </c>
       <c r="B2430" t="n">
-        <v>2795</v>
+        <v>2794</v>
       </c>
       <c r="C2430" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
+          <t>VAGO DEISIELLE J. SILVA - HB JACOBINA</t>
         </is>
       </c>
       <c r="D2430" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2431">
@@ -44181,11 +44181,11 @@
         </is>
       </c>
       <c r="B2431" t="n">
-        <v>2796</v>
+        <v>2795</v>
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
         </is>
       </c>
       <c r="D2431" t="n">
@@ -44199,11 +44199,11 @@
         </is>
       </c>
       <c r="B2432" t="n">
-        <v>2797</v>
+        <v>2796</v>
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>VAGO ESDRAS A. SANTOS-FAR (PAULO AFO)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2432" t="n">
@@ -44217,11 +44217,11 @@
         </is>
       </c>
       <c r="B2433" t="n">
-        <v>2798</v>
+        <v>2797</v>
       </c>
       <c r="C2433" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>VAGO ESDRAS A. SANTOS-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2433" t="n">
@@ -44231,55 +44231,55 @@
     <row r="2434">
       <c r="A2434" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2434" t="n">
-        <v>2668</v>
+        <v>2798</v>
       </c>
       <c r="C2434" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2434" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2435">
       <c r="A2435" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2435" t="n">
-        <v>2690</v>
+        <v>2668</v>
       </c>
       <c r="C2435" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2435" t="n">
-        <v>38</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2436">
       <c r="A2436" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2436" t="n">
-        <v>2696</v>
+        <v>2690</v>
       </c>
       <c r="C2436" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2436" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2437">
@@ -44289,11 +44289,11 @@
         </is>
       </c>
       <c r="B2437" t="n">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="C2437" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2437" t="n">
@@ -44307,11 +44307,11 @@
         </is>
       </c>
       <c r="B2438" t="n">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="C2438" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2438" t="n">
@@ -44321,19 +44321,19 @@
     <row r="2439">
       <c r="A2439" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2439" t="n">
-        <v>2775</v>
+        <v>2698</v>
       </c>
       <c r="C2439" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2439" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2440">
@@ -44343,11 +44343,11 @@
         </is>
       </c>
       <c r="B2440" t="n">
-        <v>2776</v>
+        <v>2775</v>
       </c>
       <c r="C2440" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2440" t="n">
@@ -44361,11 +44361,11 @@
         </is>
       </c>
       <c r="B2441" t="n">
-        <v>2777</v>
+        <v>2776</v>
       </c>
       <c r="C2441" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2441" t="n">
@@ -44379,11 +44379,11 @@
         </is>
       </c>
       <c r="B2442" t="n">
-        <v>2778</v>
+        <v>2777</v>
       </c>
       <c r="C2442" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2442" t="n">
@@ -44397,15 +44397,15 @@
         </is>
       </c>
       <c r="B2443" t="n">
-        <v>2781</v>
+        <v>2778</v>
       </c>
       <c r="C2443" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2443" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2444">
@@ -44415,15 +44415,15 @@
         </is>
       </c>
       <c r="B2444" t="n">
-        <v>2822</v>
+        <v>2781</v>
       </c>
       <c r="C2444" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2444" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2445">
@@ -44433,11 +44433,11 @@
         </is>
       </c>
       <c r="B2445" t="n">
-        <v>2740</v>
+        <v>2822</v>
       </c>
       <c r="C2445" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2445" t="n">
@@ -44447,90 +44447,108 @@
     <row r="2446">
       <c r="A2446" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2446" t="n">
-        <v>2710</v>
+        <v>2740</v>
       </c>
       <c r="C2446" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2446" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2447">
       <c r="A2447" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2447" t="n">
-        <v>2711</v>
+        <v>2710</v>
       </c>
       <c r="C2447" t="inlineStr">
         <is>
-          <t>CARLOS CHAPADINHA</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2447" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2448">
       <c r="A2448" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2448" t="n">
-        <v>2712</v>
+        <v>2711</v>
       </c>
       <c r="C2448" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>CARLOS CHAPADINHA</t>
         </is>
       </c>
       <c r="D2448" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2449">
       <c r="A2449" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2449" t="n">
-        <v>2717</v>
+        <v>2712</v>
       </c>
       <c r="C2449" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
         </is>
       </c>
       <c r="D2449" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2450">
       <c r="A2450" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2450" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2450" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2450" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2451">
+      <c r="A2451" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2451" t="n">
         <v>2801</v>
       </c>
-      <c r="C2450" t="inlineStr">
+      <c r="C2451" t="inlineStr">
         <is>
           <t>SETOR VAGO VIANA FARMA</t>
         </is>
       </c>
-      <c r="D2450" t="n">
+      <c r="D2451" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:02:31
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2451"/>
+  <dimension ref="A1:D2454"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41441,19 +41441,19 @@
     <row r="2279">
       <c r="A2279" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2279" t="n">
-        <v>2856</v>
+        <v>2858</v>
       </c>
       <c r="C2279" t="inlineStr">
         <is>
-          <t>ALDA SOUZA ROCHA CERQUEIRA - TLV</t>
+          <t>MARY DARLY DE ARAUJO</t>
         </is>
       </c>
       <c r="D2279" t="n">
-        <v>105</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2280">
@@ -41463,15 +41463,15 @@
         </is>
       </c>
       <c r="B2280" t="n">
-        <v>2662</v>
+        <v>2856</v>
       </c>
       <c r="C2280" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
+          <t>ALDA SOUZA ROCHA CERQUEIRA - TLV</t>
         </is>
       </c>
       <c r="D2280" t="n">
-        <v>50</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2281">
@@ -41481,15 +41481,15 @@
         </is>
       </c>
       <c r="B2281" t="n">
-        <v>2663</v>
+        <v>2662</v>
       </c>
       <c r="C2281" t="inlineStr">
         <is>
-          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
         </is>
       </c>
       <c r="D2281" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2282">
@@ -41499,15 +41499,15 @@
         </is>
       </c>
       <c r="B2282" t="n">
-        <v>2685</v>
+        <v>2663</v>
       </c>
       <c r="C2282" t="inlineStr">
         <is>
-          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
+          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
         </is>
       </c>
       <c r="D2282" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2283">
@@ -41517,15 +41517,15 @@
         </is>
       </c>
       <c r="B2283" t="n">
-        <v>2718</v>
+        <v>2685</v>
       </c>
       <c r="C2283" t="inlineStr">
         <is>
-          <t>KALILLA FERREIRA COSTA - FARMA</t>
+          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2283" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2284">
@@ -41535,15 +41535,15 @@
         </is>
       </c>
       <c r="B2284" t="n">
-        <v>2674</v>
+        <v>2718</v>
       </c>
       <c r="C2284" t="inlineStr">
         <is>
-          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
+          <t>KALILLA FERREIRA COSTA - FARMA</t>
         </is>
       </c>
       <c r="D2284" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2285">
@@ -41553,15 +41553,15 @@
         </is>
       </c>
       <c r="B2285" t="n">
-        <v>2753</v>
+        <v>2674</v>
       </c>
       <c r="C2285" t="inlineStr">
         <is>
-          <t>VAGO PATRICIA DOS S. NONATO OLIVEIRA-HB</t>
+          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
         </is>
       </c>
       <c r="D2285" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2286">
@@ -41571,15 +41571,15 @@
         </is>
       </c>
       <c r="B2286" t="n">
-        <v>2772</v>
+        <v>2753</v>
       </c>
       <c r="C2286" t="inlineStr">
         <is>
-          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
+          <t>VAGO PATRICIA DOS S. NONATO OLIVEIRA-HB</t>
         </is>
       </c>
       <c r="D2286" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2287">
@@ -41589,51 +41589,51 @@
         </is>
       </c>
       <c r="B2287" t="n">
-        <v>2827</v>
+        <v>2772</v>
       </c>
       <c r="C2287" t="inlineStr">
         <is>
-          <t>VAGO JOELTON MUNIZ DE SOUZA - HB</t>
+          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2287" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2288">
       <c r="A2288" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2288" t="n">
-        <v>2756</v>
+        <v>2827</v>
       </c>
       <c r="C2288" t="inlineStr">
         <is>
-          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
+          <t>VAGO JOELTON MUNIZ DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2288" t="n">
-        <v>39</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2289">
       <c r="A2289" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2289" t="n">
-        <v>2813</v>
+        <v>2756</v>
       </c>
       <c r="C2289" t="inlineStr">
         <is>
-          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
+          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
         </is>
       </c>
       <c r="D2289" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2290">
@@ -41643,15 +41643,15 @@
         </is>
       </c>
       <c r="B2290" t="n">
-        <v>2738</v>
+        <v>2813</v>
       </c>
       <c r="C2290" t="inlineStr">
         <is>
-          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
+          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
         </is>
       </c>
       <c r="D2290" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2291">
@@ -41661,11 +41661,11 @@
         </is>
       </c>
       <c r="B2291" t="n">
-        <v>2739</v>
+        <v>2738</v>
       </c>
       <c r="C2291" t="inlineStr">
         <is>
-          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
+          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2291" t="n">
@@ -41679,33 +41679,33 @@
         </is>
       </c>
       <c r="B2292" t="n">
-        <v>2824</v>
+        <v>2739</v>
       </c>
       <c r="C2292" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2292" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2293">
       <c r="A2293" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2293" t="n">
-        <v>2843</v>
+        <v>2824</v>
       </c>
       <c r="C2293" t="inlineStr">
         <is>
-          <t>VAGO FEIRA DE SANTANA II - FARMA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D2293" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2294">
@@ -41715,11 +41715,11 @@
         </is>
       </c>
       <c r="B2294" t="n">
-        <v>2747</v>
+        <v>2843</v>
       </c>
       <c r="C2294" t="inlineStr">
         <is>
-          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
+          <t>VAGO FEIRA DE SANTANA II - FARMA</t>
         </is>
       </c>
       <c r="D2294" t="n">
@@ -41733,11 +41733,11 @@
         </is>
       </c>
       <c r="B2295" t="n">
-        <v>2748</v>
+        <v>2747</v>
       </c>
       <c r="C2295" t="inlineStr">
         <is>
-          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
+          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
         </is>
       </c>
       <c r="D2295" t="n">
@@ -41747,73 +41747,73 @@
     <row r="2296">
       <c r="A2296" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2296" t="n">
-        <v>2766</v>
+        <v>2748</v>
       </c>
       <c r="C2296" t="inlineStr">
         <is>
-          <t>SETOR VAGO PEDREIRAS</t>
+          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
         </is>
       </c>
       <c r="D2296" t="n">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2297">
       <c r="A2297" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2297" t="n">
-        <v>2767</v>
+        <v>2766</v>
       </c>
       <c r="C2297" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>SETOR VAGO PEDREIRAS</t>
         </is>
       </c>
       <c r="D2297" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2298">
       <c r="A2298" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2298" t="n">
-        <v>2688</v>
+        <v>2767</v>
       </c>
       <c r="C2298" t="inlineStr">
         <is>
-          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D2298" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2299">
       <c r="A2299" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2299" t="n">
-        <v>2694</v>
+        <v>2688</v>
       </c>
       <c r="C2299" t="inlineStr">
         <is>
-          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
+          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2299" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2300">
@@ -41823,15 +41823,15 @@
         </is>
       </c>
       <c r="B2300" t="n">
-        <v>2714</v>
+        <v>2694</v>
       </c>
       <c r="C2300" t="inlineStr">
         <is>
-          <t>PRISCILA DOS SANTOS LOPES - HB</t>
+          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2300" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2301">
@@ -41841,15 +41841,15 @@
         </is>
       </c>
       <c r="B2301" t="n">
-        <v>2722</v>
+        <v>2714</v>
       </c>
       <c r="C2301" t="inlineStr">
         <is>
-          <t>VAGO ISALTINO BISPO DE O. JUNIOR - FARM</t>
+          <t>PRISCILA DOS SANTOS LOPES - HB</t>
         </is>
       </c>
       <c r="D2301" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2302">
@@ -41859,15 +41859,15 @@
         </is>
       </c>
       <c r="B2302" t="n">
-        <v>2723</v>
+        <v>2722</v>
       </c>
       <c r="C2302" t="inlineStr">
         <is>
-          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
+          <t>VAGO ISALTINO BISPO DE O. JUNIOR - FARM</t>
         </is>
       </c>
       <c r="D2302" t="n">
-        <v>95</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2303">
@@ -41877,15 +41877,15 @@
         </is>
       </c>
       <c r="B2303" t="n">
-        <v>2803</v>
+        <v>2723</v>
       </c>
       <c r="C2303" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
+          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2303" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2304">
@@ -41895,11 +41895,11 @@
         </is>
       </c>
       <c r="B2304" t="n">
-        <v>2804</v>
+        <v>2803</v>
       </c>
       <c r="C2304" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA - HB</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
         </is>
       </c>
       <c r="D2304" t="n">
@@ -41909,19 +41909,19 @@
     <row r="2305">
       <c r="A2305" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2305" t="n">
-        <v>2830</v>
+        <v>2804</v>
       </c>
       <c r="C2305" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 1</t>
+          <t>PAULA CARLA CALDAS MOTA - HB</t>
         </is>
       </c>
       <c r="D2305" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2306">
@@ -41931,11 +41931,11 @@
         </is>
       </c>
       <c r="B2306" t="n">
-        <v>2831</v>
+        <v>2830</v>
       </c>
       <c r="C2306" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 2</t>
+          <t>SETOR VAGO BALSAS 1</t>
         </is>
       </c>
       <c r="D2306" t="n">
@@ -41945,55 +41945,55 @@
     <row r="2307">
       <c r="A2307" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2307" t="n">
-        <v>2647</v>
+        <v>2831</v>
       </c>
       <c r="C2307" t="inlineStr">
         <is>
-          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
+          <t>SETOR VAGO BALSAS 2</t>
         </is>
       </c>
       <c r="D2307" t="n">
-        <v>148</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2308">
       <c r="A2308" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2308" t="n">
-        <v>2661</v>
+        <v>2647</v>
       </c>
       <c r="C2308" t="inlineStr">
         <is>
-          <t>MARIA ISADORA DOS REIS REGO</t>
+          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
         </is>
       </c>
       <c r="D2308" t="n">
-        <v>76</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2309">
       <c r="A2309" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2309" t="n">
-        <v>2686</v>
+        <v>2661</v>
       </c>
       <c r="C2309" t="inlineStr">
         <is>
-          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
+          <t>MARIA ISADORA DOS REIS REGO</t>
         </is>
       </c>
       <c r="D2309" t="n">
-        <v>120</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2310">
@@ -42003,11 +42003,11 @@
         </is>
       </c>
       <c r="B2310" t="n">
-        <v>2687</v>
+        <v>2686</v>
       </c>
       <c r="C2310" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
+          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2310" t="n">
@@ -42017,127 +42017,127 @@
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2311" t="n">
-        <v>2857</v>
+        <v>2687</v>
       </c>
       <c r="C2311" t="inlineStr">
         <is>
-          <t>H-VALQUIRIO OLIVEIRA SOUSA</t>
+          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
         </is>
       </c>
       <c r="D2311" t="n">
-        <v>53</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2312">
       <c r="A2312" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2312" t="n">
-        <v>2681</v>
+        <v>2857</v>
       </c>
       <c r="C2312" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL PI</t>
+          <t>H-VALQUIRIO OLIVEIRA SOUSA</t>
         </is>
       </c>
       <c r="D2312" t="n">
-        <v>69</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2313">
       <c r="A2313" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2313" t="n">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="C2313" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL MA</t>
+          <t>RCA PRINCIPIA OL PI</t>
         </is>
       </c>
       <c r="D2313" t="n">
-        <v>114</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2314">
       <c r="A2314" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2314" t="n">
-        <v>2826</v>
+        <v>2682</v>
       </c>
       <c r="C2314" t="inlineStr">
         <is>
-          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
+          <t>RCA PRINCIPIA OL MA</t>
         </is>
       </c>
       <c r="D2314" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2315">
       <c r="A2315" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2315" t="n">
-        <v>2677</v>
+        <v>2826</v>
       </c>
       <c r="C2315" t="inlineStr">
         <is>
-          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
+          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
         </is>
       </c>
       <c r="D2315" t="n">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2316">
       <c r="A2316" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2316" t="n">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="C2316" t="inlineStr">
         <is>
-          <t>ADRIEL XERXES BARROS MARTINS</t>
+          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
         </is>
       </c>
       <c r="D2316" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2317">
       <c r="A2317" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2317" t="n">
-        <v>2735</v>
+        <v>2678</v>
       </c>
       <c r="C2317" t="inlineStr">
         <is>
-          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
+          <t>ADRIEL XERXES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D2317" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2318">
@@ -42147,15 +42147,15 @@
         </is>
       </c>
       <c r="B2318" t="n">
-        <v>2736</v>
+        <v>2735</v>
       </c>
       <c r="C2318" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
+          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2318" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2319">
@@ -42165,15 +42165,15 @@
         </is>
       </c>
       <c r="B2319" t="n">
-        <v>2737</v>
+        <v>2736</v>
       </c>
       <c r="C2319" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
+          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2319" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2320">
@@ -42183,15 +42183,15 @@
         </is>
       </c>
       <c r="B2320" t="n">
-        <v>2743</v>
+        <v>2737</v>
       </c>
       <c r="C2320" t="inlineStr">
         <is>
-          <t>VAGO SEABRA - FARMA</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
         </is>
       </c>
       <c r="D2320" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2321">
@@ -42201,11 +42201,11 @@
         </is>
       </c>
       <c r="B2321" t="n">
-        <v>2744</v>
+        <v>2743</v>
       </c>
       <c r="C2321" t="inlineStr">
         <is>
-          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
+          <t>VAGO SEABRA - FARMA</t>
         </is>
       </c>
       <c r="D2321" t="n">
@@ -42219,15 +42219,15 @@
         </is>
       </c>
       <c r="B2322" t="n">
-        <v>2745</v>
+        <v>2744</v>
       </c>
       <c r="C2322" t="inlineStr">
         <is>
-          <t>CIRLANE ARAUJO SOUZA - HB</t>
+          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
         </is>
       </c>
       <c r="D2322" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2323">
@@ -42237,33 +42237,33 @@
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2783</v>
+        <v>2745</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
+          <t>CIRLANE ARAUJO SOUZA - HB</t>
         </is>
       </c>
       <c r="D2323" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2324">
       <c r="A2324" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2852</v>
+        <v>2783</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2324" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2325">
@@ -42273,11 +42273,11 @@
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2768</v>
+        <v>2852</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
         </is>
       </c>
       <c r="D2325" t="n">
@@ -42287,73 +42287,73 @@
     <row r="2326">
       <c r="A2326" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2703</v>
+        <v>2768</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2326" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2327">
       <c r="A2327" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2828</v>
+        <v>2703</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>LYERKA MARDANIA RODRIGUES MELO</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2327" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2328">
       <c r="A2328" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2750</v>
+        <v>2828</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>LYERKA MARDANIA RODRIGUES MELO</t>
         </is>
       </c>
       <c r="D2328" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2329">
       <c r="A2329" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2689</v>
+        <v>2750</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2329" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2330">
@@ -42363,69 +42363,69 @@
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2708</v>
+        <v>2689</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2330" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2331">
       <c r="A2331" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2709</v>
+        <v>2708</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2331" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2332">
       <c r="A2332" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2789</v>
+        <v>2709</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>BRUNO TEIXEIRA TORRES</t>
         </is>
       </c>
       <c r="D2332" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2333">
       <c r="A2333" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2790</v>
+        <v>2789</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>VAGO STA INES 01 HNB</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2333" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2334">
@@ -42435,11 +42435,11 @@
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2791</v>
+        <v>2790</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>DANIELY SLZ 01</t>
+          <t>VAGO STA INES 01 HNB</t>
         </is>
       </c>
       <c r="D2334" t="n">
@@ -42449,19 +42449,19 @@
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2805</v>
+        <v>2791</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>DANIELY SLZ 01</t>
         </is>
       </c>
       <c r="D2335" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2336">
@@ -42471,11 +42471,11 @@
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2806</v>
+        <v>2805</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2336" t="n">
@@ -42489,11 +42489,11 @@
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2807</v>
+        <v>2806</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2337" t="n">
@@ -42507,11 +42507,11 @@
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2808</v>
+        <v>2807</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2338" t="n">
@@ -42521,73 +42521,73 @@
     <row r="2339">
       <c r="A2339" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2820</v>
+        <v>2808</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2339" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2851</v>
+        <v>2820</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2341">
       <c r="A2341" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2765</v>
+        <v>2851</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2341" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2342">
       <c r="A2342" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2842</v>
+        <v>2765</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2343">
@@ -42597,33 +42597,33 @@
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2741</v>
+        <v>2842</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D2343" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2344">
       <c r="A2344" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2344" t="n">
-        <v>2758</v>
+        <v>2741</v>
       </c>
       <c r="C2344" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2344" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2345">
@@ -42633,11 +42633,11 @@
         </is>
       </c>
       <c r="B2345" t="n">
-        <v>2854</v>
+        <v>2758</v>
       </c>
       <c r="C2345" t="inlineStr">
         <is>
-          <t>JONILSON SANTANA SANTOS - FARMA</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2345" t="n">
@@ -42651,195 +42651,195 @@
         </is>
       </c>
       <c r="B2346" t="n">
-        <v>2659</v>
+        <v>2854</v>
       </c>
       <c r="C2346" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>JONILSON SANTANA SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2346" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2347">
       <c r="A2347" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2347" t="n">
-        <v>2669</v>
+        <v>2659</v>
       </c>
       <c r="C2347" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2347" t="n">
-        <v>135</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2348">
       <c r="A2348" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2672</v>
+        <v>2669</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2348" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2349">
       <c r="A2349" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2673</v>
+        <v>2860</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
+          <t>HERTZ CE -  TALLIS GUTTEMBERG GUIMARAES</t>
         </is>
       </c>
       <c r="D2349" t="n">
-        <v>95</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2350">
       <c r="A2350" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2676</v>
+        <v>2672</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2350" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2351">
       <c r="A2351" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2760</v>
+        <v>2673</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2351" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2352">
       <c r="A2352" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2823</v>
+        <v>2676</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2352" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2353">
       <c r="A2353" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2848</v>
+        <v>2760</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2353" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2354">
       <c r="A2354" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2792</v>
+        <v>2823</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2354" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2355">
       <c r="A2355" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2793</v>
+        <v>2848</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2355" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2356">
       <c r="A2356" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2802</v>
+        <v>2792</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2356" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2357">
@@ -42849,11 +42849,11 @@
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2656</v>
+        <v>2793</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2357" t="n">
@@ -42863,19 +42863,19 @@
     <row r="2358">
       <c r="A2358" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2657</v>
+        <v>2802</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA IMP 01 HNB</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2358" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2359">
@@ -42885,33 +42885,33 @@
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2658</v>
+        <v>2656</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2359" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2360">
       <c r="A2360" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2729</v>
+        <v>2657</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>MARIA APARECIDA IMP 01 HNB</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2361">
@@ -42921,33 +42921,33 @@
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2759</v>
+        <v>2658</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2361" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2362">
       <c r="A2362" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2832</v>
+        <v>2729</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2362" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2363">
@@ -42957,11 +42957,11 @@
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2769</v>
+        <v>2759</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2363" t="n">
@@ -42971,73 +42971,73 @@
     <row r="2364">
       <c r="A2364" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2679</v>
+        <v>2832</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
         </is>
       </c>
       <c r="D2364" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2365">
       <c r="A2365" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2680</v>
+        <v>2769</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2365" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2815</v>
+        <v>2679</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2366" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2367">
       <c r="A2367" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2816</v>
+        <v>2680</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2368">
@@ -43047,105 +43047,105 @@
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2817</v>
+        <v>2815</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2368" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2369">
       <c r="A2369" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2841</v>
+        <v>2816</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2369" t="n">
-        <v>46</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2370">
       <c r="A2370" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2701</v>
+        <v>2817</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2644</v>
+        <v>2841</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>108</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2372">
       <c r="A2372" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2645</v>
+        <v>2701</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2372" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2373">
       <c r="A2373" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2754</v>
+        <v>2644</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2374">
@@ -43155,51 +43155,51 @@
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2755</v>
+        <v>2645</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>80</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2375">
       <c r="A2375" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2665</v>
+        <v>2754</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2375" t="n">
-        <v>141</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2376">
       <c r="A2376" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2667</v>
+        <v>2755</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>VAGO AÇAILÂNDIA HNB</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2376" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2377">
@@ -43209,15 +43209,15 @@
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2727</v>
+        <v>2665</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2377" t="n">
-        <v>120</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2378">
@@ -43227,51 +43227,51 @@
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2728</v>
+        <v>2667</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>VAGO AÇAILÂNDIA HNB</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2379">
       <c r="A2379" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2833</v>
+        <v>2727</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>ADEILZA PINTO DA SILVA - FARMA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2379" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2380">
       <c r="A2380" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2814</v>
+        <v>2728</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2380" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2381">
@@ -43281,33 +43281,33 @@
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2855</v>
+        <v>2833</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>DESIREE BARROS DE CARVALHO - CCM</t>
+          <t>ADEILZA PINTO DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>14</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2382">
       <c r="A2382" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2646</v>
+        <v>2814</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2383">
@@ -43317,15 +43317,15 @@
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2650</v>
+        <v>2855</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>DESIREE BARROS DE CARVALHO - CCM</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>95</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2384">
@@ -43335,15 +43335,15 @@
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2652</v>
+        <v>2646</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2385">
@@ -43353,11 +43353,11 @@
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2653</v>
+        <v>2650</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2385" t="n">
@@ -43371,15 +43371,15 @@
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2654</v>
+        <v>2652</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2387">
@@ -43389,33 +43389,33 @@
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2655</v>
+        <v>2653</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2387" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2821</v>
+        <v>2654</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>69</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2389">
@@ -43425,231 +43425,231 @@
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2683</v>
+        <v>2655</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2684</v>
+        <v>2821</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2391">
       <c r="A2391" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2749</v>
+        <v>2683</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>111</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2812</v>
+        <v>2684</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>145</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2715</v>
+        <v>2749</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>90</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2394">
       <c r="A2394" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2834</v>
+        <v>2812</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>GILVANA MONTELES U. SANTOS HNB</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>114</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2651</v>
+        <v>2715</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>145</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2396">
       <c r="A2396" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2819</v>
+        <v>2834</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>GILVANA MONTELES U. SANTOS HNB</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2397">
       <c r="A2397" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2849</v>
+        <v>2651</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>MULTI PE (PEDRO HENRIQUE VIERA)</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>72</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2835</v>
+        <v>2819</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>ROGÉRIO LIRA DA GAMA</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>116</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2699</v>
+        <v>2849</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>MULTI PE (PEDRO HENRIQUE VIERA)</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>95</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2400">
       <c r="A2400" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2706</v>
+        <v>2835</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>VAGO BARREIRINHAS HNB</t>
+          <t>ROGÉRIO LIRA DA GAMA</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2401">
       <c r="A2401" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2707</v>
+        <v>2699</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>VAGO BACABAL HNB</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2402">
@@ -43659,15 +43659,15 @@
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2846</v>
+        <v>2706</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>VAGO BARREIRINHAS HNB</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2403">
@@ -43677,87 +43677,87 @@
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2847</v>
+        <v>2707</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>FRANCISCO WERBERTTY DA SILVA MORAIS</t>
+          <t>VAGO BACABAL HNB</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2404">
       <c r="A2404" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2693</v>
+        <v>2846</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2405">
       <c r="A2405" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2705</v>
+        <v>2847</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>FRANCISCO WERBERTTY DA SILVA MORAIS</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>146</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2664</v>
+        <v>2693</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2407">
       <c r="A2407" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2670</v>
+        <v>2705</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>69</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2408">
@@ -43767,69 +43767,69 @@
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2730</v>
+        <v>2664</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2671</v>
+        <v>2670</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2410">
       <c r="A2410" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2691</v>
+        <v>2730</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2410" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2411">
       <c r="A2411" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2692</v>
+        <v>2859</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>ALEXANDRE MARTINS CHAVES</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>80</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2412">
@@ -43839,123 +43839,123 @@
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2724</v>
+        <v>2671</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2413">
       <c r="A2413" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2773</v>
+        <v>2691</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>TIMON 01 HNB</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2414">
       <c r="A2414" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2844</v>
+        <v>2692</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>132</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2415">
       <c r="A2415" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2845</v>
+        <v>2724</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2415" t="n">
-        <v>132</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2416">
       <c r="A2416" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2825</v>
+        <v>2773</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>TIMON 01 HNB</t>
         </is>
       </c>
       <c r="D2416" t="n">
-        <v>90</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2417">
       <c r="A2417" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2787</v>
+        <v>2844</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>120</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2418">
       <c r="A2418" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2839</v>
+        <v>2845</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>RCA TENA OL PI</t>
+          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
         </is>
       </c>
       <c r="D2418" t="n">
-        <v>69</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2419">
@@ -43965,15 +43965,15 @@
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2840</v>
+        <v>2825</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>RCA TENA OL MA</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2419" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2420">
@@ -43983,69 +43983,69 @@
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2648</v>
+        <v>2787</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2421">
       <c r="A2421" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2666</v>
+        <v>2839</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>RCA TENA OL PI</t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2422">
       <c r="A2422" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2779</v>
+        <v>2840</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO - TLV</t>
+          <t>RCA TENA OL MA</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>105</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2423">
       <c r="A2423" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2780</v>
+        <v>2648</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>105</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2424">
@@ -44055,123 +44055,123 @@
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2786</v>
+        <v>2666</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2424" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2425">
       <c r="A2425" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2660</v>
+        <v>2779</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO - TLV</t>
         </is>
       </c>
       <c r="D2425" t="n">
-        <v>38</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2426">
       <c r="A2426" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2716</v>
+        <v>2780</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2426" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2427">
       <c r="A2427" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2734</v>
+        <v>2786</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2427" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2428">
       <c r="A2428" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2853</v>
+        <v>2660</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>H-ROBERTO SOARES OLIVEIRA JUNIOR</t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2428" t="n">
-        <v>53</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2429">
       <c r="A2429" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2742</v>
+        <v>2716</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS - FARMA JACOBINA</t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2429" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2430">
       <c r="A2430" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2430" t="n">
-        <v>2794</v>
+        <v>2734</v>
       </c>
       <c r="C2430" t="inlineStr">
         <is>
-          <t>VAGO DEISIELLE J. SILVA - HB JACOBINA</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2430" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2431">
@@ -44181,15 +44181,15 @@
         </is>
       </c>
       <c r="B2431" t="n">
-        <v>2795</v>
+        <v>2853</v>
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
+          <t>H-ROBERTO SOARES OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2431" t="n">
-        <v>95</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2432">
@@ -44199,11 +44199,11 @@
         </is>
       </c>
       <c r="B2432" t="n">
-        <v>2796</v>
+        <v>2742</v>
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VAGO MARCUS VINICIUS - FARMA JACOBINA</t>
         </is>
       </c>
       <c r="D2432" t="n">
@@ -44217,15 +44217,15 @@
         </is>
       </c>
       <c r="B2433" t="n">
-        <v>2797</v>
+        <v>2794</v>
       </c>
       <c r="C2433" t="inlineStr">
         <is>
-          <t>VAGO ESDRAS A. SANTOS-FAR (PAULO AFO)</t>
+          <t>VAGO DEISIELLE J. SILVA - HB JACOBINA</t>
         </is>
       </c>
       <c r="D2433" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2434">
@@ -44235,11 +44235,11 @@
         </is>
       </c>
       <c r="B2434" t="n">
-        <v>2798</v>
+        <v>2795</v>
       </c>
       <c r="C2434" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
         </is>
       </c>
       <c r="D2434" t="n">
@@ -44249,145 +44249,145 @@
     <row r="2435">
       <c r="A2435" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2435" t="n">
-        <v>2668</v>
+        <v>2796</v>
       </c>
       <c r="C2435" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2435" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2436">
       <c r="A2436" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2436" t="n">
-        <v>2690</v>
+        <v>2797</v>
       </c>
       <c r="C2436" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>VAGO ESDRAS A. SANTOS-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2436" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2437">
       <c r="A2437" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2437" t="n">
-        <v>2696</v>
+        <v>2798</v>
       </c>
       <c r="C2437" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2437" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2438">
       <c r="A2438" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2438" t="n">
-        <v>2697</v>
+        <v>2668</v>
       </c>
       <c r="C2438" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2438" t="n">
-        <v>69</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2439">
       <c r="A2439" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2439" t="n">
-        <v>2698</v>
+        <v>2690</v>
       </c>
       <c r="C2439" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2439" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2440">
       <c r="A2440" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2440" t="n">
-        <v>2775</v>
+        <v>2696</v>
       </c>
       <c r="C2440" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2440" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2441">
       <c r="A2441" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2441" t="n">
-        <v>2776</v>
+        <v>2697</v>
       </c>
       <c r="C2441" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2441" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2442">
       <c r="A2442" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2442" t="n">
-        <v>2777</v>
+        <v>2698</v>
       </c>
       <c r="C2442" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2442" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2443">
@@ -44397,11 +44397,11 @@
         </is>
       </c>
       <c r="B2443" t="n">
-        <v>2778</v>
+        <v>2775</v>
       </c>
       <c r="C2443" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2443" t="n">
@@ -44415,15 +44415,15 @@
         </is>
       </c>
       <c r="B2444" t="n">
-        <v>2781</v>
+        <v>2776</v>
       </c>
       <c r="C2444" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2444" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2445">
@@ -44433,11 +44433,11 @@
         </is>
       </c>
       <c r="B2445" t="n">
-        <v>2822</v>
+        <v>2777</v>
       </c>
       <c r="C2445" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2445" t="n">
@@ -44451,11 +44451,11 @@
         </is>
       </c>
       <c r="B2446" t="n">
-        <v>2740</v>
+        <v>2778</v>
       </c>
       <c r="C2446" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2446" t="n">
@@ -44465,37 +44465,37 @@
     <row r="2447">
       <c r="A2447" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2447" t="n">
-        <v>2710</v>
+        <v>2781</v>
       </c>
       <c r="C2447" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2447" t="n">
-        <v>69</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2448">
       <c r="A2448" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2448" t="n">
-        <v>2711</v>
+        <v>2822</v>
       </c>
       <c r="C2448" t="inlineStr">
         <is>
-          <t>CARLOS CHAPADINHA</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2448" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2449">
@@ -44505,11 +44505,11 @@
         </is>
       </c>
       <c r="B2449" t="n">
-        <v>2712</v>
+        <v>2740</v>
       </c>
       <c r="C2449" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2449" t="n">
@@ -44523,11 +44523,11 @@
         </is>
       </c>
       <c r="B2450" t="n">
-        <v>2717</v>
+        <v>2710</v>
       </c>
       <c r="C2450" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2450" t="n">
@@ -44537,18 +44537,72 @@
     <row r="2451">
       <c r="A2451" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2451" t="n">
+        <v>2711</v>
+      </c>
+      <c r="C2451" t="inlineStr">
+        <is>
+          <t>CARLOS CHAPADINHA</t>
+        </is>
+      </c>
+      <c r="D2451" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2452">
+      <c r="A2452" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2452" t="n">
+        <v>2712</v>
+      </c>
+      <c r="C2452" t="inlineStr">
+        <is>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
+        </is>
+      </c>
+      <c r="D2452" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2453">
+      <c r="A2453" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2453" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2453" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2453" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2454">
+      <c r="A2454" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2454" t="n">
         <v>2801</v>
       </c>
-      <c r="C2451" t="inlineStr">
+      <c r="C2454" t="inlineStr">
         <is>
           <t>SETOR VAGO VIANA FARMA</t>
         </is>
       </c>
-      <c r="D2451" t="n">
+      <c r="D2454" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:02:20
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -33312,7 +33312,7 @@
       </c>
       <c r="C1827" t="inlineStr">
         <is>
-          <t>PETROLINA-HB  (VAGO/VALERIA COELHO )</t>
+          <t>PETROLINA-HB  (CLISMARLEY FARIAS )</t>
         </is>
       </c>
       <c r="D1827" t="n">
@@ -40783,7 +40783,7 @@
       </c>
       <c r="C2242" t="inlineStr">
         <is>
-          <t>REDES AGRESTE - HB  (MAX WEDSON)</t>
+          <t>REDES AGRESTE - HB  (VAGO/MAX WEDSON)</t>
         </is>
       </c>
       <c r="D2242" t="n">

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:03:02
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2454"/>
+  <dimension ref="A1:D2456"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29914,7 +29914,7 @@
         </is>
       </c>
       <c r="D1638" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1639">
@@ -35747,7 +35747,7 @@
         </is>
       </c>
       <c r="D1962" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1963">
@@ -38051,7 +38051,7 @@
         </is>
       </c>
       <c r="D2090" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2091">
@@ -41333,15 +41333,15 @@
     <row r="2273">
       <c r="A2273" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2273" t="n">
-        <v>2799</v>
+        <v>2861</v>
       </c>
       <c r="C2273" t="inlineStr">
         <is>
-          <t>VOLFRAMIO DALFREDO ALMEIDA</t>
+          <t>ATIRSON DA SILVA GOMES</t>
         </is>
       </c>
       <c r="D2273" t="n">
@@ -41351,55 +41351,55 @@
     <row r="2274">
       <c r="A2274" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2274" t="n">
-        <v>2719</v>
+        <v>2862</v>
       </c>
       <c r="C2274" t="inlineStr">
         <is>
-          <t>SETOR SÃO RDO NONATO VAGO  (DEDICADA)</t>
+          <t>BRUNA RAISEYLLA SANTOS DE SALES</t>
         </is>
       </c>
       <c r="D2274" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2275">
       <c r="A2275" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2275" t="n">
-        <v>2731</v>
+        <v>2799</v>
       </c>
       <c r="C2275" t="inlineStr">
         <is>
-          <t>VAGO ANDERSON A. S. - FARMA (CAMAÇARI)</t>
+          <t>VOLFRAMIO DALFREDO ALMEIDA</t>
         </is>
       </c>
       <c r="D2275" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2276">
       <c r="A2276" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2276" t="n">
-        <v>2732</v>
+        <v>2719</v>
       </c>
       <c r="C2276" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN DE JESUS - HB</t>
+          <t>SETOR SÃO RDO NONATO VAGO  (DEDICADA)</t>
         </is>
       </c>
       <c r="D2276" t="n">
-        <v>98</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2277">
@@ -41409,11 +41409,11 @@
         </is>
       </c>
       <c r="B2277" t="n">
-        <v>2733</v>
+        <v>2731</v>
       </c>
       <c r="C2277" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAGO CENTRO CAROLINE LEMOS - FARMA </t>
+          <t>VAGO ANDERSON A. S. - FARMA (CAMAÇARI)</t>
         </is>
       </c>
       <c r="D2277" t="n">
@@ -41423,73 +41423,73 @@
     <row r="2278">
       <c r="A2278" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2278" t="n">
-        <v>2752</v>
+        <v>2732</v>
       </c>
       <c r="C2278" t="inlineStr">
         <is>
-          <t>SETOR BAIXADA PLUS (ELILTON ROMEU)</t>
+          <t>VAGO BRENO ALLAN DE JESUS - HB</t>
         </is>
       </c>
       <c r="D2278" t="n">
-        <v>114</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2279">
       <c r="A2279" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2279" t="n">
-        <v>2858</v>
+        <v>2733</v>
       </c>
       <c r="C2279" t="inlineStr">
         <is>
-          <t>MARY DARLY DE ARAUJO</t>
+          <t xml:space="preserve">VAGO CENTRO CAROLINE LEMOS - FARMA </t>
         </is>
       </c>
       <c r="D2279" t="n">
-        <v>2</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2280">
       <c r="A2280" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2280" t="n">
-        <v>2856</v>
+        <v>2752</v>
       </c>
       <c r="C2280" t="inlineStr">
         <is>
-          <t>ALDA SOUZA ROCHA CERQUEIRA - TLV</t>
+          <t>SETOR BAIXADA PLUS (ELILTON ROMEU)</t>
         </is>
       </c>
       <c r="D2280" t="n">
-        <v>105</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2281">
       <c r="A2281" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2281" t="n">
-        <v>2662</v>
+        <v>2858</v>
       </c>
       <c r="C2281" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
+          <t>MARY DARLY DE ARAUJO</t>
         </is>
       </c>
       <c r="D2281" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2282">
@@ -41499,15 +41499,15 @@
         </is>
       </c>
       <c r="B2282" t="n">
-        <v>2663</v>
+        <v>2856</v>
       </c>
       <c r="C2282" t="inlineStr">
         <is>
-          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
+          <t>ALDA SOUZA ROCHA CERQUEIRA - TLV</t>
         </is>
       </c>
       <c r="D2282" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2283">
@@ -41517,15 +41517,15 @@
         </is>
       </c>
       <c r="B2283" t="n">
-        <v>2685</v>
+        <v>2662</v>
       </c>
       <c r="C2283" t="inlineStr">
         <is>
-          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - FARMA</t>
         </is>
       </c>
       <c r="D2283" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2284">
@@ -41535,15 +41535,15 @@
         </is>
       </c>
       <c r="B2284" t="n">
-        <v>2718</v>
+        <v>2663</v>
       </c>
       <c r="C2284" t="inlineStr">
         <is>
-          <t>KALILLA FERREIRA COSTA - FARMA</t>
+          <t>ALANA FABRICIA DE SOUZA REZENDE - HB</t>
         </is>
       </c>
       <c r="D2284" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2285">
@@ -41553,11 +41553,11 @@
         </is>
       </c>
       <c r="B2285" t="n">
-        <v>2674</v>
+        <v>2685</v>
       </c>
       <c r="C2285" t="inlineStr">
         <is>
-          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
+          <t>VAGO SANDRO ALAN MARTINS DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2285" t="n">
@@ -41571,15 +41571,15 @@
         </is>
       </c>
       <c r="B2286" t="n">
-        <v>2753</v>
+        <v>2718</v>
       </c>
       <c r="C2286" t="inlineStr">
         <is>
-          <t>VAGO PATRICIA DOS S. NONATO OLIVEIRA-HB</t>
+          <t>KALILLA FERREIRA COSTA - FARMA</t>
         </is>
       </c>
       <c r="D2286" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2287">
@@ -41589,15 +41589,15 @@
         </is>
       </c>
       <c r="B2287" t="n">
-        <v>2772</v>
+        <v>2674</v>
       </c>
       <c r="C2287" t="inlineStr">
         <is>
-          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
+          <t>ELVYS BRUCE SILVA FERNANDES - HB</t>
         </is>
       </c>
       <c r="D2287" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2288">
@@ -41607,69 +41607,69 @@
         </is>
       </c>
       <c r="B2288" t="n">
-        <v>2827</v>
+        <v>2753</v>
       </c>
       <c r="C2288" t="inlineStr">
         <is>
-          <t>VAGO JOELTON MUNIZ DE SOUZA - HB</t>
+          <t>VAGO PATRICIA DOS S. NONATO OLIVEIRA-HB</t>
         </is>
       </c>
       <c r="D2288" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2289">
       <c r="A2289" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2289" t="n">
-        <v>2756</v>
+        <v>2772</v>
       </c>
       <c r="C2289" t="inlineStr">
         <is>
-          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
+          <t>CLEONICE DE LUNA NERES SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2289" t="n">
-        <v>39</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2290">
       <c r="A2290" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2290" t="n">
-        <v>2813</v>
+        <v>2827</v>
       </c>
       <c r="C2290" t="inlineStr">
         <is>
-          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
+          <t>VAGO JOELTON MUNIZ DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2290" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2291">
       <c r="A2291" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2291" t="n">
-        <v>2738</v>
+        <v>2756</v>
       </c>
       <c r="C2291" t="inlineStr">
         <is>
-          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
+          <t>CLIENTES INATIVOS COM DÉBITO SAYONARA</t>
         </is>
       </c>
       <c r="D2291" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2292">
@@ -41679,15 +41679,15 @@
         </is>
       </c>
       <c r="B2292" t="n">
-        <v>2739</v>
+        <v>2813</v>
       </c>
       <c r="C2292" t="inlineStr">
         <is>
-          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
+          <t>NATALIA FONTENELE DOS SANTOS DA SILVA</t>
         </is>
       </c>
       <c r="D2292" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2293">
@@ -41697,51 +41697,51 @@
         </is>
       </c>
       <c r="B2293" t="n">
-        <v>2824</v>
+        <v>2738</v>
       </c>
       <c r="C2293" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>NEYSE LIMA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2293" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2294">
       <c r="A2294" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2294" t="n">
-        <v>2843</v>
+        <v>2739</v>
       </c>
       <c r="C2294" t="inlineStr">
         <is>
-          <t>VAGO FEIRA DE SANTANA II - FARMA</t>
+          <t>JEANIA PIRES (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2294" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2295">
       <c r="A2295" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2295" t="n">
-        <v>2747</v>
+        <v>2824</v>
       </c>
       <c r="C2295" t="inlineStr">
         <is>
-          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D2295" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2296">
@@ -41751,11 +41751,11 @@
         </is>
       </c>
       <c r="B2296" t="n">
-        <v>2748</v>
+        <v>2843</v>
       </c>
       <c r="C2296" t="inlineStr">
         <is>
-          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
+          <t>VAGO FEIRA DE SANTANA II - FARMA</t>
         </is>
       </c>
       <c r="D2296" t="n">
@@ -41765,37 +41765,37 @@
     <row r="2297">
       <c r="A2297" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2297" t="n">
-        <v>2766</v>
+        <v>2747</v>
       </c>
       <c r="C2297" t="inlineStr">
         <is>
-          <t>SETOR VAGO PEDREIRAS</t>
+          <t>DOMINGOS PEREIRA BASTOS - FARMA</t>
         </is>
       </c>
       <c r="D2297" t="n">
-        <v>120</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2298">
       <c r="A2298" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2298" t="n">
-        <v>2767</v>
+        <v>2748</v>
       </c>
       <c r="C2298" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>VAGO WILSON PORTUGAL A. FILHO - FARMA</t>
         </is>
       </c>
       <c r="D2298" t="n">
-        <v>39</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2299">
@@ -41805,51 +41805,51 @@
         </is>
       </c>
       <c r="B2299" t="n">
-        <v>2688</v>
+        <v>2766</v>
       </c>
       <c r="C2299" t="inlineStr">
         <is>
-          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
+          <t>SETOR VAGO PEDREIRAS</t>
         </is>
       </c>
       <c r="D2299" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2300">
       <c r="A2300" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2300" t="n">
-        <v>2694</v>
+        <v>2767</v>
       </c>
       <c r="C2300" t="inlineStr">
         <is>
-          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D2300" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2301">
       <c r="A2301" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2301" t="n">
-        <v>2714</v>
+        <v>2688</v>
       </c>
       <c r="C2301" t="inlineStr">
         <is>
-          <t>PRISCILA DOS SANTOS LOPES - HB</t>
+          <t>LUZIANA OLIVEIRA DA SILVA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2301" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2302">
@@ -41859,15 +41859,15 @@
         </is>
       </c>
       <c r="B2302" t="n">
-        <v>2722</v>
+        <v>2694</v>
       </c>
       <c r="C2302" t="inlineStr">
         <is>
-          <t>VAGO ISALTINO BISPO DE O. JUNIOR - FARM</t>
+          <t>VAGO TIAGO FERNANDO DOS SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2302" t="n">
-        <v>50</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2303">
@@ -41877,15 +41877,15 @@
         </is>
       </c>
       <c r="B2303" t="n">
-        <v>2723</v>
+        <v>2714</v>
       </c>
       <c r="C2303" t="inlineStr">
         <is>
-          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
+          <t>PRISCILA DOS SANTOS LOPES - HB</t>
         </is>
       </c>
       <c r="D2303" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2304">
@@ -41895,15 +41895,15 @@
         </is>
       </c>
       <c r="B2304" t="n">
-        <v>2803</v>
+        <v>2722</v>
       </c>
       <c r="C2304" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
+          <t>VAGO ISALTINO BISPO DE O. JUNIOR - FARM</t>
         </is>
       </c>
       <c r="D2304" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2305">
@@ -41913,267 +41913,267 @@
         </is>
       </c>
       <c r="B2305" t="n">
-        <v>2804</v>
+        <v>2723</v>
       </c>
       <c r="C2305" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA - HB</t>
+          <t>VAGO ALAN CAIQUE SANTOS E SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2305" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2306">
       <c r="A2306" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2306" t="n">
-        <v>2830</v>
+        <v>2803</v>
       </c>
       <c r="C2306" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 1</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO - HB</t>
         </is>
       </c>
       <c r="D2306" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2307">
       <c r="A2307" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2307" t="n">
-        <v>2831</v>
+        <v>2804</v>
       </c>
       <c r="C2307" t="inlineStr">
         <is>
-          <t>SETOR VAGO BALSAS 2</t>
+          <t>PAULA CARLA CALDAS MOTA - HB</t>
         </is>
       </c>
       <c r="D2307" t="n">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2308">
       <c r="A2308" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2308" t="n">
-        <v>2647</v>
+        <v>2830</v>
       </c>
       <c r="C2308" t="inlineStr">
         <is>
-          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
+          <t>SETOR VAGO BALSAS 1</t>
         </is>
       </c>
       <c r="D2308" t="n">
-        <v>148</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2309">
       <c r="A2309" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2309" t="n">
-        <v>2661</v>
+        <v>2831</v>
       </c>
       <c r="C2309" t="inlineStr">
         <is>
-          <t>MARIA ISADORA DOS REIS REGO</t>
+          <t>SETOR VAGO BALSAS 2</t>
         </is>
       </c>
       <c r="D2309" t="n">
-        <v>76</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2310">
       <c r="A2310" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2310" t="n">
-        <v>2686</v>
+        <v>2647</v>
       </c>
       <c r="C2310" t="inlineStr">
         <is>
-          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
+          <t>ZONA OESTE- FARMA(HUGO MATHEUS)</t>
         </is>
       </c>
       <c r="D2310" t="n">
-        <v>120</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2311">
       <c r="A2311" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2311" t="n">
-        <v>2687</v>
+        <v>2661</v>
       </c>
       <c r="C2311" t="inlineStr">
         <is>
-          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
+          <t>MARIA ISADORA DOS REIS REGO</t>
         </is>
       </c>
       <c r="D2311" t="n">
-        <v>120</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2312">
       <c r="A2312" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2312" t="n">
-        <v>2857</v>
+        <v>2686</v>
       </c>
       <c r="C2312" t="inlineStr">
         <is>
-          <t>H-VALQUIRIO OLIVEIRA SOUSA</t>
+          <t>JOSE DO NASCIMENTO ALVES PEREIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2312" t="n">
-        <v>53</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2313">
       <c r="A2313" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2313" t="n">
-        <v>2681</v>
+        <v>2687</v>
       </c>
       <c r="C2313" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL PI</t>
+          <t>GILBERTO MOREIRA MENESES JUNIOR (FARMA)</t>
         </is>
       </c>
       <c r="D2313" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2314">
       <c r="A2314" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2314" t="n">
-        <v>2682</v>
+        <v>2857</v>
       </c>
       <c r="C2314" t="inlineStr">
         <is>
-          <t>RCA PRINCIPIA OL MA</t>
+          <t>H-VALQUIRIO OLIVEIRA SOUSA</t>
         </is>
       </c>
       <c r="D2314" t="n">
-        <v>114</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2315">
       <c r="A2315" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2315" t="n">
-        <v>2826</v>
+        <v>2681</v>
       </c>
       <c r="C2315" t="inlineStr">
         <is>
-          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
+          <t>RCA PRINCIPIA OL PI</t>
         </is>
       </c>
       <c r="D2315" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2316">
       <c r="A2316" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2316" t="n">
-        <v>2677</v>
+        <v>2682</v>
       </c>
       <c r="C2316" t="inlineStr">
         <is>
-          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
+          <t>RCA PRINCIPIA OL MA</t>
         </is>
       </c>
       <c r="D2316" t="n">
-        <v>72</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2317">
       <c r="A2317" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2317" t="n">
-        <v>2678</v>
+        <v>2826</v>
       </c>
       <c r="C2317" t="inlineStr">
         <is>
-          <t>ADRIEL XERXES BARROS MARTINS</t>
+          <t>CRISTIANE ANDRADE DOS REIS N. - FARMA</t>
         </is>
       </c>
       <c r="D2317" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2318">
       <c r="A2318" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2318" t="n">
-        <v>2735</v>
+        <v>2677</v>
       </c>
       <c r="C2318" t="inlineStr">
         <is>
-          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
+          <t>ROSA SELVAGEM OL - JOACI GUILHERME</t>
         </is>
       </c>
       <c r="D2318" t="n">
-        <v>100</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2319">
       <c r="A2319" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2319" t="n">
-        <v>2736</v>
+        <v>2678</v>
       </c>
       <c r="C2319" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
+          <t>ADRIEL XERXES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D2319" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2320">
@@ -42183,11 +42183,11 @@
         </is>
       </c>
       <c r="B2320" t="n">
-        <v>2737</v>
+        <v>2735</v>
       </c>
       <c r="C2320" t="inlineStr">
         <is>
-          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
+          <t>RICARDO BARBOSA DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2320" t="n">
@@ -42201,11 +42201,11 @@
         </is>
       </c>
       <c r="B2321" t="n">
-        <v>2743</v>
+        <v>2736</v>
       </c>
       <c r="C2321" t="inlineStr">
         <is>
-          <t>VAGO SEABRA - FARMA</t>
+          <t>VAGO VINICIUS GUEDES DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2321" t="n">
@@ -42219,15 +42219,15 @@
         </is>
       </c>
       <c r="B2322" t="n">
-        <v>2744</v>
+        <v>2737</v>
       </c>
       <c r="C2322" t="inlineStr">
         <is>
-          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
+          <t>VAGO MURILO CHIBANA ALVES CRUZ - HB</t>
         </is>
       </c>
       <c r="D2322" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2323">
@@ -42237,15 +42237,15 @@
         </is>
       </c>
       <c r="B2323" t="n">
-        <v>2745</v>
+        <v>2743</v>
       </c>
       <c r="C2323" t="inlineStr">
         <is>
-          <t>CIRLANE ARAUJO SOUZA - HB</t>
+          <t>VAGO SEABRA - FARMA</t>
         </is>
       </c>
       <c r="D2323" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2324">
@@ -42255,11 +42255,11 @@
         </is>
       </c>
       <c r="B2324" t="n">
-        <v>2783</v>
+        <v>2744</v>
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
+          <t>CLAUDIO ROBERTO S. SOUZA- FAR. (VALENÇA)</t>
         </is>
       </c>
       <c r="D2324" t="n">
@@ -42269,55 +42269,55 @@
     <row r="2325">
       <c r="A2325" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2325" t="n">
-        <v>2852</v>
+        <v>2745</v>
       </c>
       <c r="C2325" t="inlineStr">
         <is>
-          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
+          <t>CIRLANE ARAUJO SOUZA - HB</t>
         </is>
       </c>
       <c r="D2325" t="n">
-        <v>69</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2326">
       <c r="A2326" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2326" t="n">
-        <v>2768</v>
+        <v>2783</v>
       </c>
       <c r="C2326" t="inlineStr">
         <is>
-          <t>LAURIENE SILVA BARBOSA</t>
+          <t>VAGO CAROLINE HORA - FARMA (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2326" t="n">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2327">
       <c r="A2327" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2327" t="n">
-        <v>2703</v>
+        <v>2852</v>
       </c>
       <c r="C2327" t="inlineStr">
         <is>
-          <t>VAGO ANA PAULA N. Z. - FARMA</t>
+          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
         </is>
       </c>
       <c r="D2327" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2328">
@@ -42327,15 +42327,15 @@
         </is>
       </c>
       <c r="B2328" t="n">
-        <v>2828</v>
+        <v>2768</v>
       </c>
       <c r="C2328" t="inlineStr">
         <is>
-          <t>LYERKA MARDANIA RODRIGUES MELO</t>
+          <t>LAURIENE SILVA BARBOSA</t>
         </is>
       </c>
       <c r="D2328" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2329">
@@ -42345,69 +42345,69 @@
         </is>
       </c>
       <c r="B2329" t="n">
-        <v>2750</v>
+        <v>2703</v>
       </c>
       <c r="C2329" t="inlineStr">
         <is>
-          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
+          <t>VAGO ANA PAULA N. Z. - FARMA</t>
         </is>
       </c>
       <c r="D2329" t="n">
-        <v>50</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2330">
       <c r="A2330" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2330" t="n">
-        <v>2689</v>
+        <v>2828</v>
       </c>
       <c r="C2330" t="inlineStr">
         <is>
-          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
+          <t>LYERKA MARDANIA RODRIGUES MELO</t>
         </is>
       </c>
       <c r="D2330" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2331">
       <c r="A2331" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2331" t="n">
-        <v>2708</v>
+        <v>2750</v>
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
+          <t>RIOLANDO FERREIRA DE SOUZA JR - FARMA</t>
         </is>
       </c>
       <c r="D2331" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2332">
       <c r="A2332" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2332" t="n">
-        <v>2709</v>
+        <v>2689</v>
       </c>
       <c r="C2332" t="inlineStr">
         <is>
-          <t>BRUNO TEIXEIRA TORRES</t>
+          <t>JOSE FRANCISCO SANTOS OLIVEIRA</t>
         </is>
       </c>
       <c r="D2332" t="n">
-        <v>39</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2333">
@@ -42417,11 +42417,11 @@
         </is>
       </c>
       <c r="B2333" t="n">
-        <v>2789</v>
+        <v>2708</v>
       </c>
       <c r="C2333" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>CARLOS JEANDERSON DA SILVA GUTIERRES</t>
         </is>
       </c>
       <c r="D2333" t="n">
@@ -42431,73 +42431,73 @@
     <row r="2334">
       <c r="A2334" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2334" t="n">
-        <v>2790</v>
+        <v>2709</v>
       </c>
       <c r="C2334" t="inlineStr">
         <is>
-          <t>VAGO STA INES 01 HNB</t>
+          <t>BRUNO TEIXEIRA TORRES</t>
         </is>
       </c>
       <c r="D2334" t="n">
-        <v>114</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2335">
       <c r="A2335" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2335" t="n">
-        <v>2791</v>
+        <v>2789</v>
       </c>
       <c r="C2335" t="inlineStr">
         <is>
-          <t>DANIELY SLZ 01</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2335" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2336">
       <c r="A2336" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2336" t="n">
-        <v>2805</v>
+        <v>2790</v>
       </c>
       <c r="C2336" t="inlineStr">
         <is>
-          <t>JANAINA BARBOSA DA SILVA</t>
+          <t>VAGO STA INES 01 HNB</t>
         </is>
       </c>
       <c r="D2336" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2337">
       <c r="A2337" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2337" t="n">
-        <v>2806</v>
+        <v>2791</v>
       </c>
       <c r="C2337" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>DANIELY SLZ 01</t>
         </is>
       </c>
       <c r="D2337" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2338">
@@ -42507,11 +42507,11 @@
         </is>
       </c>
       <c r="B2338" t="n">
-        <v>2807</v>
+        <v>2805</v>
       </c>
       <c r="C2338" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t>JANAINA BARBOSA DA SILVA</t>
         </is>
       </c>
       <c r="D2338" t="n">
@@ -42525,11 +42525,11 @@
         </is>
       </c>
       <c r="B2339" t="n">
-        <v>2808</v>
+        <v>2806</v>
       </c>
       <c r="C2339" t="inlineStr">
         <is>
-          <t>REBEKA DELGADO GUIMARAES</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D2339" t="n">
@@ -42539,127 +42539,127 @@
     <row r="2340">
       <c r="A2340" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2340" t="n">
-        <v>2820</v>
+        <v>2807</v>
       </c>
       <c r="C2340" t="inlineStr">
         <is>
-          <t>EMERSON FELIPE MELO DE AGUIAR</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D2340" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2341">
       <c r="A2341" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2341" t="n">
-        <v>2851</v>
+        <v>2808</v>
       </c>
       <c r="C2341" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>REBEKA DELGADO GUIMARAES</t>
         </is>
       </c>
       <c r="D2341" t="n">
-        <v>69</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2342">
       <c r="A2342" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2342" t="n">
-        <v>2765</v>
+        <v>2820</v>
       </c>
       <c r="C2342" t="inlineStr">
         <is>
-          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
+          <t>EMERSON FELIPE MELO DE AGUIAR</t>
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2343">
       <c r="A2343" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2343" t="n">
-        <v>2842</v>
+        <v>2851</v>
       </c>
       <c r="C2343" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2343" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2344">
       <c r="A2344" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2344" t="n">
-        <v>2741</v>
+        <v>2765</v>
       </c>
       <c r="C2344" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
+          <t>SUELMA BRAZ DE JESUS NUNES - HB</t>
         </is>
       </c>
       <c r="D2344" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2345">
       <c r="A2345" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2345" t="n">
-        <v>2758</v>
+        <v>2842</v>
       </c>
       <c r="C2345" t="inlineStr">
         <is>
-          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D2345" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2346">
       <c r="A2346" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2346" t="n">
-        <v>2854</v>
+        <v>2741</v>
       </c>
       <c r="C2346" t="inlineStr">
         <is>
-          <t>JONILSON SANTANA SANTOS - FARMA</t>
+          <t>JARDSON ROBERTH (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2346" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2347">
@@ -42669,213 +42669,213 @@
         </is>
       </c>
       <c r="B2347" t="n">
-        <v>2659</v>
+        <v>2758</v>
       </c>
       <c r="C2347" t="inlineStr">
         <is>
-          <t>ANA PAULA ALVES CAJAIBA - HB</t>
+          <t>CLAUDIONOR A. DE B. - FAR (SR DO BONFIM)</t>
         </is>
       </c>
       <c r="D2347" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2348">
       <c r="A2348" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2348" t="n">
-        <v>2669</v>
+        <v>2854</v>
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>KA AGRESTE - HB 2 (VAGO)</t>
+          <t>JONILSON SANTANA SANTOS - FARMA</t>
         </is>
       </c>
       <c r="D2348" t="n">
-        <v>135</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2349">
       <c r="A2349" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2349" t="n">
-        <v>2860</v>
+        <v>2659</v>
       </c>
       <c r="C2349" t="inlineStr">
         <is>
-          <t>HERTZ CE -  TALLIS GUTTEMBERG GUIMARAES</t>
+          <t>ANA PAULA ALVES CAJAIBA - HB</t>
         </is>
       </c>
       <c r="D2349" t="n">
-        <v>111</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2350">
       <c r="A2350" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2350" t="n">
-        <v>2672</v>
+        <v>2669</v>
       </c>
       <c r="C2350" t="inlineStr">
         <is>
-          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
+          <t>KA AGRESTE - HB 2 (VAGO)</t>
         </is>
       </c>
       <c r="D2350" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2351">
       <c r="A2351" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2351" t="n">
-        <v>2673</v>
+        <v>2860</v>
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
+          <t>HERTZ CE -  TALLIS GUTTEMBERG GUIMARAES</t>
         </is>
       </c>
       <c r="D2351" t="n">
-        <v>95</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2352">
       <c r="A2352" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2352" t="n">
-        <v>2676</v>
+        <v>2672</v>
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
+          <t>VAGO ROGERIO PEREIRA DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2352" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2353">
       <c r="A2353" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2353" t="n">
-        <v>2760</v>
+        <v>2673</v>
       </c>
       <c r="C2353" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>VAGO CARLOS ALBERTO VIRIATO S. - FARMA</t>
         </is>
       </c>
       <c r="D2353" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2354">
       <c r="A2354" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2354" t="n">
-        <v>2823</v>
+        <v>2676</v>
       </c>
       <c r="C2354" t="inlineStr">
         <is>
-          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
+          <t>LAYLLA LEAL BEZERRA (DEDICADA)</t>
         </is>
       </c>
       <c r="D2354" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2355">
       <c r="A2355" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2355" t="n">
-        <v>2848</v>
+        <v>2760</v>
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D2355" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2356">
       <c r="A2356" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2356" t="n">
-        <v>2792</v>
+        <v>2823</v>
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>LUCIMARA SOUSA LIMA</t>
+          <t>JOAO VICTOR GUEDES DE AZEVEDO</t>
         </is>
       </c>
       <c r="D2356" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2357">
       <c r="A2357" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2357" t="n">
-        <v>2793</v>
+        <v>2848</v>
       </c>
       <c r="C2357" t="inlineStr">
         <is>
-          <t>EMERSON SANTOS DE SOUSA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2357" t="n">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2358">
       <c r="A2358" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2358" t="n">
-        <v>2802</v>
+        <v>2792</v>
       </c>
       <c r="C2358" t="inlineStr">
         <is>
-          <t>FABRICIO DO CARMO MEDEIROS</t>
+          <t>LUCIMARA SOUSA LIMA</t>
         </is>
       </c>
       <c r="D2358" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2359">
@@ -42885,33 +42885,33 @@
         </is>
       </c>
       <c r="B2359" t="n">
-        <v>2656</v>
+        <v>2793</v>
       </c>
       <c r="C2359" t="inlineStr">
         <is>
-          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
+          <t>EMERSON SANTOS DE SOUSA</t>
         </is>
       </c>
       <c r="D2359" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2360">
       <c r="A2360" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2360" t="n">
-        <v>2657</v>
+        <v>2802</v>
       </c>
       <c r="C2360" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA IMP 01 HNB</t>
+          <t>FABRICIO DO CARMO MEDEIROS</t>
         </is>
       </c>
       <c r="D2360" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2361">
@@ -42921,33 +42921,33 @@
         </is>
       </c>
       <c r="B2361" t="n">
-        <v>2658</v>
+        <v>2656</v>
       </c>
       <c r="C2361" t="inlineStr">
         <is>
-          <t>PEROLA DE JESUS AMORIM SOUSA</t>
+          <t>RAIMUNDO VICTOR DE SOUSA FERNANDES</t>
         </is>
       </c>
       <c r="D2361" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2362">
       <c r="A2362" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2362" t="n">
-        <v>2729</v>
+        <v>2657</v>
       </c>
       <c r="C2362" t="inlineStr">
         <is>
-          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
+          <t>MARIA APARECIDA IMP 01 HNB</t>
         </is>
       </c>
       <c r="D2362" t="n">
-        <v>50</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2363">
@@ -42957,33 +42957,33 @@
         </is>
       </c>
       <c r="B2363" t="n">
-        <v>2759</v>
+        <v>2658</v>
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
+          <t>PEROLA DE JESUS AMORIM SOUSA</t>
         </is>
       </c>
       <c r="D2363" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2364">
       <c r="A2364" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2364" t="n">
-        <v>2832</v>
+        <v>2729</v>
       </c>
       <c r="C2364" t="inlineStr">
         <is>
-          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
+          <t>LETICIA BENTO SILVA VIANA - FARMA</t>
         </is>
       </c>
       <c r="D2364" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2365">
@@ -42993,11 +42993,11 @@
         </is>
       </c>
       <c r="B2365" t="n">
-        <v>2769</v>
+        <v>2759</v>
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>MARDONIO CUNHA BASILIO</t>
+          <t>CLIENTE INATIVOS COM DÉBITO NUBIA</t>
         </is>
       </c>
       <c r="D2365" t="n">
@@ -43007,73 +43007,73 @@
     <row r="2366">
       <c r="A2366" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2366" t="n">
-        <v>2679</v>
+        <v>2832</v>
       </c>
       <c r="C2366" t="inlineStr">
         <is>
-          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
+          <t>JEANIA PIRES DE ARAUJO (ZÉ DOCA)</t>
         </is>
       </c>
       <c r="D2366" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2367">
       <c r="A2367" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2367" t="n">
-        <v>2680</v>
+        <v>2769</v>
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
+          <t>MARDONIO CUNHA BASILIO</t>
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2368">
       <c r="A2368" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2368" t="n">
-        <v>2815</v>
+        <v>2679</v>
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
+          <t>MAX DAYLLE PINHEIRO ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2368" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2369">
       <c r="A2369" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2369" t="n">
-        <v>2816</v>
+        <v>2680</v>
       </c>
       <c r="C2369" t="inlineStr">
         <is>
-          <t>TIAGO SILVA DE SOUZA - HB</t>
+          <t>LUCAS GABRIEL CAVALCANTE DA COSTA</t>
         </is>
       </c>
       <c r="D2369" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2370">
@@ -43083,105 +43083,105 @@
         </is>
       </c>
       <c r="B2370" t="n">
-        <v>2817</v>
+        <v>2815</v>
       </c>
       <c r="C2370" t="inlineStr">
         <is>
-          <t>MICHAEL CARVALHO FERREIRA - HB</t>
+          <t>LUIZ FELIPE MACHADO BARRETO - FARMA</t>
         </is>
       </c>
       <c r="D2370" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2371">
       <c r="A2371" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2371" t="n">
-        <v>2841</v>
+        <v>2816</v>
       </c>
       <c r="C2371" t="inlineStr">
         <is>
-          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
+          <t>TIAGO SILVA DE SOUZA - HB</t>
         </is>
       </c>
       <c r="D2371" t="n">
-        <v>46</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2372">
       <c r="A2372" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2372" t="n">
-        <v>2701</v>
+        <v>2817</v>
       </c>
       <c r="C2372" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>MICHAEL CARVALHO FERREIRA - HB</t>
         </is>
       </c>
       <c r="D2372" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2373">
       <c r="A2373" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2373" t="n">
-        <v>2644</v>
+        <v>2841</v>
       </c>
       <c r="C2373" t="inlineStr">
         <is>
-          <t>THAMIRES DA SILVA MONTEIRO</t>
+          <t>CRISTIANE DA SILVA SOUSA RODRIGUES</t>
         </is>
       </c>
       <c r="D2373" t="n">
-        <v>108</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2374">
       <c r="A2374" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2374" t="n">
-        <v>2645</v>
+        <v>2701</v>
       </c>
       <c r="C2374" t="inlineStr">
         <is>
-          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D2374" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2375">
       <c r="A2375" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2375" t="n">
-        <v>2754</v>
+        <v>2644</v>
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>RCA SUPERVISÃO HERTZ PI</t>
+          <t>THAMIRES DA SILVA MONTEIRO</t>
         </is>
       </c>
       <c r="D2375" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2376">
@@ -43191,51 +43191,51 @@
         </is>
       </c>
       <c r="B2376" t="n">
-        <v>2755</v>
+        <v>2645</v>
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>RUBYA DANILLA ARAUJO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2376" t="n">
-        <v>80</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2377">
       <c r="A2377" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2377" t="n">
-        <v>2665</v>
+        <v>2754</v>
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>RCA SUPERVISÃO HERTZ PI</t>
         </is>
       </c>
       <c r="D2377" t="n">
-        <v>141</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2378">
       <c r="A2378" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2378" t="n">
-        <v>2667</v>
+        <v>2755</v>
       </c>
       <c r="C2378" t="inlineStr">
         <is>
-          <t>VAGO AÇAILÂNDIA HNB</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D2378" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2379">
@@ -43245,15 +43245,15 @@
         </is>
       </c>
       <c r="B2379" t="n">
-        <v>2727</v>
+        <v>2665</v>
       </c>
       <c r="C2379" t="inlineStr">
         <is>
-          <t>SETOR VAGO (MEGUEGA)</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D2379" t="n">
-        <v>120</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2380">
@@ -43263,51 +43263,51 @@
         </is>
       </c>
       <c r="B2380" t="n">
-        <v>2728</v>
+        <v>2667</v>
       </c>
       <c r="C2380" t="inlineStr">
         <is>
-          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
+          <t>VAGO AÇAILÂNDIA HNB</t>
         </is>
       </c>
       <c r="D2380" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2381">
       <c r="A2381" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2381" t="n">
-        <v>2833</v>
+        <v>2727</v>
       </c>
       <c r="C2381" t="inlineStr">
         <is>
-          <t>ADEILZA PINTO DA SILVA - FARMA</t>
+          <t>SETOR VAGO (MEGUEGA)</t>
         </is>
       </c>
       <c r="D2381" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2382">
       <c r="A2382" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2382" t="n">
-        <v>2814</v>
+        <v>2728</v>
       </c>
       <c r="C2382" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA (PI)</t>
+          <t>CARLOS GABRIEL DOS SANTOS LACERDA</t>
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2383">
@@ -43317,33 +43317,33 @@
         </is>
       </c>
       <c r="B2383" t="n">
-        <v>2855</v>
+        <v>2833</v>
       </c>
       <c r="C2383" t="inlineStr">
         <is>
-          <t>DESIREE BARROS DE CARVALHO - CCM</t>
+          <t>ADEILZA PINTO DA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2383" t="n">
-        <v>14</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2384">
       <c r="A2384" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2384" t="n">
-        <v>2646</v>
+        <v>2814</v>
       </c>
       <c r="C2384" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
+          <t>MATHEUS LIMA BATISTA (PI)</t>
         </is>
       </c>
       <c r="D2384" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2385">
@@ -43353,15 +43353,15 @@
         </is>
       </c>
       <c r="B2385" t="n">
-        <v>2650</v>
+        <v>2855</v>
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
+          <t>DESIREE BARROS DE CARVALHO - CCM</t>
         </is>
       </c>
       <c r="D2385" t="n">
-        <v>95</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2386">
@@ -43371,15 +43371,15 @@
         </is>
       </c>
       <c r="B2386" t="n">
-        <v>2652</v>
+        <v>2646</v>
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>JAILTON PEREIRA MERCES - HB</t>
+          <t>HERMANS SERGIO GUERREIRO - SUPER</t>
         </is>
       </c>
       <c r="D2386" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2387">
@@ -43389,11 +43389,11 @@
         </is>
       </c>
       <c r="B2387" t="n">
-        <v>2653</v>
+        <v>2650</v>
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
+          <t>VAGO ANAELSON FREITAS VIEIRA - FARMA</t>
         </is>
       </c>
       <c r="D2387" t="n">
@@ -43407,15 +43407,15 @@
         </is>
       </c>
       <c r="B2388" t="n">
-        <v>2654</v>
+        <v>2652</v>
       </c>
       <c r="C2388" t="inlineStr">
         <is>
-          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
+          <t>JAILTON PEREIRA MERCES - HB</t>
         </is>
       </c>
       <c r="D2388" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2389">
@@ -43425,33 +43425,33 @@
         </is>
       </c>
       <c r="B2389" t="n">
-        <v>2655</v>
+        <v>2653</v>
       </c>
       <c r="C2389" t="inlineStr">
         <is>
-          <t>FABIO BORGES DOS SANTOS - HB</t>
+          <t>MARCO ANTONIO DOS SANTOS BARROS - FARMA</t>
         </is>
       </c>
       <c r="D2389" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2390">
       <c r="A2390" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2390" t="n">
-        <v>2821</v>
+        <v>2654</v>
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>HENILDA ALVES PEREIRA</t>
+          <t>VAGO ITANA NASCIMENTO SIMÕES - FARMA</t>
         </is>
       </c>
       <c r="D2390" t="n">
-        <v>69</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2391">
@@ -43461,231 +43461,231 @@
         </is>
       </c>
       <c r="B2391" t="n">
-        <v>2683</v>
+        <v>2655</v>
       </c>
       <c r="C2391" t="inlineStr">
         <is>
-          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
+          <t>FABIO BORGES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2391" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2392" t="n">
-        <v>2684</v>
+        <v>2821</v>
       </c>
       <c r="C2392" t="inlineStr">
         <is>
-          <t>MARCELO PEREIRA BASTOS - HB</t>
+          <t>HENILDA ALVES PEREIRA</t>
         </is>
       </c>
       <c r="D2392" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2393">
       <c r="A2393" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2393" t="n">
-        <v>2749</v>
+        <v>2683</v>
       </c>
       <c r="C2393" t="inlineStr">
         <is>
-          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
+          <t>VAGO LILIAN OITABEN P. COUTINHO - FARMA</t>
         </is>
       </c>
       <c r="D2393" t="n">
-        <v>111</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2394">
       <c r="A2394" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2394" t="n">
-        <v>2812</v>
+        <v>2684</v>
       </c>
       <c r="C2394" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>MARCELO PEREIRA BASTOS - HB</t>
         </is>
       </c>
       <c r="D2394" t="n">
-        <v>145</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2395">
       <c r="A2395" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2395" t="n">
-        <v>2715</v>
+        <v>2749</v>
       </c>
       <c r="C2395" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>INATIVO - HERTZ CE - DAVID EVANGELISTA</t>
         </is>
       </c>
       <c r="D2395" t="n">
-        <v>90</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2396">
       <c r="A2396" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2396" t="n">
-        <v>2834</v>
+        <v>2812</v>
       </c>
       <c r="C2396" t="inlineStr">
         <is>
-          <t>GILVANA MONTELES U. SANTOS HNB</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D2396" t="n">
-        <v>114</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2397">
       <c r="A2397" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2397" t="n">
-        <v>2651</v>
+        <v>2715</v>
       </c>
       <c r="C2397" t="inlineStr">
         <is>
-          <t>CAIO DE SOUZA VINHAS</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D2397" t="n">
-        <v>145</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2398" t="n">
-        <v>2819</v>
+        <v>2834</v>
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA - FARMA</t>
+          <t>GILVANA MONTELES U. SANTOS HNB</t>
         </is>
       </c>
       <c r="D2398" t="n">
-        <v>95</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2399">
       <c r="A2399" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2399" t="n">
-        <v>2849</v>
+        <v>2651</v>
       </c>
       <c r="C2399" t="inlineStr">
         <is>
-          <t>MULTI PE (PEDRO HENRIQUE VIERA)</t>
+          <t>CAIO DE SOUZA VINHAS</t>
         </is>
       </c>
       <c r="D2399" t="n">
-        <v>72</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2400">
       <c r="A2400" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2400" t="n">
-        <v>2835</v>
+        <v>2819</v>
       </c>
       <c r="C2400" t="inlineStr">
         <is>
-          <t>ROGÉRIO LIRA DA GAMA</t>
+          <t>FABIO OLIVEIRA SILVA - FARMA</t>
         </is>
       </c>
       <c r="D2400" t="n">
-        <v>116</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2401">
       <c r="A2401" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2401" t="n">
-        <v>2699</v>
+        <v>2849</v>
       </c>
       <c r="C2401" t="inlineStr">
         <is>
-          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
+          <t>MULTI PE (PEDRO HENRIQUE VIERA)</t>
         </is>
       </c>
       <c r="D2401" t="n">
-        <v>95</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2402">
       <c r="A2402" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2402" t="n">
-        <v>2706</v>
+        <v>2835</v>
       </c>
       <c r="C2402" t="inlineStr">
         <is>
-          <t>VAGO BARREIRINHAS HNB</t>
+          <t>ROGÉRIO LIRA DA GAMA</t>
         </is>
       </c>
       <c r="D2402" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2403">
       <c r="A2403" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2403" t="n">
-        <v>2707</v>
+        <v>2699</v>
       </c>
       <c r="C2403" t="inlineStr">
         <is>
-          <t>VAGO BACABAL HNB</t>
+          <t>VAGO LUAN SANTOS BAHIA - FARMA</t>
         </is>
       </c>
       <c r="D2403" t="n">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2404">
@@ -43695,15 +43695,15 @@
         </is>
       </c>
       <c r="B2404" t="n">
-        <v>2846</v>
+        <v>2706</v>
       </c>
       <c r="C2404" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>VAGO BARREIRINHAS HNB</t>
         </is>
       </c>
       <c r="D2404" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2405">
@@ -43713,87 +43713,87 @@
         </is>
       </c>
       <c r="B2405" t="n">
-        <v>2847</v>
+        <v>2707</v>
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>FRANCISCO WERBERTTY DA SILVA MORAIS</t>
+          <t>VAGO BACABAL HNB</t>
         </is>
       </c>
       <c r="D2405" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2406">
       <c r="A2406" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2406" t="n">
-        <v>2693</v>
+        <v>2846</v>
       </c>
       <c r="C2406" t="inlineStr">
         <is>
-          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D2406" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2407">
       <c r="A2407" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2407" t="n">
-        <v>2705</v>
+        <v>2847</v>
       </c>
       <c r="C2407" t="inlineStr">
         <is>
-          <t>PAULISTA-HB(BRENDA LIMA)</t>
+          <t>FRANCISCO WERBERTTY DA SILVA MORAIS</t>
         </is>
       </c>
       <c r="D2407" t="n">
-        <v>146</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2408">
       <c r="A2408" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2408" t="n">
-        <v>2664</v>
+        <v>2693</v>
       </c>
       <c r="C2408" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t>SETOR VAGO CAPITAL ( KLEY HERTZ )</t>
         </is>
       </c>
       <c r="D2408" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2409" t="n">
-        <v>2670</v>
+        <v>2705</v>
       </c>
       <c r="C2409" t="inlineStr">
         <is>
-          <t>GISLENE MENDES SANTANA</t>
+          <t>PAULISTA-HB(BRENDA LIMA)</t>
         </is>
       </c>
       <c r="D2409" t="n">
-        <v>69</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2410">
@@ -43803,213 +43803,213 @@
         </is>
       </c>
       <c r="B2410" t="n">
-        <v>2730</v>
+        <v>2664</v>
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>ANCELIO MELO PLACIDO</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D2410" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2411">
       <c r="A2411" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2411" t="n">
-        <v>2859</v>
+        <v>2670</v>
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>ALEXANDRE MARTINS CHAVES</t>
+          <t>GISLENE MENDES SANTANA</t>
         </is>
       </c>
       <c r="D2411" t="n">
-        <v>132</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2412">
       <c r="A2412" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2412" t="n">
-        <v>2671</v>
+        <v>2730</v>
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>DIOGENES ALVES DOS SANTOS - HB</t>
+          <t>ANCELIO MELO PLACIDO</t>
         </is>
       </c>
       <c r="D2412" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2413">
       <c r="A2413" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2413" t="n">
-        <v>2691</v>
+        <v>2859</v>
       </c>
       <c r="C2413" t="inlineStr">
         <is>
-          <t>MARCELO DIAS DO AMARAL</t>
+          <t>ALEXANDRE MARTINS CHAVES</t>
         </is>
       </c>
       <c r="D2413" t="n">
-        <v>80</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2414">
       <c r="A2414" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2414" t="n">
-        <v>2692</v>
+        <v>2671</v>
       </c>
       <c r="C2414" t="inlineStr">
         <is>
-          <t>BRUNO ALEXANDRE SOUSA</t>
+          <t>DIOGENES ALVES DOS SANTOS - HB</t>
         </is>
       </c>
       <c r="D2414" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2415">
       <c r="A2415" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2415" t="n">
-        <v>2724</v>
+        <v>2691</v>
       </c>
       <c r="C2415" t="inlineStr">
         <is>
-          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
+          <t>MARCELO DIAS DO AMARAL</t>
         </is>
       </c>
       <c r="D2415" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2416">
       <c r="A2416" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2416" t="n">
-        <v>2773</v>
+        <v>2692</v>
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>TIMON 01 HNB</t>
+          <t>BRUNO ALEXANDRE SOUSA</t>
         </is>
       </c>
       <c r="D2416" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2417">
       <c r="A2417" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2417" t="n">
-        <v>2844</v>
+        <v>2724</v>
       </c>
       <c r="C2417" t="inlineStr">
         <is>
-          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
+          <t>VAGO MARCIO LUCAS DA SILVA LIMA - FARMA</t>
         </is>
       </c>
       <c r="D2417" t="n">
-        <v>132</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2418">
       <c r="A2418" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2418" t="n">
-        <v>2845</v>
+        <v>2773</v>
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
+          <t>TIMON 01 HNB</t>
         </is>
       </c>
       <c r="D2418" t="n">
-        <v>132</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2419">
       <c r="A2419" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2419" t="n">
-        <v>2825</v>
+        <v>2844</v>
       </c>
       <c r="C2419" t="inlineStr">
         <is>
-          <t>DANIEL BOTELHO DE SOUSA</t>
+          <t>MOACY BANDEIRA CAMILO DE QUEIROZ BRITO</t>
         </is>
       </c>
       <c r="D2419" t="n">
-        <v>90</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2420">
       <c r="A2420" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2420" t="n">
-        <v>2787</v>
+        <v>2845</v>
       </c>
       <c r="C2420" t="inlineStr">
         <is>
-          <t>MATHEUS LIMA BATISTA</t>
+          <t xml:space="preserve">MAYCON GEAN DE LIMA SILVA </t>
         </is>
       </c>
       <c r="D2420" t="n">
-        <v>120</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2421">
       <c r="A2421" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2421" t="n">
-        <v>2839</v>
+        <v>2825</v>
       </c>
       <c r="C2421" t="inlineStr">
         <is>
-          <t>RCA TENA OL PI</t>
+          <t>DANIEL BOTELHO DE SOUSA</t>
         </is>
       </c>
       <c r="D2421" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2422">
@@ -44019,69 +44019,69 @@
         </is>
       </c>
       <c r="B2422" t="n">
-        <v>2840</v>
+        <v>2787</v>
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>RCA TENA OL MA</t>
+          <t>MATHEUS LIMA BATISTA</t>
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>114</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2423">
       <c r="A2423" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2423" t="n">
-        <v>2648</v>
+        <v>2839</v>
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t>RCA TENA OL PI</t>
         </is>
       </c>
       <c r="D2423" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2424">
       <c r="A2424" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2424" t="n">
-        <v>2666</v>
+        <v>2840</v>
       </c>
       <c r="C2424" t="inlineStr">
         <is>
-          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
+          <t>RCA TENA OL MA</t>
         </is>
       </c>
       <c r="D2424" t="n">
-        <v>63</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2425">
       <c r="A2425" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2425" t="n">
-        <v>2779</v>
+        <v>2648</v>
       </c>
       <c r="C2425" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO - TLV</t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D2425" t="n">
-        <v>105</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2426">
@@ -44091,15 +44091,15 @@
         </is>
       </c>
       <c r="B2426" t="n">
-        <v>2780</v>
+        <v>2666</v>
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>VAGO GUILHERME HENRIQUE S. DA SILVA - HB</t>
         </is>
       </c>
       <c r="D2426" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2427">
@@ -44109,51 +44109,51 @@
         </is>
       </c>
       <c r="B2427" t="n">
-        <v>2786</v>
+        <v>2779</v>
       </c>
       <c r="C2427" t="inlineStr">
         <is>
-          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO - TLV</t>
         </is>
       </c>
       <c r="D2427" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2428">
       <c r="A2428" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2428" t="n">
-        <v>2660</v>
+        <v>2780</v>
       </c>
       <c r="C2428" t="inlineStr">
         <is>
-          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D2428" t="n">
-        <v>38</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2429">
       <c r="A2429" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2429" t="n">
-        <v>2716</v>
+        <v>2786</v>
       </c>
       <c r="C2429" t="inlineStr">
         <is>
-          <t>DURVAL LOPES DE OLIVEIRA</t>
+          <t>RONEY BASTOS CUNHA - HB (ITAPETINGA)</t>
         </is>
       </c>
       <c r="D2429" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2430">
@@ -44163,51 +44163,51 @@
         </is>
       </c>
       <c r="B2430" t="n">
-        <v>2734</v>
+        <v>2660</v>
       </c>
       <c r="C2430" t="inlineStr">
         <is>
-          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
+          <t>JARDSON ROBERTH CUTRIM SOUZA</t>
         </is>
       </c>
       <c r="D2430" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2431">
       <c r="A2431" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2431" t="n">
-        <v>2853</v>
+        <v>2716</v>
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>H-ROBERTO SOARES OLIVEIRA JUNIOR</t>
+          <t>DURVAL LOPES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2431" t="n">
-        <v>53</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2432">
       <c r="A2432" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2432" t="n">
-        <v>2742</v>
+        <v>2734</v>
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>VAGO MARCUS VINICIUS - FARMA JACOBINA</t>
+          <t xml:space="preserve">JOAO ALEX - SETOR HERTZ </t>
         </is>
       </c>
       <c r="D2432" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2433">
@@ -44217,15 +44217,15 @@
         </is>
       </c>
       <c r="B2433" t="n">
-        <v>2794</v>
+        <v>2853</v>
       </c>
       <c r="C2433" t="inlineStr">
         <is>
-          <t>VAGO DEISIELLE J. SILVA - HB JACOBINA</t>
+          <t>H-ROBERTO SOARES OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D2433" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2434">
@@ -44235,11 +44235,11 @@
         </is>
       </c>
       <c r="B2434" t="n">
-        <v>2795</v>
+        <v>2742</v>
       </c>
       <c r="C2434" t="inlineStr">
         <is>
-          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
+          <t>VAGO MARCUS VINICIUS - FARMA JACOBINA</t>
         </is>
       </c>
       <c r="D2434" t="n">
@@ -44253,15 +44253,15 @@
         </is>
       </c>
       <c r="B2435" t="n">
-        <v>2796</v>
+        <v>2794</v>
       </c>
       <c r="C2435" t="inlineStr">
         <is>
-          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
+          <t>VAGO DEISIELLE J. SILVA - HB JACOBINA</t>
         </is>
       </c>
       <c r="D2435" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2436">
@@ -44271,11 +44271,11 @@
         </is>
       </c>
       <c r="B2436" t="n">
-        <v>2797</v>
+        <v>2795</v>
       </c>
       <c r="C2436" t="inlineStr">
         <is>
-          <t>VAGO ESDRAS A. SANTOS-FAR (PAULO AFO)</t>
+          <t>VAGO VINICIUS RAMOS (CAMAÇARÍ) - FARMA</t>
         </is>
       </c>
       <c r="D2436" t="n">
@@ -44289,11 +44289,11 @@
         </is>
       </c>
       <c r="B2437" t="n">
-        <v>2798</v>
+        <v>2796</v>
       </c>
       <c r="C2437" t="inlineStr">
         <is>
-          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
+          <t>VAGO BRENO ALLAN - FARM (SSA CENTRO)</t>
         </is>
       </c>
       <c r="D2437" t="n">
@@ -44303,73 +44303,73 @@
     <row r="2438">
       <c r="A2438" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2438" t="n">
-        <v>2668</v>
+        <v>2797</v>
       </c>
       <c r="C2438" t="inlineStr">
         <is>
-          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
+          <t>VAGO ESDRAS A. SANTOS-FAR (PAULO AFO)</t>
         </is>
       </c>
       <c r="D2438" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2439">
       <c r="A2439" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2439" t="n">
-        <v>2690</v>
+        <v>2798</v>
       </c>
       <c r="C2439" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON DA PAZ LIMA - FARMA (LAURO DE FRE)</t>
         </is>
       </c>
       <c r="D2439" t="n">
-        <v>38</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2440">
       <c r="A2440" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B2440" t="n">
-        <v>2696</v>
+        <v>2668</v>
       </c>
       <c r="C2440" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>OLINDA - FARMA(JAILSON/VAGO)</t>
         </is>
       </c>
       <c r="D2440" t="n">
-        <v>69</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2441">
       <c r="A2441" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2441" t="n">
-        <v>2697</v>
+        <v>2690</v>
       </c>
       <c r="C2441" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D2441" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2442">
@@ -44379,11 +44379,11 @@
         </is>
       </c>
       <c r="B2442" t="n">
-        <v>2698</v>
+        <v>2696</v>
       </c>
       <c r="C2442" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D2442" t="n">
@@ -44393,37 +44393,37 @@
     <row r="2443">
       <c r="A2443" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2443" t="n">
-        <v>2775</v>
+        <v>2697</v>
       </c>
       <c r="C2443" t="inlineStr">
         <is>
-          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D2443" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2444">
       <c r="A2444" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2444" t="n">
-        <v>2776</v>
+        <v>2698</v>
       </c>
       <c r="C2444" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D2444" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2445">
@@ -44433,11 +44433,11 @@
         </is>
       </c>
       <c r="B2445" t="n">
-        <v>2777</v>
+        <v>2775</v>
       </c>
       <c r="C2445" t="inlineStr">
         <is>
-          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
+          <t>ANTONIO LUIZ GONZAGA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2445" t="n">
@@ -44451,11 +44451,11 @@
         </is>
       </c>
       <c r="B2446" t="n">
-        <v>2778</v>
+        <v>2776</v>
       </c>
       <c r="C2446" t="inlineStr">
         <is>
-          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
+          <t>CARLOS JEANDERSON (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2446" t="n">
@@ -44469,15 +44469,15 @@
         </is>
       </c>
       <c r="B2447" t="n">
-        <v>2781</v>
+        <v>2777</v>
       </c>
       <c r="C2447" t="inlineStr">
         <is>
-          <t>PABLO DIEGO DE ARAUJO COSTA</t>
+          <t>FRANCISCO IRASLHEY (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2447" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2448">
@@ -44487,11 +44487,11 @@
         </is>
       </c>
       <c r="B2448" t="n">
-        <v>2822</v>
+        <v>2778</v>
       </c>
       <c r="C2448" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>BRUNO STEFAN SANTOS (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2448" t="n">
@@ -44505,87 +44505,87 @@
         </is>
       </c>
       <c r="B2449" t="n">
-        <v>2740</v>
+        <v>2781</v>
       </c>
       <c r="C2449" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
+          <t>PABLO DIEGO DE ARAUJO COSTA</t>
         </is>
       </c>
       <c r="D2449" t="n">
-        <v>38</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2450">
       <c r="A2450" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2450" t="n">
-        <v>2710</v>
+        <v>2822</v>
       </c>
       <c r="C2450" t="inlineStr">
         <is>
-          <t>SETOR VAGO PLUS PI (MAX)</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D2450" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2451">
       <c r="A2451" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B2451" t="n">
-        <v>2711</v>
+        <v>2740</v>
       </c>
       <c r="C2451" t="inlineStr">
         <is>
-          <t>CARLOS CHAPADINHA</t>
+          <t>FERNANDA DA SILVA (CLIENTES INATIVOS)</t>
         </is>
       </c>
       <c r="D2451" t="n">
-        <v>114</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2452">
       <c r="A2452" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2452" t="n">
-        <v>2712</v>
+        <v>2710</v>
       </c>
       <c r="C2452" t="inlineStr">
         <is>
-          <t>RCA DEDICADA MA (SAO LUIS)</t>
+          <t>SETOR VAGO PLUS PI (MAX)</t>
         </is>
       </c>
       <c r="D2452" t="n">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2453">
       <c r="A2453" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2453" t="n">
-        <v>2717</v>
+        <v>2711</v>
       </c>
       <c r="C2453" t="inlineStr">
         <is>
-          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+          <t>CARLOS CHAPADINHA</t>
         </is>
       </c>
       <c r="D2453" t="n">
-        <v>69</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2454">
@@ -44595,14 +44595,50 @@
         </is>
       </c>
       <c r="B2454" t="n">
+        <v>2712</v>
+      </c>
+      <c r="C2454" t="inlineStr">
+        <is>
+          <t>RCA DEDICADA MA (SAO LUIS)</t>
+        </is>
+      </c>
+      <c r="D2454" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2455">
+      <c r="A2455" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2455" t="n">
+        <v>2717</v>
+      </c>
+      <c r="C2455" t="inlineStr">
+        <is>
+          <t>SILAS INVESTIMENTOS PI - PLUS</t>
+        </is>
+      </c>
+      <c r="D2455" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2456">
+      <c r="A2456" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2456" t="n">
         <v>2801</v>
       </c>
-      <c r="C2454" t="inlineStr">
+      <c r="C2456" t="inlineStr">
         <is>
           <t>SETOR VAGO VIANA FARMA</t>
         </is>
       </c>
-      <c r="D2454" t="n">
+      <c r="D2456" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:02:16
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -11243,7 +11243,7 @@
       </c>
       <c r="C601" t="inlineStr">
         <is>
-          <t>KAWA ALMEIDA CAMPOS</t>
+          <t>ALEXANDRE MARTINS CHAVES</t>
         </is>
       </c>
       <c r="D601" t="n">
@@ -29914,7 +29914,7 @@
         </is>
       </c>
       <c r="D1638" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="1639">
@@ -35747,7 +35747,7 @@
         </is>
       </c>
       <c r="D1962" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="1963">
@@ -38051,7 +38051,7 @@
         </is>
       </c>
       <c r="D2090" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2091">
@@ -42587,7 +42587,7 @@
         </is>
       </c>
       <c r="D2342" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2343">
@@ -42893,7 +42893,7 @@
         </is>
       </c>
       <c r="D2359" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2360">
@@ -43037,7 +43037,7 @@
         </is>
       </c>
       <c r="D2367" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2368">
@@ -43307,7 +43307,7 @@
         </is>
       </c>
       <c r="D2382" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2383">
@@ -44027,7 +44027,7 @@
         </is>
       </c>
       <c r="D2422" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2423">

</xml_diff>

<commit_message>
chore(data): batch update intraday dim_rca - 08:03:22
</commit_message>
<xml_diff>
--- a/data/dim_rca.xlsx
+++ b/data/dim_rca.xlsx
@@ -36373,7 +36373,7 @@
       </c>
       <c r="C1997" t="inlineStr">
         <is>
-          <t>LETICIA AMANDA DE JESUS - MULTILAB</t>
+          <t>VAGO LETICIA AMANDA DE JESUS - MULTILAB</t>
         </is>
       </c>
       <c r="D1997" t="n">
@@ -43951,7 +43951,7 @@
       </c>
       <c r="C2418" t="inlineStr">
         <is>
-          <t>TIMON 01 HNB</t>
+          <t>TIMON 01 HNB (VIVIANE)</t>
         </is>
       </c>
       <c r="D2418" t="n">

</xml_diff>